<commit_message>
Add confirmed viscosity spec (<2,500 cps) — closes the last spec blocker
Brookfield, spindle #3, 10 RPM, 25 C. Updates:
- Action Plan: viscosity blocker marked RESOLVED/DONE (only the NDA remains open)
- RFQ email and web-form templates now carry the viscosity in the product line
- New 'full spec' block on the RFQ tab to send once a supplier confirms capability
- Read Me and Stakeholder Map updated

Note: under 2,500 cps is an easily pumped and filtered fluid, so no blender can
price this as a difficult high-viscosity job.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Supplier_Longlist.xlsx
+++ b/PVA second supplier initiative/PVA_Supplier_Longlist.xlsx
@@ -119,12 +119,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -181,16 +181,16 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,16 +202,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -238,28 +238,28 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -272,10 +272,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -296,10 +296,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C26"/>
+  <dimension ref="B2:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -736,7 +736,7 @@
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>MAJOR CORRECTIONS TO v1 (why the tiers moved)</t>
+          <t>SPEC NOW CONFIRMED — both open blockers closed</t>
         </is>
       </c>
       <c r="C9" s="4" t="n"/>
@@ -744,194 +744,226 @@
     <row r="10">
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>PhilChem — was Tier A, now B</t>
+          <t>Viscosity target — CONFIRMED</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>MIS-TARGETED. PhilChem (Greer, SC) is a DRY blending / repackaging house — 'specialty formulated dry blends,' 250 MM lb/yr dry capacity. The jacketed heated-vessel language that earned it Tier A lives on the PARENT site (Mount Vernon Chemicals) and describes other plants. Contact the group and ask which plant runs jacketed liquid batches.</t>
+          <t>&lt; 2,500 cps, Brookfield spindle #3, 10 RPM, 25 C. This was the longest-standing open item on the project and it gated every firm quote. Two consequences: (1) suppliers can now quote firmly and a qualification batch can be judged pass/fail against a real number; (2) commercially it is good news — under 2,500 cps is an easily pumped and easily filtered fluid, so no blender can price this as a 'difficult, high-viscosity' job. Put the number in every RFQ and require it on every CoA.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="7" t="inlineStr">
         <is>
+          <t>ISO 13485 — NOT required</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed: no ISO 13485 supplier needed. Still require ISO 9001, lot traceability, and a CoA with lot #, production date, %TS, pH, and viscosity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>MAJOR CORRECTIONS TO v1 (why the tiers moved)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>PhilChem — was Tier A, now B</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>MIS-TARGETED. PhilChem (Greer, SC) is a DRY blending / repackaging house — 'specialty formulated dry blends,' 250 MM lb/yr dry capacity. The jacketed heated-vessel language that earned it Tier A lives on the PARENT site (Mount Vernon Chemicals) and describes other plants. Contact the group and ask which plant runs jacketed liquid batches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
           <t>Chemjet — was Tier A, now C</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>TWO ERRORS. Houston is a sales office; the plants are in Conroe and Odessa, TX. And it's an oilfield / drilling-fluids house — a poor fit for a medical-device component. A 'heat room' is also not a jacketed vessel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>MFG Chemical — was Tier A, now C</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>SCALE MISMATCH. Heat is a slam dunk (hot oil to 290 C) but the smallest production reactor is 2,000 gal against our ~50 gal. This is exactly the profile that produced the $8/lb quote you just declined. Also now PE-owned (Windjammer, Jan 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Tiarco / TRCC — was Tier A, now B</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>No published basis for Tier A — the site publishes zero equipment, temperature, batch-size or certification data. Real company, right geography, but everything must be established by phone. (Their 'verify before proceeding with POs' banner is an anti-fraud notice, not financial distress.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>REXCO-USA — was Tier A, now C</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Makes pigmented aqueous PVA solutions, but publishes nothing supporting toll manufacturing, heat capability, or a quality system. Keep as a technical resource / long shot.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
+          <t>MFG Chemical — was Tier A, now C</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>SCALE MISMATCH. Heat is a slam dunk (hot oil to 290 C) but the smallest production reactor is 2,000 gal against our ~50 gal. This is exactly the profile that produced the $8/lb quote you just declined. Also now PE-owned (Windjammer, Jan 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Tiarco / TRCC — was Tier A, now B</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>No published basis for Tier A — the site publishes zero equipment, temperature, batch-size or certification data. Real company, right geography, but everything must be established by phone. (Their 'verify before proceeding with POs' banner is an anti-fraud notice, not financial distress.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>REXCO-USA — was Tier A, now C</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Makes pigmented aqueous PVA solutions, but publishes nothing supporting toll manufacturing, heat capability, or a quality system. Keep as a technical resource / long shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
           <t>5 companies DROPPED</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Peach State Labs (dead URL — the Rome GA business is now Polyventive), Aicello (no US manufacturing), Troy Chemical (listing conflated two companies; intended one acquired 2022), CHT USA (Richmond VA is a SILICONE plant — silicone contamination is close to worst-case for a waterborne coating), South Coast Terminals (self-documented disqualification: 10 MT minimum batches).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="3" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>WHAT'S NEW IN v2</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>ISO 13485 NOT required — RESOLVED</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Confirmed by Oscar: we do not need an ISO 13485 supplier. That closes an open blocker and simplifies the search. The medical-grade candidates found in research (Polysciences, Hydromer, HR Pharmaceuticals, Strukmyer, GeminiBio, Kingchem, Alpha Teknova, Biocoat, NEXT Medical) are therefore DEPRIORITIZED to Tier C — they would price well above the incumbent for a certification we do not need. They stay listed only as a fallback if Quality later asks for a stricter supply chain. What we DO still want from any supplier: ISO 9001, a QC lab, lot traceability, and a CoA carrying %TS, pH and Brookfield viscosity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Best small-batch find</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Avion Manufacturing (Medina, OH) publishes batch sizes of 1–55 gallons and 60–275 gallons — the best cadence fit found anywhere. ISO 9001. Heat capability is the one unknown; ask it first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Regional coverage filled</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>West: Sunland Chemical (LA — jacketed from 50 gal). Northeast: Shamrock Technologies (Newark NJ — 50-gal jacketed oil-heated kettles, ISO 9001). Midwest: Applied Material Solutions (WI — steam and hot-oil reactors from 140 gal).</t>
-        </is>
-      </c>
+      <c r="C19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Non-obvious category worth a look</t>
+          <t>ISO 13485 NOT required — RESOLVED</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Mallard Creek Polymers (Charlotte, NC) — emulsion polymer plants DISSOLVE PVOH IN HOT WATER as a routine step in vinyl acetate emulsion production. That capability is real but never advertised as 'PVA tolling.'</t>
+          <t>Confirmed by Oscar: we do not need an ISO 13485 supplier. That closes an open blocker and simplifies the search. The medical-grade candidates found in research (Polysciences, Hydromer, HR Pharmaceuticals, Strukmyer, GeminiBio, Kingchem, Alpha Teknova, Biocoat, NEXT Medical) are therefore DEPRIORITIZED to Tier C — they would price well above the incumbent for a certification we do not need. They stay listed only as a fallback if Quality later asks for a stricter supply chain. What we DO still want from any supplier: ISO 9001, a QC lab, lot traceability, and a CoA carrying %TS, pH and Brookfield viscosity.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
+          <t>Best small-batch find</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Avion Manufacturing (Medina, OH) publishes batch sizes of 1–55 gallons and 60–275 gallons — the best cadence fit found anywhere. ISO 9001. Heat capability is the one unknown; ask it first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Regional coverage filled</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>West: Sunland Chemical (LA — jacketed from 50 gal). Northeast: Shamrock Technologies (Newark NJ — 50-gal jacketed oil-heated kettles, ISO 9001). Midwest: Applied Material Solutions (WI — steam and hot-oil reactors from 140 gal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Non-obvious category worth a look</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Mallard Creek Polymers (Charlotte, NC) — emulsion polymer plants DISSOLVE PVOH IN HOT WATER as a routine step in vinyl acetate emulsion production. That capability is real but never advertised as 'PVA tolling.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="11" t="inlineStr">
+        <is>
           <t>One diligence warning</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Medical Products Laboratories (Philadelphia) looks like a strong process match on paper but has an FDA warning letter. Do not advance without confirming it is closed out. Listed so it's on your radar, not as a recommendation.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>HOW TO READ THE TIERS</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="7" t="inlineStr">
+      <c r="C25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Tier A</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Published evidence supports the heat gate AND a toll model AND a workable batch size. Call these first.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="7" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Tier B</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Real, capable shops where one or both gates are unpublished. One phone call moves them to A or out.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="7" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Tier C</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Special role — resin supplier, distributor, technical resource — or a scale/focus mismatch. Not primary toll targets.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="7" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Two questions decide everything</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>(1) Can you reach AND HOLD 90–95 C for 30–45 min? (2) What is your minimum batch size? Most candidates die on one of these, and both are cheap to ask.</t>
         </is>
@@ -4984,46 +5016,50 @@
       <c r="H5" s="32" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="n">
+      <c r="A6" s="20" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>BLOCKER</t>
-        </is>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>Internal — whoever holds SNP CoA history</t>
-        </is>
-      </c>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="inlineStr">
-        <is>
-          <t>Pull the viscosity target AND tolerance from SNP CoA history (Brookfield, spindle #3, 10 RPM, 25 C). Until this exists, nobody can quote firmly or pass/fail a trial batch.</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="inlineStr">
-        <is>
-          <t>This has been pending the whole project and gates every firm quote and every qualification.</t>
-        </is>
-      </c>
-      <c r="G6" s="29" t="inlineStr">
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Viscosity specification</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>SPEC CONFIRMED: Brookfield viscosity &lt; 2,500 cps, spindle #3, 10 RPM, 25 C. Put this in every RFQ and on every CoA, and use it as the pass/fail criterion for any qualification batch.</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Was the longest-standing blocker on this project. With it, suppliers can quote firmly and a trial batch can actually be judged pass/fail. Also good news commercially: under 2,500 cps is an easily pumpable, easily filterable fluid — no special high-viscosity equipment needed, so no blender can charge a premium for 'difficult' handling.</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
         <is>
           <t>Oscar</t>
         </is>
       </c>
-      <c r="H6" s="29" t="inlineStr"/>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
@@ -5063,7 +5099,7 @@
       <c r="A8" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="33" t="inlineStr">
+      <c r="B8" s="34" t="inlineStr">
         <is>
           <t>BLOCKER</t>
         </is>
@@ -5271,7 +5307,7 @@
       <c r="A15" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="34" t="inlineStr">
+      <c r="B15" s="33" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -5307,7 +5343,7 @@
       <c r="A16" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="34" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -5343,7 +5379,7 @@
       <c r="A17" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="B17" s="33" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5379,7 +5415,7 @@
       <c r="A18" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="34" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -5415,7 +5451,7 @@
       <c r="A19" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="34" t="inlineStr">
+      <c r="B19" s="33" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -5451,7 +5487,7 @@
       <c r="A20" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="34" t="inlineStr">
+      <c r="B20" s="33" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -5487,7 +5523,7 @@
       <c r="A21" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="34" t="inlineStr">
+      <c r="B21" s="33" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -5523,7 +5559,7 @@
       <c r="A22" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="34" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -5559,7 +5595,7 @@
       <c r="A23" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="34" t="inlineStr">
+      <c r="B23" s="33" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -5609,7 +5645,7 @@
       <c r="A25" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="34" t="inlineStr">
+      <c r="B25" s="33" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -5645,7 +5681,7 @@
       <c r="A26" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="34" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -5681,7 +5717,7 @@
       <c r="A27" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="34" t="inlineStr">
+      <c r="B27" s="33" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -5717,7 +5753,7 @@
       <c r="A28" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="34" t="inlineStr">
+      <c r="B28" s="33" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -5753,7 +5789,7 @@
       <c r="A29" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="34" t="inlineStr">
+      <c r="B29" s="33" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -5789,7 +5825,7 @@
       <c r="A30" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="34" t="inlineStr">
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -5825,7 +5861,7 @@
       <c r="A31" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="34" t="inlineStr">
+      <c r="B31" s="33" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -5861,7 +5897,7 @@
       <c r="A32" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="34" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -5911,7 +5947,7 @@
       <c r="A34" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="34" t="inlineStr">
+      <c r="B34" s="33" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -5947,7 +5983,7 @@
       <c r="A35" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="34" t="inlineStr">
+      <c r="B35" s="33" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -5990,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C18"/>
+  <dimension ref="B2:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6022,7 +6058,7 @@
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="36" t="inlineStr"/>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Toll blend, 1 drum/week: aqueous PVA, must hold 90-95 C</t>
         </is>
@@ -6036,13 +6072,13 @@
       </c>
       <c r="C8" s="4" t="n"/>
     </row>
-    <row r="9" ht="290" customHeight="1">
+    <row r="9" ht="300" customHeight="1">
       <c r="B9" s="36" t="inlineStr"/>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Hello,
 We're setting up a second source for a recurring toll blend: one 55-gallon drum a week, about 50 a year, made to order. We supply the raw materials and the formula; you charge a conversion fee.
-The product is an aqueous PVA solution, roughly 10-12% solids. One step is pass/fail: the batch has to reach 90-95 C and hold there 30-45 minutes under agitation. If your equipment tops out below 90 C, this isn't a fit — better we both know now.
+The product is an aqueous PVA solution, roughly 10-12% solids, finished viscosity under 2,500 cps (Brookfield, spindle #3, 10 RPM, 25 C). One step is pass/fail: the batch has to reach 90-95 C and hold there 30-45 minutes under agitation. If your equipment tops out below 90 C, this isn't a fit — better we both know now.
 If it can, three questions:
 1. Can you run this?
 2. What's your minimum batch size?
@@ -6061,12 +6097,12 @@
       </c>
       <c r="C11" s="4" t="n"/>
     </row>
-    <row r="12" ht="170" customHeight="1">
+    <row r="12" ht="180" customHeight="1">
       <c r="B12" s="36" t="inlineStr"/>
       <c r="C12" s="37" t="inlineStr">
         <is>
           <t>Looking for a second source for a recurring toll blend: one 55-gallon drum a week, about 50 a year, made to order. We supply the raw materials and the formula; you charge a conversion fee.
-Product is an aqueous PVA solution, ~10-12% solids, that has to reach 90-95 C and hold 30-45 minutes under agitation. If your equipment tops out below 90 C, this isn't a fit.
+Product is an aqueous PVA solution, ~10-12% solids, under 2,500 cps, that has to reach 90-95 C and hold 30-45 minutes under agitation. If your equipment tops out below 90 C, this isn't a fit.
 If it can: can you run it, what's your minimum batch size, and roughly what would you charge per 55-gallon drum (~450 lb net)? If you quote per pound, please say per pound of what — finished solution or dry resin.</t>
         </is>
       </c>
@@ -6090,14 +6126,40 @@
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>IF THEY ASK FOR SPEC DETAIL (send after they confirm they can do it)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="210" customHeight="1">
+      <c r="B18" s="36" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Aqueous polyvinyl alcohol solution, made to order.
+• Total solids: 10-12%, in water
+• Viscosity: UNDER 2,500 cps — Brookfield, spindle #3, 10 RPM, 25 C
+• Process: heat to 90-95 C and hold 30-45 min under agitation to fully dissolve; cool to &lt;=40 C; filter to 200 micron; fill 55-gal drums (~450 lb net)
+• Materials: we supply the resin and all other raw materials
+• Shelf life: 18 days — made fresh to order, no stockpiling
+• Cadence: ~1 drum/week, ~50 drums/year
+• CoA required every shipment: lot #, production date, % total solids, final pH, Brookfield viscosity (spindle #3, 10 RPM, 25 C)
+• Quality: ISO 9001 and lot traceability preferred. ISO 13485 not required.
+• Handling: protect from freezing in transit and storage
+Full formula released under NDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
           <t>WHAT CHANGED vs your original, and why</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n"/>
-    </row>
-    <row r="18" ht="300" customHeight="1">
-      <c r="B18" s="36" t="inlineStr"/>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="300" customHeight="1">
+      <c r="B21" s="36" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Your original was good and short — these keep that. What was added, and the reason for each:
 • THE HOLD, not just the temperature. Your version said 'heat up to 95 C.' The real gate is holding 90-95 C for 30-45 minutes — that is what separates a real heating system from one that can briefly touch temperature. It also states the failure mode plainly ('if your equipment tops out below 90 C') so a shop running 85 C cannot talk itself into a yes.
@@ -6280,19 +6342,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="48" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>Internal — spec owner</t>
         </is>
       </c>
-      <c r="C13" s="49" t="inlineStr">
-        <is>
-          <t>Whoever holds SNP CoA history</t>
-        </is>
-      </c>
-      <c r="D13" s="49" t="inlineStr">
-        <is>
-          <t>The viscosity target and tolerance. Still pending, and it blocks every firm quote and every trial pass/fail.</t>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Viscosity specification</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>RESOLVED — &lt; 2,500 cps, Brookfield spindle #3, 10 RPM, 25 C. Now the pass/fail criterion for any qualification batch, and a required CoA field.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Glossary tab explaining project acronyms and concepts
74 entries in 7 sections, written for the buyer rather than the chemist, each
with a 'why it matters to us' column. Sections: the viscosity spec decoded
(cps, Brookfield, spindle #3, 10 RPM, 25 C, and why all four must be stated
together); PVA chemistry incl. why degree of hydrolysis drives the 90-95 C
requirement; process and equipment; materials of construction; quality and
documentation; commercial terms; units and conversions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Supplier_Longlist.xlsx
+++ b/PVA second supplier initiative/PVA_Supplier_Longlist.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Action Plan" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="RFQ Templates" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Stakeholder Map" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Glossary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,6 +100,12 @@
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -169,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -300,6 +307,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6395,4 +6410,1240 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:D78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Glossary — the acronyms and concepts in this project, in plain English</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Written for the buyer, not the chemist. 'Why it matters to us' is the practical consequence for this sourcing decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="50" t="inlineStr">
+        <is>
+          <t>1. THE VISCOSITY SPEC, DECODED  —  'less than 2,500 cps, Brookfield, spindle #3, 10 RPM, 25 C'</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Viscosity</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>How thick a liquid is — its resistance to flowing. Water is thin, honey is thick.</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>It is our main quality number. Too thin or too thick means the PVA did not dissolve correctly, or the solids are off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>cps  (or cP) — centipoise</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>The unit viscosity is measured in. Reference points: water ≈ 1 cps; olive oil ≈ 80; motor oil ≈ 200-400; corn syrup ≈ 2,000-5,000; honey ≈ 10,000; ketchup ≈ 50,000. (1 cps = 1 mPa·s, the metric equivalent you may see instead.)</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>Our limit of 2,500 cps is roughly thick-syrup consistency — clearly viscous, but pourable and pumpable with ordinary equipment. For a coatings or adhesives toll blender this is an easy fluid; many of them routinely run 50,000+ cps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Brookfield</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>The brand of viscometer that became the industry standard method. It spins a metal probe in the liquid and measures how hard the liquid resists — that resistance converts to viscosity.</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>Saying 'Brookfield' pins down the METHOD. A different instrument type can give a different number for the same liquid, so the method has to match or the numbers are not comparable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Spindle #3</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>The specific probe that spins in the liquid. Brookfield spindles are numbered — lower numbers are physically larger (for thin liquids), higher numbers are smaller (for thick liquids). #3 is a mid-range probe.</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>The spindle sets the measuring range. The SAME liquid measured with a different spindle gives a DIFFERENT number. This is why the spindle must be named, not assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>10 RPM</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>How fast the spindle turns — 10 revolutions per minute.</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>This is the one people miss. Polymer solutions like ours are 'shear-thinning': the faster you stir them, the thinner they read. The same drum can measure ~3,000 cps at 5 RPM and ~2,000 at 20 RPM. Quote a viscosity without the RPM and the number means nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>25 C  (77 F)</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>The temperature of the sample when measured.</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Viscosity falls sharply as liquid warms. A sample measured warm reads far lower than the same sample at 25 C. Specifying 25 C stops a supplier from passing a batch simply by testing it warm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Why all four together</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Method + spindle + speed + temperature.</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Change any one and the number changes. This is why our CoA requirement names all four — it is the difference between a spec and a suggestion. If a supplier reports viscosity their own way, we cannot compare it to the incumbent's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="50" t="inlineStr">
+        <is>
+          <t>2. THE CHEMISTRY</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C15" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D15" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="52" t="inlineStr">
+        <is>
+          <t>PVA  /  PVOH</t>
+        </is>
+      </c>
+      <c r="C16" s="53" t="inlineStr">
+        <is>
+          <t>Polyvinyl alcohol. A synthetic polymer that dissolves in water. Both abbreviations mean the same thing (PVOH is used to avoid confusion with polyvinyl acetate, PVAc).</t>
+        </is>
+      </c>
+      <c r="D16" s="53" t="inlineStr">
+        <is>
+          <t>The active ingredient of our product. We buy it as a dry solid and dissolve it in water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="48" t="inlineStr">
+        <is>
+          <t>Resin</t>
+        </is>
+      </c>
+      <c r="C17" s="49" t="inlineStr">
+        <is>
+          <t>In this industry, the dry solid polymer before it is dissolved — granules or powder.</t>
+        </is>
+      </c>
+      <c r="D17" s="49" t="inlineStr">
+        <is>
+          <t>Distinguishes the dry raw material from the finished liquid. This distinction is exactly what made CJB's '$8.00 per pound' quote ambiguous: per pound of dry resin, or of finished liquid? A 450 lb drum contains only ~45-50 lb of resin — a ~10x difference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Degree of hydrolysis</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>PVA is made by converting polyvinyl acetate. The degree of hydrolysis is how much of that conversion was completed: partially hydrolyzed ≈ 87-89%, fully ≈ 98-99%, SUPER-hydrolyzed &gt; 99%.</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>THE reason our process needs 90-95 C. The more hydrolyzed the polymer, the more tightly its chains pack together, and the hotter the water must be to pull them apart. Partially hydrolyzed PVA dissolves in warm water; ours does not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="52" t="inlineStr">
+        <is>
+          <t>High molecular weight (high-MW)</t>
+        </is>
+      </c>
+      <c r="C19" s="53" t="inlineStr">
+        <is>
+          <t>Long polymer chains rather than short ones.</t>
+        </is>
+      </c>
+      <c r="D19" s="53" t="inlineStr">
+        <is>
+          <t>Long chains dissolve more slowly (hence the 30-45 minute hold) and thicken the solution more (hence a viscosity spec at all).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="52" t="inlineStr">
+        <is>
+          <t>Total solids  /  %TS</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="inlineStr">
+        <is>
+          <t>The percentage of the finished liquid that is actual material rather than water. Ours is 10-12%.</t>
+        </is>
+      </c>
+      <c r="D20" s="53" t="inlineStr">
+        <is>
+          <t>The concentration check. Measured by drying a sample and weighing what remains. If water boils off during an uncovered cook, %TS drifts up and viscosity with it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="52" t="inlineStr">
+        <is>
+          <t>Aqueous</t>
+        </is>
+      </c>
+      <c r="C21" s="53" t="inlineStr">
+        <is>
+          <t>Water-based — the liquid it is dissolved in is water.</t>
+        </is>
+      </c>
+      <c r="D21" s="53" t="inlineStr">
+        <is>
+          <t>Distinguishes our product from solvent-based chemistry. It also means suppliers set up only for solvent work are the wrong shops.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>Brand names you will see</t>
+        </is>
+      </c>
+      <c r="C22" s="53" t="inlineStr">
+        <is>
+          <t>Selvol (Sekisui) · Poval and Elvanol (Kuraray) · Gohsenol (Mitsubishi Chemical). Our spec references Selvol S-1551F-D or equivalent.</t>
+        </is>
+      </c>
+      <c r="D22" s="53" t="inlineStr">
+        <is>
+          <t>These are competing brands of the same class of material. 'Or equivalent' means another maker's matching grade is acceptable — useful leverage on resin price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>NaCl</t>
+        </is>
+      </c>
+      <c r="C23" s="53" t="inlineStr">
+        <is>
+          <t>Common salt (sodium chloride), a minor ingredient in our formula.</t>
+        </is>
+      </c>
+      <c r="D23" s="53" t="inlineStr">
+        <is>
+          <t>Small amount, but it is why 316L stainless matters — chlorides corrode lesser steels (see section 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>Biocide  /  Proxel BD20</t>
+        </is>
+      </c>
+      <c r="C24" s="53" t="inlineStr">
+        <is>
+          <t>A preservative that stops bacteria and mould growing in a water-based product. Proxel is a specific brand.</t>
+        </is>
+      </c>
+      <c r="D24" s="53" t="inlineStr">
+        <is>
+          <t>Water-based products spoil. Our process adds it hot in the final 10 minutes — a sequencing detail a blender must follow exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="50" t="inlineStr">
+        <is>
+          <t>3. THE PROCESS AND EQUIPMENT</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C26" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D26" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>Toll blending  /  toll manufacturing</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
+        <is>
+          <t>WE supply the raw materials and the formula; the manufacturer only processes them and charges a conversion fee.</t>
+        </is>
+      </c>
+      <c r="D27" s="41" t="inlineStr">
+        <is>
+          <t>Our preferred model. It removes their markup on materials and lets us control the exact resin grade — which matters for consistency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>Contract manufacturing</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="inlineStr">
+        <is>
+          <t>The manufacturer BUYS the raw materials themselves and sells us finished product, marking up the materials.</t>
+        </is>
+      </c>
+      <c r="D28" s="53" t="inlineStr">
+        <is>
+          <t>The alternative model. Usually simpler but more expensive, because you pay a margin on materials too (CJB proposed cost + 15%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="52" t="inlineStr">
+        <is>
+          <t>Conversion fee</t>
+        </is>
+      </c>
+      <c r="C29" s="53" t="inlineStr">
+        <is>
+          <t>The charge for the processing work alone — labour, energy, QC, cleaning, packaging, overhead and profit. No materials.</t>
+        </is>
+      </c>
+      <c r="D29" s="53" t="inlineStr">
+        <is>
+          <t>The number to compare across toll blenders. Ask for it per drum or per batch, never as a bare 'per pound'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="52" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="C30" s="53" t="inlineStr">
+        <is>
+          <t>One discrete production run. Everything is mixed together, processed, then packaged.</t>
+        </is>
+      </c>
+      <c r="D30" s="53" t="inlineStr">
+        <is>
+          <t>Our product is made in batches, one drum at a time. Opposite of continuous production, which runs nonstop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t>Minimum batch size</t>
+        </is>
+      </c>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>The smallest quantity a given vessel can run properly — a tank must be filled to a certain level for the agitator to work.</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="inlineStr">
+        <is>
+          <t>One of our two killer questions. Our drum is ~50 gallons. A shop whose smallest vessel is 2,000 gallons cannot make it economically, whatever their price list says.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="52" t="inlineStr">
+        <is>
+          <t>MOQ — minimum order quantity</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="inlineStr">
+        <is>
+          <t>The smallest ORDER they will accept commercially. Different from minimum batch size, which is a physical limit.</t>
+        </is>
+      </c>
+      <c r="D32" s="53" t="inlineStr">
+        <is>
+          <t>A shop might physically manage 50 gallons but refuse orders under 500. Ask both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="42" t="inlineStr">
+        <is>
+          <t>Jacketed vessel</t>
+        </is>
+      </c>
+      <c r="C33" s="43" t="inlineStr">
+        <is>
+          <t>A tank with a hollow outer layer — the 'jacket' — through which steam, hot oil, or cooling water flows to heat or cool the contents. The heating fluid never touches the product.</t>
+        </is>
+      </c>
+      <c r="D33" s="43" t="inlineStr">
+        <is>
+          <t>This is the equipment that clears our 90-95 C requirement. A tank without a jacket generally cannot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="52" t="inlineStr">
+        <is>
+          <t>Steam jacket  /  hot oil</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="inlineStr">
+        <is>
+          <t>The two common heating fluids. Low-pressure steam runs about 110-120 C; hot oil systems can exceed 250 C.</t>
+        </is>
+      </c>
+      <c r="D34" s="53" t="inlineStr">
+        <is>
+          <t>Either comfortably clears our 90-95 C. This is why 'steam-jacketed' on a supplier's website is a strong positive signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="52" t="inlineStr">
+        <is>
+          <t>Reactor</t>
+        </is>
+      </c>
+      <c r="C35" s="53" t="inlineStr">
+        <is>
+          <t>A jacketed vessel built for chemical reactions — heavier duty, often pressure-rated, with better temperature control.</t>
+        </is>
+      </c>
+      <c r="D35" s="53" t="inlineStr">
+        <is>
+          <t>More capability than we need (we only dissolve, we do not react), but reactors always clear the heat gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="40" t="inlineStr">
+        <is>
+          <t>Pilot plant  /  pilot reactor</t>
+        </is>
+      </c>
+      <c r="C36" s="41" t="inlineStr">
+        <is>
+          <t>Small-scale equipment used for trial batches and development before full production.</t>
+        </is>
+      </c>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>Our best opening. Piedmont's 5-100 gallon pilot reactors fit our ~50-gallon batch almost exactly, where their production vessels would be far too big.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="52" t="inlineStr">
+        <is>
+          <t>Agitation</t>
+        </is>
+      </c>
+      <c r="C37" s="53" t="inlineStr">
+        <is>
+          <t>Stirring. 'Variable speed' means the rate can be adjusted.</t>
+        </is>
+      </c>
+      <c r="D37" s="53" t="inlineStr">
+        <is>
+          <t>PVA must be stirred steadily as it dissolves or it clumps. Too vigorous too early also causes problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="48" t="inlineStr">
+        <is>
+          <t>Fisheyes  /  gels</t>
+        </is>
+      </c>
+      <c r="C38" s="49" t="inlineStr">
+        <is>
+          <t>Lumps of partly-dissolved polymer — a soft outer layer wrapped around dry powder inside.</t>
+        </is>
+      </c>
+      <c r="D38" s="49" t="inlineStr">
+        <is>
+          <t>The classic PVA failure, and what a trial batch is really testing for. Caused by too-low temperature, too-short hold, or bad addition order. Brenntag's attempt failed this way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="52" t="inlineStr">
+        <is>
+          <t>200 micron filtration</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="inlineStr">
+        <is>
+          <t>Straining the finished liquid through a screen with 200-micrometre openings (about 0.2 mm) to catch undissolved bits. Roughly equivalent to a 70-mesh screen.</t>
+        </is>
+      </c>
+      <c r="D39" s="53" t="inlineStr">
+        <is>
+          <t>A relatively coarse polish, not fine filtration. It removes gels and specks; it does not sterilise or clarify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="52" t="inlineStr">
+        <is>
+          <t>Micron vs mesh</t>
+        </is>
+      </c>
+      <c r="C40" s="53" t="inlineStr">
+        <is>
+          <t>Two ways of stating filter fineness, running in OPPOSITE directions. Micron = hole size, so smaller number = finer. Mesh = wires per inch, so higher number = finer. 200 micron ≈ 70 mesh; 100 mesh ≈ 150 micron (finer than we require).</t>
+        </is>
+      </c>
+      <c r="D40" s="53" t="inlineStr">
+        <is>
+          <t>Easy to misread in a supplier's spec. If they say '100 mesh', that is finer than our 200 micron and therefore acceptable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="42" t="inlineStr">
+        <is>
+          <t>Shelf life — 18 days</t>
+        </is>
+      </c>
+      <c r="C41" s="43" t="inlineStr">
+        <is>
+          <t>How long the product stays usable after production.</t>
+        </is>
+      </c>
+      <c r="D41" s="43" t="inlineStr">
+        <is>
+          <t>Drives everything about cadence. We cannot stockpile, so we need weekly made-to-order batches — which is why a shop with a 250-gallon minimum is a problem: ~4.5 drums made, only ~2 usable in time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="50" t="inlineStr">
+        <is>
+          <t>4. MATERIALS OF CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C43" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D43" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="52" t="inlineStr">
+        <is>
+          <t>Stainless steel  304 vs 316L</t>
+        </is>
+      </c>
+      <c r="C44" s="53" t="inlineStr">
+        <is>
+          <t>Grades of stainless. 316L contains molybdenum, which resists pitting from chlorides. The 'L' means low carbon, which resists corrosion at welds.</t>
+        </is>
+      </c>
+      <c r="D44" s="53" t="inlineStr">
+        <is>
+          <t>Our formula contains salt (NaCl) — a chloride. Over time chlorides pit ordinary 304 steel, which risks both corrosion and metal contamination. 316L is the safer contact surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="52" t="inlineStr">
+        <is>
+          <t>Glass-lined</t>
+        </is>
+      </c>
+      <c r="C45" s="53" t="inlineStr">
+        <is>
+          <t>A steel vessel with a fused glass interior — chemically inert.</t>
+        </is>
+      </c>
+      <c r="D45" s="53" t="inlineStr">
+        <is>
+          <t>Common in reactors for aggressive chemistry. Fine for us, simply more than we need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="52" t="inlineStr">
+        <is>
+          <t>Hastelloy</t>
+        </is>
+      </c>
+      <c r="C46" s="53" t="inlineStr">
+        <is>
+          <t>A high-nickel alloy for severely corrosive service.</t>
+        </is>
+      </c>
+      <c r="D46" s="53" t="inlineStr">
+        <is>
+          <t>Seeing it on a supplier's equipment list signals a heavy-duty synthesis shop — usually a sign they are bigger and pricier than we need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="50" t="inlineStr">
+        <is>
+          <t>5. QUALITY AND DOCUMENTATION</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C48" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D48" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="40" t="inlineStr">
+        <is>
+          <t>CoA — Certificate of Analysis</t>
+        </is>
+      </c>
+      <c r="C49" s="41" t="inlineStr">
+        <is>
+          <t>A document listing the ACTUAL measured test results for that specific lot.</t>
+        </is>
+      </c>
+      <c r="D49" s="41" t="inlineStr">
+        <is>
+          <t>What we require every shipment: lot #, production date, %TS, final pH, and Brookfield viscosity. Real numbers, per batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="52" t="inlineStr">
+        <is>
+          <t>CoC — Certificate of Conformance</t>
+        </is>
+      </c>
+      <c r="C50" s="53" t="inlineStr">
+        <is>
+          <t>A statement that the product meets spec, without necessarily giving the measured numbers.</t>
+        </is>
+      </c>
+      <c r="D50" s="53" t="inlineStr">
+        <is>
+          <t>Weaker than a CoA. If a supplier offers a CoC, ask for a CoA instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="52" t="inlineStr">
+        <is>
+          <t>Lot  /  batch number</t>
+        </is>
+      </c>
+      <c r="C51" s="53" t="inlineStr">
+        <is>
+          <t>The unique ID for one production run.</t>
+        </is>
+      </c>
+      <c r="D51" s="53" t="inlineStr">
+        <is>
+          <t>Traceability. If a problem appears later, the lot number identifies exactly which batch and when it was made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="52" t="inlineStr">
+        <is>
+          <t>Retained sample</t>
+        </is>
+      </c>
+      <c r="C52" s="53" t="inlineStr">
+        <is>
+          <t>A sample of each batch kept by the manufacturer for a set period.</t>
+        </is>
+      </c>
+      <c r="D52" s="53" t="inlineStr">
+        <is>
+          <t>Lets a dispute be settled later by re-testing what was actually shipped. Worth asking who retains and for how long.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="52" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="C53" s="53" t="inlineStr">
+        <is>
+          <t>Acidity or alkalinity, 0-14. Neutral is 7.</t>
+        </is>
+      </c>
+      <c r="D53" s="53" t="inlineStr">
+        <is>
+          <t>One of our three QC checks. Drift indicates a formulation or contamination problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="40" t="inlineStr">
+        <is>
+          <t>ISO 9001</t>
+        </is>
+      </c>
+      <c r="C54" s="41" t="inlineStr">
+        <is>
+          <t>The general quality-management standard — documented, repeatable processes and records. Not industry-specific.</t>
+        </is>
+      </c>
+      <c r="D54" s="41" t="inlineStr">
+        <is>
+          <t>Our practical baseline requirement. Widely held, so asking for it costs nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="40" t="inlineStr">
+        <is>
+          <t>ISO 13485</t>
+        </is>
+      </c>
+      <c r="C55" s="41" t="inlineStr">
+        <is>
+          <t>The quality-management standard specific to MEDICAL DEVICES. Stricter documentation, validation and traceability.</t>
+        </is>
+      </c>
+      <c r="D55" s="41" t="inlineStr">
+        <is>
+          <t>CONFIRMED NOT REQUIRED for us. Worth knowing because it commands a real price premium — which is why the medical-grade suppliers were deprioritised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="52" t="inlineStr">
+        <is>
+          <t>cGMP</t>
+        </is>
+      </c>
+      <c r="C56" s="53" t="inlineStr">
+        <is>
+          <t>'Current Good Manufacturing Practice' — the FDA-enforced rules for making drugs and some devices.</t>
+        </is>
+      </c>
+      <c r="D56" s="53" t="inlineStr">
+        <is>
+          <t>More than we need. Signals a pharma-grade shop and pharma-grade pricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="52" t="inlineStr">
+        <is>
+          <t>FDA registration</t>
+        </is>
+      </c>
+      <c r="C57" s="53" t="inlineStr">
+        <is>
+          <t>A facility listing itself with the FDA. A registration, not an approval or endorsement.</t>
+        </is>
+      </c>
+      <c r="D57" s="53" t="inlineStr">
+        <is>
+          <t>Relevant only if the end use demands it. Ours does not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="52" t="inlineStr">
+        <is>
+          <t>QMSR</t>
+        </is>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
+        <is>
+          <t>FDA's Quality Management System Regulation, which harmonises the old US device rules with ISO 13485.</t>
+        </is>
+      </c>
+      <c r="D58" s="53" t="inlineStr">
+        <is>
+          <t>Came up early as a possible requirement. With ISO 13485 confirmed unnecessary, this is background only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="48" t="inlineStr">
+        <is>
+          <t>FDA warning letter</t>
+        </is>
+      </c>
+      <c r="C59" s="49" t="inlineStr">
+        <is>
+          <t>A formal FDA notice of significant violations at a facility.</t>
+        </is>
+      </c>
+      <c r="D59" s="49" t="inlineStr">
+        <is>
+          <t>A genuine red flag in supplier diligence — one candidate (Medical Products Laboratories) has one open. Never advance a supplier without confirming it is closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="50" t="inlineStr">
+        <is>
+          <t>6. COMMERCIAL AND SOURCING TERMS</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n"/>
+      <c r="D60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C61" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D61" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="52" t="inlineStr">
+        <is>
+          <t>RFQ  /  RFP  /  RFI</t>
+        </is>
+      </c>
+      <c r="C62" s="53" t="inlineStr">
+        <is>
+          <t>Request for Quote (price for a defined thing) · Request for Proposal (how would you solve this) · Request for Information (general capability enquiry).</t>
+        </is>
+      </c>
+      <c r="D62" s="53" t="inlineStr">
+        <is>
+          <t>Ours is genuinely an RFQ: the specification is fixed and we want a price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="40" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="C63" s="41" t="inlineStr">
+        <is>
+          <t>Non-disclosure agreement — a confidentiality contract.</t>
+        </is>
+      </c>
+      <c r="D63" s="41" t="inlineStr">
+        <is>
+          <t>Must be signed before we share the full formula. Our RFQ template deliberately withholds the formula so outreach can start before the NDA is in place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="52" t="inlineStr">
+        <is>
+          <t>Qualification  /  first article</t>
+        </is>
+      </c>
+      <c r="C64" s="53" t="inlineStr">
+        <is>
+          <t>The trial batch proving a new supplier can make the product to spec before production begins.</t>
+        </is>
+      </c>
+      <c r="D64" s="53" t="inlineStr">
+        <is>
+          <t>What the $4,900 CJB batch was. Its pass/fail test is now concrete: does it come in under 2,500 cps at our stated conditions?</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="52" t="inlineStr">
+        <is>
+          <t>Second source  /  dual sourcing</t>
+        </is>
+      </c>
+      <c r="C65" s="53" t="inlineStr">
+        <is>
+          <t>Deliberately qualifying a second supplier for the same item.</t>
+        </is>
+      </c>
+      <c r="D65" s="53" t="inlineStr">
+        <is>
+          <t>The whole point of this project. It is insurance against a single supplier failing — and the premium is the extra cost over single-sourcing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="40" t="inlineStr">
+        <is>
+          <t>Cost of redundancy  /  premium</t>
+        </is>
+      </c>
+      <c r="C66" s="41" t="inlineStr">
+        <is>
+          <t>The EXTRA annual cost of buying some volume from a pricier second source instead of all from the incumbent.</t>
+        </is>
+      </c>
+      <c r="D66" s="41" t="inlineStr">
+        <is>
+          <t>The real decision number — not total spend, since those drums get bought either way. See the cost-scenarios workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="52" t="inlineStr">
+        <is>
+          <t>Incumbent</t>
+        </is>
+      </c>
+      <c r="C67" s="53" t="inlineStr">
+        <is>
+          <t>The current supplier.</t>
+        </is>
+      </c>
+      <c r="D67" s="53" t="inlineStr">
+        <is>
+          <t>SNP, at $0.75/lb delivered. Also our price benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="52" t="inlineStr">
+        <is>
+          <t>Lead time</t>
+        </is>
+      </c>
+      <c r="C68" s="53" t="inlineStr">
+        <is>
+          <t>Time from placing the order to receiving goods.</t>
+        </is>
+      </c>
+      <c r="D68" s="53" t="inlineStr">
+        <is>
+          <t>With an 18-day shelf life, a long lead time eats the usable window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="52" t="inlineStr">
+        <is>
+          <t>LTL freight</t>
+        </is>
+      </c>
+      <c r="C69" s="53" t="inlineStr">
+        <is>
+          <t>'Less than truckload' — shipping that does not fill a truck, so the load is consolidated with others.</t>
+        </is>
+      </c>
+      <c r="D69" s="53" t="inlineStr">
+        <is>
+          <t>How a single drum ships. Costs much more per pound than a full load, which is why freight is a real line item at our volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="52" t="inlineStr">
+        <is>
+          <t>Drum  /  IBC tote</t>
+        </is>
+      </c>
+      <c r="C70" s="53" t="inlineStr">
+        <is>
+          <t>55-gallon drum ≈ 450 lb of our product. An IBC tote is a large cube, typically 275-330 gallons.</t>
+        </is>
+      </c>
+      <c r="D70" s="53" t="inlineStr">
+        <is>
+          <t>We buy drums. A tote would exceed what we can use inside the 18-day shelf life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="52" t="inlineStr">
+        <is>
+          <t>Consignment</t>
+        </is>
+      </c>
+      <c r="C71" s="53" t="inlineStr">
+        <is>
+          <t>We own the raw materials and place them at the supplier's site; they process from our stock.</t>
+        </is>
+      </c>
+      <c r="D71" s="53" t="inlineStr">
+        <is>
+          <t>The purest version of tolling, and worth proposing — it removes any markup on materials entirely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="50" t="inlineStr">
+        <is>
+          <t>7. UNITS AND QUICK CONVERSIONS</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="n"/>
+      <c r="D72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="51" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="C73" s="51" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D73" s="51" t="inlineStr">
+        <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="40" t="inlineStr">
+        <is>
+          <t>Our drum</t>
+        </is>
+      </c>
+      <c r="C74" s="41" t="inlineStr">
+        <is>
+          <t>55 US gallons ≈ 450 lb net of finished solution (density just above water, ~8.5 lb/gal).</t>
+        </is>
+      </c>
+      <c r="D74" s="41" t="inlineStr">
+        <is>
+          <t>Convert every quote to $ per drum. It is the only way to compare a per-pound quote against a per-batch one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="52" t="inlineStr">
+        <is>
+          <t>Our demand</t>
+        </is>
+      </c>
+      <c r="C75" s="53" t="inlineStr">
+        <is>
+          <t>1,300 lb/week ≈ 2.9 drums/week ≈ 150 drums/year. A 35% second-source share ≈ 1 drum/week.</t>
+        </is>
+      </c>
+      <c r="D75" s="53" t="inlineStr">
+        <is>
+          <t>The volume any supplier is being asked to serve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="40" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C76" s="41" t="inlineStr">
+        <is>
+          <t>90-95 C = 194-203 F.  25 C = 77 F.  40 C = 104 F.</t>
+        </is>
+      </c>
+      <c r="D76" s="41" t="inlineStr">
+        <is>
+          <t>US shops often work in Fahrenheit. Quoting both avoids a misunderstanding on the single most important requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="52" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C77" s="53" t="inlineStr">
+        <is>
+          <t>1 kg = 2.205 lb.  1 metric tonne (MT) = 1,000 kg = 2,205 lb ≈ 4.9 of our drums.</t>
+        </is>
+      </c>
+      <c r="D77" s="53" t="inlineStr">
+        <is>
+          <t>Commodity resin prices are usually published per kg or per MT, so converting to $/lb is needed to compare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="52" t="inlineStr">
+        <is>
+          <t>Viscosity</t>
+        </is>
+      </c>
+      <c r="C78" s="53" t="inlineStr">
+        <is>
+          <t>1 cps = 1 mPa·s (millipascal-second).</t>
+        </is>
+      </c>
+      <c r="D78" s="53" t="inlineStr">
+        <is>
+          <t>Some suppliers and instruments report in mPa·s. The numbers are identical — no conversion needed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Eliminate Columbus Chemical Industries (CCI) — cannot hold temperature
CCI Phoenix confirmed directly to Oscar that they cannot hold the required
temperature. Marked ELIMINATED. This overrides the old roster note recording
'heating/cooling: Yes', which was never verified.

Added a prominent warning distinguishing COLUMBUS Chemical INDUSTRIES (eliminated)
from COLUMBIA Chemical of Akron OH (active Tier B) — the names are one letter
apart and both are Midwest chemical firms.

Also recorded: the heat gate has now eliminated 3 suppliers (ILC Dover, ArroChem,
CCI), confirming it should be the opening question on every contact.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Supplier_Longlist.xlsx
+++ b/PVA second supplier initiative/PVA_Supplier_Longlist.xlsx
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C36"/>
+  <dimension ref="B2:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -931,134 +931,178 @@
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>NATIONWIDE SWEEP — what searching beyond the East Coast actually found</t>
+          <t>SUPPLIER RESPONSES — live status</t>
         </is>
       </c>
       <c r="C25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>The structural finding</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Across the Midwest, Mountain, South-Central and Western states, a clear pattern emerged: shops that publish a batch MINIMUM publish 200-3,000 gallons, and shops that publish HEAT capability don't publish minimums. Almost nobody publishes both. That is the real explanation for the $8.00-8.50/lb quote — it was not bad luck or a bad actor, it is what the industry's published capability floor implies for a 50-gallon job. The handful of shops that break the pattern are the ones worth our time.</t>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>ELIMINATED: Columbus Chemical Industries (CCI), Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>CCI told Oscar directly they CANNOT HOLD THE TEMPERATURE. Eliminated. Note this overrides the old roster entry, which recorded 'heating/cooling: Yes' — that was never verified, and direct contact has now disproven it. Their excellent batch range (20 L to 20,000 L) is irrelevant: the heat gate is binary.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>3 companies now publish BOTH gates</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Specialty Organics (Adelanto CA) — 5-to-500-gallon jacketed mixers plus a 150 psi steam boiler. Ascent Chemicals (Cleveland TN) — 5-gal jacketed reactors, steam and hot-oil, ISO 9001, CoA every shipment, and a stated customer-supplies-materials toll model. Seatex (Rosenberg TX) — a 100-gal steam-jacketed pilot reactor plus a 100-ton chilling system, which is precisely our heat-then-cool cycle. All three go to Tier A.</t>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>WATCH THE NAME — two different companies</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>COLUMBUS Chemical INDUSTRIES (Columbus WI / Phoenix AZ) is ELIMINATED. COLUMBIA Chemical (Akron OH) is a SEPARATE company and remains an active Tier B candidate. The names are one letter apart and both are Midwest chemical firms — do not let the CCI elimination knock out Columbia by mistake.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
         <is>
+          <t>The heat gate is now 3-for-3 as a screen</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>ILC Dover (85 C ceiling), ArroChem (85 C ceiling), and now CCI have all failed on holding temperature. That is three suppliers eliminated by one question. It confirms the tactic: ask about the 90-95 C hold in the first sixty seconds of every contact, before discussing anything else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>NATIONWIDE SWEEP — what searching beyond the East Coast actually found</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>The structural finding</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Across the Midwest, Mountain, South-Central and Western states, a clear pattern emerged: shops that publish a batch MINIMUM publish 200-3,000 gallons, and shops that publish HEAT capability don't publish minimums. Almost nobody publishes both. That is the real explanation for the $8.00-8.50/lb quote — it was not bad luck or a bad actor, it is what the industry's published capability floor implies for a 50-gallon job. The handful of shops that break the pattern are the ones worth our time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>3 companies now publish BOTH gates</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Specialty Organics (Adelanto CA) — 5-to-500-gallon jacketed mixers plus a 150 psi steam boiler. Ascent Chemicals (Cleveland TN) — 5-gal jacketed reactors, steam and hot-oil, ISO 9001, CoA every shipment, and a stated customer-supplies-materials toll model. Seatex (Rosenberg TX) — a 100-gal steam-jacketed pilot reactor plus a 100-ton chilling system, which is precisely our heat-then-cool cycle. All three go to Tier A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
           <t>One error corrected</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Columbia Chemical was previously dropped as 'Brunswick OH — too big' with no evidence cited. Verified directly: they are in AKRON, hold ISO 9001:2015, publish 'heating and cooling capabilities', package into drums/totes/pails, and explicitly market 'smaller scale custom blending'. Un-dropped to Tier B.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="5" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Lead every call with the heat question</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>In roughly 30 Western sites checked, exactly ONE published heat capability. The gate will mostly have to be cleared by phone, not by research. Open with 'do you have a jacketed vessel that will hold 90-95 C for 45 minutes?' and let it disqualify people inside the first minute.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Regions that came back empty</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>Honest answer so nobody re-walks this ground: Louisiana, Arkansas, Mississippi, Kansas and Nebraska produced nothing verifiable. Nevada, Arizona, Idaho and Washington produced nothing qualified. Colorado and Utah are one-name states. Oregon has one verified option (FORREST) plus one unverifiable (Griffin). California carries essentially the entire Western list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>Rejected for scale, with reasons</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>Not padded into the list: Bernard Labs Cincinnati (excellent 250 F heat but a 300-gal minimum = 6 drums, which outlives our 18-day shelf life), McGean (1,000-7,000 gal), Jayne Products (300-2,100 gal), Goodwin (500-40,000 gal), Custom Ag Formulators (200 gal min), Crown Technology and Superior Industrial (5,000 gal), Third Coast (1,000-90,000 gal), Kinpak (300,000 gal). Also rejected: the Texas/Louisiana oilfield blenders as a class, Cosway (no drums), Chemsultants (output is coated film, not drums), and Accublends (domain now for sale — defunct).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO READ THE TIERS</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>Published evidence supports the heat gate AND a toll model AND a workable batch size. Call these first.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="9" t="inlineStr">
         <is>
+          <t>Regions that came back empty</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Honest answer so nobody re-walks this ground: Louisiana, Arkansas, Mississippi, Kansas and Nebraska produced nothing verifiable. Nevada, Arizona, Idaho and Washington produced nothing qualified. Colorado and Utah are one-name states. Oregon has one verified option (FORREST) plus one unverifiable (Griffin). California carries essentially the entire Western list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Rejected for scale, with reasons</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Not padded into the list: Bernard Labs Cincinnati (excellent 250 F heat but a 300-gal minimum = 6 drums, which outlives our 18-day shelf life), McGean (1,000-7,000 gal), Jayne Products (300-2,100 gal), Goodwin (500-40,000 gal), Custom Ag Formulators (200 gal min), Crown Technology and Superior Industrial (5,000 gal), Third Coast (1,000-90,000 gal), Kinpak (300,000 gal). Also rejected: the Texas/Louisiana oilfield blenders as a class, Cosway (no drums), Chemsultants (output is coated film, not drums), and Accublends (domain now for sale — defunct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO READ THE TIERS</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Tier A</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Published evidence supports the heat gate AND a toll model AND a workable batch size. Call these first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="9" t="inlineStr">
+        <is>
           <t>Tier B</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>Real, capable shops where one or both gates are unpublished. One phone call moves them to A or out.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="9" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>Tier C</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Special role — resin supplier, distributor, technical resource — or a scale/focus mismatch. Not primary toll targets.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="9" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>Two questions decide everything</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>(1) Can you reach AND HOLD 90–95 C for 30–45 min? (2) What is your minimum batch size? Most candidates die on one of these, and both are cheap to ask.</t>
         </is>
@@ -2434,42 +2478,42 @@
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>Columbus Chemical (CCI)</t>
+          <t>Custom Chemical Formulators, Inc. (CCFI)</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Columbus WI / Phoenix AZ</t>
+          <t>Santa Fe Springs, CA</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
         <is>
-          <t>https://www.columbuschemical.com</t>
+          <t>https://www.customchem.com</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>Yes — heating/cooling capability</t>
+          <t>PARTIAL, EXPLICIT BUT THIN. Contract manufacturing page lists "In-process heating" as a liquid-production capability, alongside "high shear mixing and variable speed agitation for high viscosity products." So heating exists. NO jacketing detail, NO maximum te…</t>
         </is>
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>Excellent — 20 L to 20,000 L (~5 gal floor); widest range = least shelf-life waste</t>
+          <t>HARD PUBLISHED FLOOR, AND IT IS A PROBLEM: "200 gallon to 6,000 gallon batch size" for liquids (powders: "1,500-6,000 lb. batch size"). They state over 50 tank…</t>
         </is>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001, in-house lab</t>
+          <t>BEST REGULATORY SIGNALS IN THE BATCH: "CCFI is a certified blending facility for FDA, EPA, NSF, Kosher, OMRI, USDA." Also holds a US Drug M…</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>on roster — resume</t>
+          <t>https://www.customchem.com/contact/ | (562) 699-5070 | toll-free (877) 344-2436 | sales@customchem.com</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>ON OUR ROSTER. Lowest batch floor of the roster group; can scale if demand grows.</t>
+          <t>CORRECTION: None on location — 8707 Millergrove Drive, Santa Fe Springs, CA 90670 confirmed. The listing gives no capability claim to contradict, but it omits the single most decisive fact about this vendor: their published minimum…  |  KEEP at B, but flag the 200-gallon minimum batch prominently in the longlist so the buyer opens with it. Strong QA/regulatory posture (drug manufacturing license, FDA/NSF blending ce…</t>
         </is>
       </c>
       <c r="J27" s="21" t="inlineStr">
@@ -2486,42 +2530,42 @@
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>Custom Chemical Formulators, Inc. (CCFI)</t>
+          <t>Hanson Chemicals (Friendship, NY)</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>Santa Fe Springs, CA</t>
+          <t>Friendship, NY</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>https://www.customchem.com</t>
+          <t>https://hansonchemicals.com</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>PARTIAL, EXPLICIT BUT THIN. Contract manufacturing page lists "In-process heating" as a liquid-production capability, alongside "high shear mixing and variable speed agitation for high viscosity products." So heating exists. NO jacketing detail, NO maximum te…</t>
+          <t>WEAK AND AMBIGUOUS. Toll page states "Temperature-controlled blending and agitation for process stability" and "Stainless steel mixing tanks up to 5,000 gallons." Temperature CONTROL is claimed; heating to a specific setpoint is NOT. "Temperature-controlled" …</t>
         </is>
       </c>
       <c r="F28" s="19" t="inlineStr">
         <is>
-          <t>HARD PUBLISHED FLOOR, AND IT IS A PROBLEM: "200 gallon to 6,000 gallon batch size" for liquids (powders: "1,500-6,000 lb. batch size"). They state over 50 tank…</t>
+          <t>"small pilot batches to large-scale production runs" — no number, no MOQ, no minimum vessel size published. Packaging: "Drum, tote, and bulk packaging options"…</t>
         </is>
       </c>
       <c r="G28" s="19" t="inlineStr">
         <is>
-          <t>BEST REGULATORY SIGNALS IN THE BATCH: "CCFI is a certified blending facility for FDA, EPA, NSF, Kosher, OMRI, USDA." Also holds a US Drug M…</t>
+          <t>Only a vague claim: "ISO-certified quality and safety assurance" — THE STANDARD IS NEVER NAMED. Do not record this as ISO 9001 without a ce…</t>
         </is>
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>https://www.customchem.com/contact/ | (562) 699-5070 | toll-free (877) 344-2436 | sales@customchem.com</t>
+          <t>https://hansonchemicals.com/contact-us/ ("Send a Message" form; no dedicated RFQ form) | 216-306-0506 (US) | 416-457-8271 (Canada) | info@hansonchemicals.com</t>
         </is>
       </c>
       <c r="I28" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: None on location — 8707 Millergrove Drive, Santa Fe Springs, CA 90670 confirmed. The listing gives no capability claim to contradict, but it omits the single most decisive fact about this vendor: their published minimum…  |  KEEP at B, but flag the 200-gallon minimum batch prominently in the longlist so the buyer opens with it. Strong QA/regulatory posture (drug manufacturing license, FDA/NSF blending ce…</t>
+          <t>CORRECTION: The Friendship NY address is correct (4732 Castle Garden Road, Friendship, NY 14739), but the listing omits a material fact: HANSON IS A CANADIAN-HEADQUARTERED CHEMICAL DISTRIBUTOR, not a US manufacturer. Primary operat…  |  KEEP at B, but downgrade expectations and verify identity first. Three unresolved risks: (1) distributor-vs-manufacturer — confirm they own the Friendship NY blending assets rather t…</t>
         </is>
       </c>
       <c r="J28" s="21" t="inlineStr">
@@ -2538,47 +2582,47 @@
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Hanson Chemicals (Friendship, NY)</t>
+          <t>Harcros Chemicals Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Friendship, NY</t>
+          <t>Kansas City, KS (HQ and main plant); ~30 branch/blending locations across the US including the West Coast</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
         <is>
-          <t>https://hansonchemicals.com</t>
+          <t>https://www.harcros.com/services/chemical-toll-manufacturing/</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>WEAK AND AMBIGUOUS. Toll page states "Temperature-controlled blending and agitation for process stability" and "Stainless steel mixing tanks up to 5,000 gallons." Temperature CONTROL is claimed; heating to a specific setpoint is NOT. "Temperature-controlled" …</t>
+          <t>PARTIAL. Reactors are shown and referenced on their toll manufacturing page (they picture an R4/R5/R6 reactor train), but no vessel sizes or temperature ranges are published. A surfactant/alkoxylation house of this type will have steam-jacketed reactors well …</t>
         </is>
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>"small pilot batches to large-scale production runs" — no number, no MOQ, no minimum vessel size published. Packaging: "Drum, tote, and bulk packaging options"…</t>
+          <t>Not published. They do state lab, pilot-plant and commercial scale capability, which implies small-batch is possible. Packaging down to drums and pails is publ…</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Only a vague claim: "ISO-certified quality and safety assurance" — THE STANDARD IS NEVER NAMED. Do not record this as ISO 9001 without a ce…</t>
+          <t>Holds 'various ISO certifications,' NACD Responsible Distribution 7th cycle certified, EcoVadis Silver, SQF certified for food-grade storag…</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>https://hansonchemicals.com/contact-us/ ("Send a Message" form; no dedicated RFQ form) | 216-306-0506 (US) | 416-457-8271 (Canada) | info@hansonchemicals.com</t>
+          <t>Via harcros.com contact form; Kansas City, KS headquarters.</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: The Friendship NY address is correct (4732 Castle Garden Road, Friendship, NY 14739), but the listing omits a material fact: HANSON IS A CANADIAN-HEADQUARTERED CHEMICAL DISTRIBUTOR, not a US manufacturer. Primary operat…  |  KEEP at B, but downgrade expectations and verify identity first. Three unresolved risks: (1) distributor-vs-manufacturer — confirm they own the Friendship NY blending assets rather t…</t>
+          <t>A genuine manufacturer-plus-distributor hybrid that runs its own reaction and blending plants - which is the honest answer to your 'do distributors actually blend' question. They publish custom synthesis, custom blending and scale-up from lab through pilot to commercial, with reactors on site. Kansas City anchors the Midwest and their branch network extends West, so they could potentially serve a second geography if…</t>
         </is>
       </c>
       <c r="J29" s="21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>High on realness and to…</t>
         </is>
       </c>
     </row>
@@ -2590,47 +2634,47 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Harcros Chemicals Inc.  [NEW]</t>
+          <t>Hubbard-Hall (Waterbury, CT + Inman, SC)</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Kansas City, KS (HQ and main plant); ~30 branch/blending locations across the US including the West Coast</t>
+          <t>Waterbury CT + Inman SC</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
         <is>
-          <t>https://www.harcros.com/services/chemical-toll-manufacturing/</t>
+          <t>https://www.hubbardhall.com</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>PARTIAL. Reactors are shown and referenced on their toll manufacturing page (they picture an R4/R5/R6 reactor train), but no vessel sizes or temperature ranges are published. A surfactant/alkoxylation house of this type will have steam-jacketed reactors well …</t>
+          <t>SILENT. No published statement about heated, jacketed, or steam vessels, and no temperature specification found anywhere on the site or in third-party profiles. Their capability list is generic: blending, packaging, formulation, lab analysis, process auditing…</t>
         </is>
       </c>
       <c r="F30" s="19" t="inlineStr">
         <is>
-          <t>Not published. They do state lab, pilot-plant and commercial scale capability, which implies small-batch is possible. Packaging down to drums and pails is publ…</t>
+          <t>SILENT. No batch size range, no minimum, no MOQ published anywhere.</t>
         </is>
       </c>
       <c r="G30" s="19" t="inlineStr">
         <is>
-          <t>Holds 'various ISO certifications,' NACD Responsible Distribution 7th cycle certified, EcoVadis Silver, SQF certified for food-grade storag…</t>
+          <t>ISO 9001:2015 certified. Three in-house laboratories with analytical services. NO ISO 13485, NO FDA registration, NO cGMP. Their core marke…</t>
         </is>
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>Via harcros.com contact form; Kansas City, KS headquarters.</t>
+          <t>https://www.hubbardhall.com/contact/locations | HQ 203-756-5521 | Inman SC plant 864-472-9031 | info@hubbardhall.com</t>
         </is>
       </c>
       <c r="I30" s="19" t="inlineStr">
         <is>
-          <t>A genuine manufacturer-plus-distributor hybrid that runs its own reaction and blending plants - which is the honest answer to your 'do distributors actually blend' question. They publish custom synthesis, custom blending and scale-up from lab through pilot to commercial, with reactors on site. Kansas City anchors the Midwest and their branch network extends West, so they could potentially serve a second geography if…</t>
+          <t>CORRECTION: Listing is INCOMPLETE rather than wrong. Hubbard-Hall runs FIVE US facilities, not two: Waterbury CT (HQ, 563 South Leonard Street, Waterbury CT 06708 — note some directories list zip 06725, which is a PO-box zip); Wilm…  |  KEEP at B. Real, long-established, independent, ISO 9001:2015 certified with genuine custom-blending and in-house lab capability — all good. But BOTH gates are silent: no published h…</t>
         </is>
       </c>
       <c r="J30" s="21" t="inlineStr">
         <is>
-          <t>High on realness and to…</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2642,47 +2686,43 @@
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Hubbard-Hall (Waterbury, CT + Inman, SC)</t>
+          <t>Hydrite Chemical</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Waterbury CT + Inman SC</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>https://www.hubbardhall.com</t>
-        </is>
-      </c>
+          <t>Brookfield WI (multi-site)</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr"/>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>SILENT. No published statement about heated, jacketed, or steam vessels, and no temperature specification found anywhere on the site or in third-party profiles. Their capability list is generic: blending, packaging, formulation, lab analysis, process auditing…</t>
+          <t>PASSES on capability. Contract Manufacturing page states 'Hot oil heating to 575° F' (attached to thin film evaporators), plus 'Glass line reactors pressurized to 100 psig; stainless steel to 150 psig.' Note the 575 F figure is tied to specific equipment, not…</t>
         </is>
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>SILENT. No batch size range, no minimum, no MOQ published anywhere.</t>
+          <t>MAJOR CONCERN. Listed equipment: stainless steel reactors '2,700-15,000 Gallons'; glass line reactors '4,000 Gallons'; distillation pots '4,500, 6,500 and 9,50…</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001:2015 certified. Three in-house laboratories with analytical services. NO ISO 13485, NO FDA registration, NO cGMP. Their core marke…</t>
+          <t>ISO 9001:2015 certified. 'FDA and EPA registered facilities' and 'manufacture EPA and FDA regulated products.' No ISO 13485, no cGMP claim …</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>https://www.hubbardhall.com/contact/locations | HQ 203-756-5521 | Inman SC plant 864-472-9031 | info@hubbardhall.com</t>
+          <t>https://www.hydrite.com/Contact.htm — main 262-792-1450, customer service 855-365-7500, marketing@hydrite.com. No RFQ form published; phone/email only.</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: Listing is INCOMPLETE rather than wrong. Hubbard-Hall runs FIVE US facilities, not two: Waterbury CT (HQ, 563 South Leonard Street, Waterbury CT 06708 — note some directories list zip 06725, which is a PO-box zip); Wilm…  |  KEEP at B. Real, long-established, independent, ISO 9001:2015 certified with genuine custom-blending and in-house lab capability — all good. But BOTH gates are silent: no published h…</t>
+          <t>CORRECTION: Location correct (17385 Golf Parkway, Brookfield WI 53045). One capability caveat: the site's marketing copy claims blends 'in a variety of batch sizes from drums to railcars,' but the equipment list on the Contract Man…  |  Keep B. Credible, certified, genuinely high-temp capable, FDA-registered — good on paper for a medical supply chain. But the smallest published vessel is ~50x our batch and 110 MM lb…</t>
         </is>
       </c>
       <c r="J31" s="21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -2694,43 +2734,47 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>Hydrite Chemical</t>
+          <t>Mallard Creek Polymers, LLC  [NEW]</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Brookfield WI (multi-site)</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="inlineStr"/>
+          <t>8901 Research Drive, Charlotte, NC 28262</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>https://www.mcpolymers.com/</t>
+        </is>
+      </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>PASSES on capability. Contract Manufacturing page states 'Hot oil heating to 575° F' (attached to thin film evaporators), plus 'Glass line reactors pressurized to 100 psig; stainless steel to 150 psig.' Note the 575 F figure is tied to specific equipment, not…</t>
+          <t>STRONG BY INFERENCE, unverified in writing. Emulsion polymerization reactors are jacketed for steam heating and chilled-water cooling with tight temperature control; 90-95 C hold then cool to &lt;=40 C is a normal duty cycle for this equipment. Get it confirmed …</t>
         </is>
       </c>
       <c r="F32" s="19" t="inlineStr">
         <is>
-          <t>MAJOR CONCERN. Listed equipment: stainless steel reactors '2,700-15,000 Gallons'; glass line reactors '4,000 Gallons'; distillation pots '4,500, 6,500 and 9,50…</t>
+          <t>CLAIMED — 'from small custom batches to large-scale orders.' Emulsion reactors are usually 1,000+ gal, so a 50-gal batch is the real risk. Ask for their smalle…</t>
         </is>
       </c>
       <c r="G32" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001:2015 certified. 'FDA and EPA registered facilities' and 'manufacture EPA and FDA regulated products.' No ISO 13485, no cGMP claim …</t>
+          <t>'ISO-certified quality systems' stated on site without the specific standard named. Confirm ISO 9001 registration number and CoA content.</t>
         </is>
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>https://www.hydrite.com/Contact.htm — main 262-792-1450, customer service 855-365-7500, marketing@hydrite.com. No RFQ form published; phone/email only.</t>
+          <t>Sales &amp; Marketing 1-877-240-0171; general +1-704-547-0622</t>
         </is>
       </c>
       <c r="I32" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: Location correct (17385 Golf Parkway, Brookfield WI 53045). One capability caveat: the site's marketing copy claims blends 'in a variety of batch sizes from drums to railcars,' but the equipment list on the Contract Man…  |  Keep B. Credible, certified, genuinely high-temp capable, FDA-registered — good on paper for a medical supply chain. But the smallest published vessel is ~50x our batch and 110 MM lb…</t>
+          <t>Emulsion polymer plants are an underrated source for this capability: vinyl acetate emulsion polymerization requires DISSOLVING PVOH IN HOT WATER as the protective colloid before the monomer feed, so these plants own the 90-95 C PVOH cook as a routine in-house unit operation even though they do not sell PVA solution as a product. MCP has manufactured water-based emulsion polymers in Charlotte since 1962 (styrene-but…</t>
         </is>
       </c>
       <c r="J32" s="21" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -2742,47 +2786,47 @@
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>Mallard Creek Polymers, LLC  [NEW]</t>
+          <t>Moon Chemical Products  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>8901 Research Drive, Charlotte, NC 28262</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>https://www.mcpolymers.com/</t>
+          <t>https://moonchemical.com/custom-blending</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>STRONG BY INFERENCE, unverified in writing. Emulsion polymerization reactors are jacketed for steam heating and chilled-water cooling with tight temperature control; 90-95 C hold then cool to &lt;=40 C is a normal duty cycle for this equipment. Get it confirmed …</t>
+          <t>SILENT on jackets/steam. Nearest signals: 'processing both endothermic and exothermic reactions' and 'ability to hydrate polymers using high-speed sheer blades'.</t>
         </is>
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>CLAIMED — 'from small custom batches to large-scale orders.' Emulsion reactors are usually 1,000+ gal, so a 50-gal batch is the real risk. Ask for their smalle…</t>
+          <t>'from 5 gallons up to 12,000 gallons' — a genuine 5-gal floor</t>
         </is>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>'ISO-certified quality systems' stated on site without the specific standard named. Confirm ISO 9001 registration number and CoA content.</t>
+          <t>No ISO. Retained samples kept 6 months minimum; lot number recorded on package, batch record, BOL and invoice</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing 1-877-240-0171; general +1-704-547-0622</t>
+          <t>moonchemical.com/contact | 405-787-4110</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Emulsion polymer plants are an underrated source for this capability: vinyl acetate emulsion polymerization requires DISSOLVING PVOH IN HOT WATER as the protective colloid before the monomer feed, so these plants own the 90-95 C PVOH cook as a routine in-house unit operation even though they do not sell PVA solution as a product. MCP has manufactured water-based emulsion polymers in Charlotte since 1962 (styrene-but…</t>
+          <t>BEST PRICE-CULTURE MATCH FOUND: a 60-year-old independent that genuinely runs 5-55 gallon liquid batches and already talks about polymer hydration. Most likely of any candidate to quote near the incumbent rather than at a big-house rate.</t>
         </is>
       </c>
       <c r="J33" s="21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2794,47 +2838,47 @@
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>Moon Chemical Products  [NATIONWIDE]</t>
+          <t>Nova Specialty Chemicals LLC  [NEW]</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Vermont (802 area code; exact city not published on their site)</t>
         </is>
       </c>
       <c r="D34" s="20" t="inlineStr">
         <is>
-          <t>https://moonchemical.com/custom-blending</t>
+          <t>https://novaspecialties.com/toll-manufacturing/</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>SILENT on jackets/steam. Nearest signals: 'processing both endothermic and exothermic reactions' and 'ability to hydrate polymers using high-speed sheer blades'.</t>
+          <t>STRONGEST published temperature spec of any candidate: '-15 C to 400 C' on jacketed glass-lined and stainless reactors. 90-95 C hold is trivially within range.</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>'from 5 gallons up to 12,000 gallons' — a genuine 5-gal floor</t>
+          <t>WEAK - this is the real problem. Smallest published reactor is 500 gallons, roughly 10 drums. With an 18-day shelf life and 1 drum/week you cannot consume a 50…</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
         <is>
-          <t>No ISO. Retained samples kept 6 months minimum; lot number recorded on package, batch record, BOL and invoice</t>
+          <t>None published. Operates under an NPDES permit with VOC/acid emission containment. Ask directly about ISO 9001 and CoA content.</t>
         </is>
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>moonchemical.com/contact | 405-787-4110</t>
+          <t>802-448-2117 / info@novaspecialties.com</t>
         </is>
       </c>
       <c r="I34" s="19" t="inlineStr">
         <is>
-          <t>BEST PRICE-CULTURE MATCH FOUND: a 60-year-old independent that genuinely runs 5-55 gallon liquid batches and already talks about polymer hydration. Most likely of any candidate to quote near the incumbent rather than at a big-house rate.</t>
+          <t>Unambiguously clears the heat gate, which almost no one else publishes plainly. Their toll manufacturing page states glass-lined and stainless steel JACKETED reactors from 500 to 4,000 gallons with temperature control from -15 C to 400 C. They also explicitly list 'custom liquid blending and formulation' and 'drum filling and repackaging' as services. They manufacture concentrated liquid dyes including a water-based…</t>
         </is>
       </c>
       <c r="J34" s="21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>High on heat capability…</t>
         </is>
       </c>
     </row>
@@ -2846,47 +2890,47 @@
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>Nova Specialty Chemicals LLC  [NEW]</t>
+          <t>PhilChem (Mount Vernon Chemicals)</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Vermont (802 area code; exact city not published on their site)</t>
+          <t>Greer, SC (parent: Mount Vernon Chemicals)</t>
         </is>
       </c>
       <c r="D35" s="20" t="inlineStr">
         <is>
-          <t>https://novaspecialties.com/toll-manufacturing/</t>
+          <t>https://philchem.us</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>STRONGEST published temperature spec of any candidate: '-15 C to 400 C' on jacketed glass-lined and stainless reactors. 90-95 C hold is trivially within range.</t>
+          <t>philchem.us itself: SILENT - no mention of jacketed vessels, heating, or temperature anywhere. Parent mvchemicals.com states: 'The plants are equipped with stainless steel blending vessels with capacities ranging from 3 drum quantities to 100 drum quantities.…</t>
         </is>
       </c>
       <c r="F35" s="19" t="inlineStr">
         <is>
-          <t>WEAK - this is the real problem. Smallest published reactor is 500 gallons, roughly 10 drums. With an 18-day shelf life and 1 drum/week you cannot consume a 50…</t>
+          <t>philchem.us: SILENT. Parent mvchemicals.com: vessels 'ranging from 3 drum quantities to 100 drum quantities' - a 3-drum minimum vessel would fit a ~1-drum batc…</t>
         </is>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>None published. Operates under an NPDES permit with VOC/acid emission containment. Ask directly about ISO 9001 and CoA content.</t>
+          <t>ISO 9001:2015 certified (certificate posted on philchem.us). No ISO 13485, no FDA registration, no cGMP, no lot traceability language found.</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>802-448-2117 / info@novaspecialties.com</t>
+          <t>https://philchem.us/contact-philchem (working inquiry form with Product Interest field) | Phone (864) 848-9811 | Fax (864) 848-9822</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Unambiguously clears the heat gate, which almost no one else publishes plainly. Their toll manufacturing page states glass-lined and stainless steel JACKETED reactors from 500 to 4,000 gallons with temperature control from -15 C to 400 C. They also explicitly list 'custom liquid blending and formulation' and 'drum filling and repackaging' as services. They manufacture concentrated liquid dyes including a water-based…</t>
+          <t>CORRECTION: MATERIAL ERROR: PhilChem Greer SC is a DRY blending / repackaging operation, not a liquid blender. Its own site says 'specialty formulated dry blends to the Textile, Adhesive, and Paper Markets' and the company page lis…  |  MOVE A -&gt; B, and re-target the contact. As listed, this is a mis-target: you would be asking a dry-blend/repack house to run a heated aqueous solution. The heated jacketed capability…</t>
         </is>
       </c>
       <c r="J35" s="21" t="inlineStr">
         <is>
-          <t>High on heat capability…</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2898,47 +2942,43 @@
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>PhilChem (Mount Vernon Chemicals)</t>
+          <t>Sandstrom Coating Technologies</t>
         </is>
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Greer, SC (parent: Mount Vernon Chemicals)</t>
-        </is>
-      </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>https://philchem.us</t>
-        </is>
-      </c>
+          <t>Port Byron, IL</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr"/>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>philchem.us itself: SILENT - no mention of jacketed vessels, heating, or temperature anywhere. Parent mvchemicals.com states: 'The plants are equipped with stainless steel blending vessels with capacities ranging from 3 drum quantities to 100 drum quantities.…</t>
+          <t>SILENT. Nothing on the homepage, toll production page, or in search results mentions heated or jacketed vessels, temperature capability, or hot processing. Their published equipment is described as 'multi-speed mixers, various mills, as well as customized tan…</t>
         </is>
       </c>
       <c r="F36" s="19" t="inlineStr">
         <is>
-          <t>philchem.us: SILENT. Parent mvchemicals.com: vessels 'ranging from 3 drum quantities to 100 drum quantities' - a 3-drum minimum vessel would fit a ~1-drum batc…</t>
+          <t>EXCELLENT. Toll production page states 'tanks with capacities from 1-5,000 gallons' — a 1-gallon low end, the smallest floor of any candidate audited. Facility…</t>
         </is>
       </c>
       <c r="G36" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001:2015 certified (certificate posted on philchem.us). No ISO 13485, no FDA registration, no cGMP, no lot traceability language found.</t>
+          <t>STRONGEST QUALITY SYSTEM IN THE GROUP. ISO 9001:2015 AND AS9100 Rev. D (aerospace/defense standard), with the certificate published at http…</t>
         </is>
       </c>
       <c r="H36" s="19" t="inlineStr">
         <is>
-          <t>https://philchem.us/contact-philchem (working inquiry form with Product Interest field) | Phone (864) 848-9811 | Fax (864) 848-9822</t>
+          <t>https://sandstromproducts.com/ (contact page linked site-wide; /services/toll-production/ describes the model) — toll-free 1-800-747-1084, direct 309-523-2121</t>
         </is>
       </c>
       <c r="I36" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: MATERIAL ERROR: PhilChem Greer SC is a DRY blending / repackaging operation, not a liquid blender. Its own site says 'specialty formulated dry blends to the Textile, Adhesive, and Paper Markets' and the company page lis…  |  MOVE A -&gt; B, and re-target the contact. As listed, this is a mis-target: you would be asking a dry-blend/repack house to run a heated aqueous solution. The heated jacketed capability…</t>
+          <t>CORRECTION: Location correct (224 S. Main Street, Port Byron IL 61275). Minor naming note: the legal/registry name is 'Sandstrom Products Company' (matching the domain and the D-U-N-S/CAGE listing); 'Sandstrom Coating Technologies'…  |  Keep B, but treat as the strongest B and call early. Their published toll model is an exact description of ours: 'root formulas are provided by... coating companies, with chemical ra…</t>
         </is>
       </c>
       <c r="J36" s="21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -2950,38 +2990,42 @@
       </c>
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>Sandstrom Coating Technologies</t>
+          <t>Seacole (Seacole-CRC / Seacole Specialty Chemical)</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Port Byron, IL</t>
-        </is>
-      </c>
-      <c r="D37" s="19" t="inlineStr"/>
+          <t>CORRECTED: Plymouth, MN</t>
+        </is>
+      </c>
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>https://seacole.com</t>
+        </is>
+      </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>SILENT. Nothing on the homepage, toll production page, or in search results mentions heated or jacketed vessels, temperature capability, or hot processing. Their published equipment is described as 'multi-speed mixers, various mills, as well as customized tan…</t>
+          <t>PARTIAL PASS, EXPLICIT. Seacole's own contract-manufacturing content states liquid custom blending takes place in an indoor tank farm equipped with 20 blending tanks ranging from 150 to 3,000 gallons, and that "jacketed tanks are available when cooling or hea…</t>
         </is>
       </c>
       <c r="F37" s="19" t="inlineStr">
         <is>
-          <t>EXCELLENT. Toll production page states 'tanks with capacities from 1-5,000 gallons' — a 1-gallon low end, the smallest floor of any candidate audited. Facility…</t>
+          <t>SMALLEST LIQUID VESSEL IS 150 GALLONS ("20 blending tanks ranging from 150 to 3,000 gallons"). Our batch is ~53 gallons, so their floor is roughly 3x our batch…</t>
         </is>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>STRONGEST QUALITY SYSTEM IN THE GROUP. ISO 9001:2015 AND AS9100 Rev. D (aerospace/defense standard), with the certificate published at http…</t>
+          <t>ISO 9001:2015 certified. Active NACD member. Quality-control language present ("every production batch meets designated specifications"). N…</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>https://sandstromproducts.com/ (contact page linked site-wide; /services/toll-production/ describes the model) — toll-free 1-800-747-1084, direct 309-523-2121</t>
+          <t>https://seacole.com/contact-us/ | (763) 582-1140 | Sales@seacole.com</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: Location correct (224 S. Main Street, Port Byron IL 61275). Minor naming note: the legal/registry name is 'Sandstrom Products Company' (matching the domain and the D-U-N-S/CAGE listing); 'Sandstrom Coating Technologies'…  |  Keep B, but treat as the strongest B and call early. Their published toll model is an exact description of ours: 'root formulas are provided by... coating companies, with chemical ra…</t>
+          <t>CORRECTION: FACTUAL ERROR IN THE LONGLIST — LOCATION IS WRONG. Seacole is in PLYMOUTH, MN, not Maple Grove, MN. Confirmed address: 13505 Industrial Park Blvd, Plymouth, MN 55441 (consistent across Seacole's own site, D&amp;B, BBB, Thom…  |  KEEP at B, but correct the location to Plymouth MN before contacting. Jacketed heating is a genuine plus and ISO 9001:2015 is solid, but two things hold it out of A: the 150-gal mini…</t>
         </is>
       </c>
       <c r="J37" s="21" t="inlineStr">
@@ -2998,47 +3042,47 @@
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>Seacole (Seacole-CRC / Seacole Specialty Chemical)</t>
+          <t>Seal Bond  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>CORRECTED: Plymouth, MN</t>
+          <t>Norton Shores, MI</t>
         </is>
       </c>
       <c r="D38" s="20" t="inlineStr">
         <is>
-          <t>https://seacole.com</t>
+          <t>https://seal-bond.com/toll-private-label-manufacturing</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>PARTIAL PASS, EXPLICIT. Seacole's own contract-manufacturing content states liquid custom blending takes place in an indoor tank farm equipped with 20 blending tanks ranging from 150 to 3,000 gallons, and that "jacketed tanks are available when cooling or hea…</t>
+          <t>SILENT — nothing on jackets, steam, or temperature. This is the one question to ask.</t>
         </is>
       </c>
       <c r="F38" s="19" t="inlineStr">
         <is>
-          <t>SMALLEST LIQUID VESSEL IS 150 GALLONS ("20 blending tanks ranging from 150 to 3,000 gallons"). Our batch is ~53 gallons, so their floor is roughly 3x our batch…</t>
+          <t>BEST PUBLISHED SMALL BATCH IN THE MIDWEST: 'Scale-up capabilities from 500 g to 500 gal' — our 50-gal batch is comfortably inside</t>
         </is>
       </c>
       <c r="G38" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001:2015 certified. Active NACD member. Quality-control language present ("every production batch meets designated specifications"). N…</t>
+          <t>ISO 9001 certified</t>
         </is>
       </c>
       <c r="H38" s="19" t="inlineStr">
         <is>
-          <t>https://seacole.com/contact-us/ | (763) 582-1140 | Sales@seacole.com</t>
+          <t>seal-bond.com/contact-us | 616-850-0507 | dketelhut@seal-bond.com</t>
         </is>
       </c>
       <c r="I38" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: FACTUAL ERROR IN THE LONGLIST — LOCATION IS WRONG. Seacole is in PLYMOUTH, MN, not Maple Grove, MN. Confirmed address: 13505 Industrial Park Blvd, Plymouth, MN 55441 (consistent across Seacole's own site, D&amp;B, BBB, Thom…  |  KEEP at B, but correct the location to Plymouth MN before contacting. Jacketed heating is a genuine plus and ISO 9001:2015 is solid, but two things hold it out of A: the 150-gal mini…</t>
+          <t>Passes the small-batch gate outright and in writing — the gate that killed most candidates. Toll model stated as 'outsource adhesive or sealant production while retaining ownership of proprietary formulas'. One phone question decides it.</t>
         </is>
       </c>
       <c r="J38" s="21" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -3050,47 +3094,47 @@
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>Seal Bond  [NATIONWIDE]</t>
+          <t>Shamrock Technologies, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Norton Shores, MI</t>
+          <t>Newark, NJ (HQ and main plant); also Henderson, KY and Fountain Inn, SC</t>
         </is>
       </c>
       <c r="D39" s="20" t="inlineStr">
         <is>
-          <t>https://seal-bond.com/toll-private-label-manufacturing</t>
+          <t>https://shamrocktechnologies.com/capabilities/contract-manufacturing/</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>SILENT — nothing on jackets, steam, or temperature. This is the one question to ask.</t>
+          <t>STRONG. Published: '500-gallon and 1,200-gallon jacketed kettles with oil heating' and jacketed 50/350-gallon mixers. Oil-heated jackets are well above 95 C capability; they also run tray ovens to 600 F. Confirm the specific vessel they would assign and its c…</t>
         </is>
       </c>
       <c r="F39" s="19" t="inlineStr">
         <is>
-          <t>BEST PUBLISHED SMALL BATCH IN THE MIDWEST: 'Scale-up capabilities from 500 g to 500 gal' — our 50-gal batch is comfortably inside</t>
+          <t>GOOD. 50-gallon jacketed high-shear mixer is essentially one drum. They state batch capability from 0.1 lb to 500,000 lb depending on process.</t>
         </is>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001 certified</t>
+          <t>ISO 9001:2015 certified facilities, plus a Class 100,000 cGMP clean room - unusually strong for a toll blender and relevant to a medical-de…</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>seal-bond.com/contact-us | 616-850-0507 | dketelhut@seal-bond.com</t>
+          <t>Frank Contangelo, (973) 242-2999 ext. 1051</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Passes the small-batch gate outright and in writing — the gate that killed most candidates. Toll model stated as 'outsource adhesive or sealant production while retaining ownership of proprietary formulas'. One phone question decides it.</t>
+          <t>Best NORTHEAST fit and a toll-blender CATEGORY not on the current list: a micronized-wax / dispersion-and-emulsion house. Their contract manufacturing page publishes 500-gallon and 1,200-gallon JACKETED kettles with OIL HEATING, plus 50-gallon and 350-gallon jacketed, vacuum, high-shear, side-scraping mixers. Wax emulsification is a heat-to-90-95-C-and-hold process, so the duty cycle is directly analogous to dissolv…</t>
         </is>
       </c>
       <c r="J39" s="21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>High - real, working UR…</t>
         </is>
       </c>
     </row>
@@ -3102,47 +3146,43 @@
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>Shamrock Technologies, Inc.  [NEW]</t>
+          <t>Sierra Performance Coatings</t>
         </is>
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Newark, NJ (HQ and main plant); also Henderson, KY and Fountain Inn, SC</t>
-        </is>
-      </c>
-      <c r="D40" s="20" t="inlineStr">
-        <is>
-          <t>https://shamrocktechnologies.com/capabilities/contract-manufacturing/</t>
-        </is>
-      </c>
+          <t>Minnetonka, MN</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr"/>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>STRONG. Published: '500-gallon and 1,200-gallon jacketed kettles with oil heating' and jacketed 50/350-gallon mixers. Oil-heated jackets are well above 95 C capability; they also run tray ovens to 600 F. Confirm the specific vessel they would assign and its c…</t>
+          <t>SILENT. No mention of heated or jacketed vessels, temperature capability, or hot processing on the homepage, About page, or toll blending page. Described as an 80,000 sq ft manufacturing area 'capable of water and solvent-borne blends and dispersions' — ambie…</t>
         </is>
       </c>
       <c r="F40" s="19" t="inlineStr">
         <is>
-          <t>GOOD. 50-gallon jacketed high-shear mixer is essentially one drum. They state batch capability from 0.1 lb to 500,000 lb depending on process.</t>
+          <t>NO NUMBERS, but posture is favorable. Toll blending page offers 'a single, short run, or consistent truckloads of product' and 'a nearly limitless variety of l…</t>
         </is>
       </c>
       <c r="G40" s="19" t="inlineStr">
         <is>
-          <t>ISO 9001:2015 certified facilities, plus a Class 100,000 cGMP clean room - unusually strong for a toll blender and relevant to a medical-de…</t>
+          <t>AMBIGUOUS — DO NOT CREDIT AS CERTIFIED. The About page lists 'International Organization for Standardization (ISO)', EPA/VOC/HAPS, 'FDA/USD…</t>
         </is>
       </c>
       <c r="H40" s="19" t="inlineStr">
         <is>
-          <t>Frank Contangelo, (973) 242-2999 ext. 1051</t>
+          <t>https://sierrapaint.com/contact-2/ — toll-free 800-441-2129, local 952-938-7223, fax 952-938-8084</t>
         </is>
       </c>
       <c r="I40" s="19" t="inlineStr">
         <is>
-          <t>Best NORTHEAST fit and a toll-blender CATEGORY not on the current list: a micronized-wax / dispersion-and-emulsion house. Their contract manufacturing page publishes 500-gallon and 1,200-gallon JACKETED kettles with OIL HEATING, plus 50-gallon and 350-gallon jacketed, vacuum, high-shear, side-scraping mixers. Wax emulsification is a heat-to-90-95-C-and-hold process, so the duty cycle is directly analogous to dissolv…</t>
+          <t>CORRECTION: Location correct (11400 W. 47th Street, Minnetonka MN 55343). One caution on the listing if it credited certifications: see the medical/quality field — the ISO and FDA references on their About page appear to be standar…  |  Keep B. Genuinely toll-oriented — 'You provide the formula or the specifications, and we blend and package your finished product,' and on customer-supplied raw materials, 'We can or …</t>
         </is>
       </c>
       <c r="J40" s="21" t="inlineStr">
         <is>
-          <t>High - real, working UR…</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -3154,38 +3194,42 @@
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>Sierra Performance Coatings</t>
+          <t>Specialty Adhesives &amp; Coatings  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Minnetonka, MN</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="inlineStr"/>
+          <t>Memphis, TN (+ a Texas plant)</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="inlineStr">
+        <is>
+          <t>https://specialtyadhesivesinc.com/our_products/water-based-product/</t>
+        </is>
+      </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>SILENT. No mention of heated or jacketed vessels, temperature capability, or hot processing on the homepage, About page, or toll blending page. Described as an 80,000 sq ft manufacturing area 'capable of water and solvent-borne blends and dispersions' — ambie…</t>
+          <t>Not stated, but STRONGLY IMPLIED: they manufacture starch/dextrin adhesives, which are a 85-95 C cook. You cannot run that product line without hold-temperature kettles. Verify — this is inference, not a quote.</t>
         </is>
       </c>
       <c r="F41" s="19" t="inlineStr">
         <is>
-          <t>NO NUMBERS, but posture is favorable. Toll blending page offers 'a single, short run, or consistent truckloads of product' and 'a nearly limitless variety of l…</t>
+          <t>SILENT. Packages '5 gal pails, 55 gallon drums (metal or fiber), tote bins and bulk'</t>
         </is>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>AMBIGUOUS — DO NOT CREDIT AS CERTIFIED. The About page lists 'International Organization for Standardization (ISO)', EPA/VOC/HAPS, 'FDA/USD…</t>
+          <t>No ISO stated; documented quality program covering raw materials through logistics</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>https://sierrapaint.com/contact-2/ — toll-free 800-441-2129, local 952-938-7223, fax 952-938-8084</t>
+          <t>specialtyadhesivesinc.com/contact | 1-800-728-9171</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>CORRECTION: Location correct (11400 W. 47th Street, Minnetonka MN 55343). One caution on the listing if it credited certifications: see the medical/quality field — the ISO and FDA references on their About page appear to be standar…  |  Keep B. Genuinely toll-oriented — 'You provide the formula or the specifications, and we blend and package your finished product,' and on customer-supplied raw materials, 'We can or …</t>
+          <t>ALREADY MAKES PVOH PRODUCTS — their water-based line is explicitly 'PVOH and starch/dextrin based'. Closest chemistry culture found in the region, and custom formulation turnaround is 'a matter of days'. Consider them as a possible SUPPLIER of the finished solution, not only as a toller.</t>
         </is>
       </c>
       <c r="J41" s="21" t="inlineStr">
@@ -3202,47 +3246,47 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>Specialty Adhesives &amp; Coatings  [NATIONWIDE]</t>
+          <t>Sunland Chemical &amp; Research Corp.  [NEW]</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Memphis, TN (+ a Texas plant)</t>
+          <t>5447 San Fernando Road West, Los Angeles, CA 90039</t>
         </is>
       </c>
       <c r="D42" s="20" t="inlineStr">
         <is>
-          <t>https://specialtyadhesivesinc.com/our_products/water-based-product/</t>
+          <t>https://sunlandchemical.com/our-process/blending/</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>Not stated, but STRONGLY IMPLIED: they manufacture starch/dextrin adhesives, which are a 85-95 C cook. You cannot run that product line without hold-temperature kettles. Verify — this is inference, not a quote.</t>
+          <t>GOOD. Their own pages say jacketed tanks heat or cool liquids while blending, and that they manage 'thermal reactions, heating, and cooling.' Maximum temperature is NOT published - the 90-95 C hold must be confirmed directly. Do not assume.</t>
         </is>
       </c>
       <c r="F42" s="19" t="inlineStr">
         <is>
-          <t>SILENT. Packages '5 gal pails, 55 gallon drums (metal or fiber), tote bins and bulk'</t>
+          <t>STRONG. Tanks from 5 gallons up; jacketed heating available from 50 gallons up. That is the closest published match to a ~52-gallon single-drum batch of anyone…</t>
         </is>
       </c>
       <c r="G42" s="19" t="inlineStr">
         <is>
-          <t>No ISO stated; documented quality program covering raw materials through logistics</t>
+          <t>In-house lab with HPLC, GC, pH and flash point. Personnel DOT/HazMat certified. No ISO 9001 published - treat as a gap given the Intuitive …</t>
         </is>
       </c>
       <c r="H42" s="19" t="inlineStr">
         <is>
-          <t>specialtyadhesivesinc.com/contact | 1-800-728-9171</t>
+          <t>(818) 244-9600 / info@sunlandchemical.com</t>
         </is>
       </c>
       <c r="I42" s="19" t="inlineStr">
         <is>
-          <t>ALREADY MAKES PVOH PRODUCTS — their water-based line is explicitly 'PVOH and starch/dextrin based'. Closest chemistry culture found in the region, and custom formulation turnaround is 'a matter of days'. Consider them as a possible SUPPLIER of the finished solution, not only as a toller.</t>
+          <t>The single best WEST-coast fit found. They publish 18 blending tanks ranging from 5 gallons to 6,000 gallons, and state that 'many of the blending tanks have jackets that allow liquids from 50 gallons to 6000 gallons to be heated or cooled while blending.' A 50-gallon jacketed tank is essentially a one-drum batch - which matches the 1 drum/week, make-fresh-to-order cadence better than anything else on this list. Fam…</t>
         </is>
       </c>
       <c r="J42" s="21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>High on realness and ja…</t>
         </is>
       </c>
     </row>
@@ -3254,99 +3298,99 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>Sunland Chemical &amp; Research Corp.  [NEW]</t>
+          <t>Tiarco / TRCC (Tiarco Chemical)</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>5447 San Fernando Road West, Los Angeles, CA 90039</t>
+          <t>Dalton, GA</t>
         </is>
       </c>
       <c r="D43" s="20" t="inlineStr">
         <is>
-          <t>https://sunlandchemical.com/our-process/blending/</t>
+          <t>https://trcc.com</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>GOOD. Their own pages say jacketed tanks heat or cool liquids while blending, and that they manage 'thermal reactions, heating, and cooling.' Maximum temperature is NOT published - the 90-95 C hold must be confirmed directly. Do not assume.</t>
+          <t>SILENT. No mention of jacketed vessels, reactors, heating, or any temperature anywhere on the pages reviewed. The site lists 'Custom Toll &amp; Contract Manufacturing' as a service but publishes no equipment specifications.</t>
         </is>
       </c>
       <c r="F43" s="19" t="inlineStr">
         <is>
-          <t>STRONG. Tanks from 5 gallons up; jacketed heating available from 50 gallons up. That is the closest published match to a ~52-gallon single-drum batch of anyone…</t>
+          <t>SILENT. No minimum batch size or MOQ published.</t>
         </is>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>In-house lab with HPLC, GC, pH and flash point. Personnel DOT/HazMat certified. No ISO 9001 published - treat as a gap given the Intuitive …</t>
+          <t>None found. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no lot traceability language on the pages reviewed.</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>(818) 244-9600 / info@sunlandchemical.com</t>
+          <t>https://trcc.com/contact/ (general Contact Us form - name, email, company, comments) | Phone (706) 277-1300 | Toll free (888) 706-1300 | Fax (706) 277-1111</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>The single best WEST-coast fit found. They publish 18 blending tanks ranging from 5 gallons to 6,000 gallons, and state that 'many of the blending tanks have jackets that allow liquids from 50 gallons to 6000 gallons to be heated or cooled while blending.' A 50-gallon jacketed tank is essentially a one-drum batch - which matches the 1 drum/week, make-fresh-to-order cadence better than anything else on this list. Fam…</t>
+          <t>CORRECTION: Minor naming issue: the parent entity is Textile Rubber and Chemical Company (TRCC); Tiarco Chemical is its specialty-chemical arm, not the parent. TRCC realigned six North American groups under the TRCC brand in 2023, …  |  MOVE A -&gt; B. Real, long-established toll manufacturer in the right geography, but the website publishes literally zero equipment, temperature, batch-size, or quality-certification da…</t>
         </is>
       </c>
       <c r="J43" s="21" t="inlineStr">
         <is>
-          <t>High on realness and ja…</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B44" s="19" t="inlineStr">
-        <is>
-          <t>Tiarco / TRCC (Tiarco Chemical)</t>
-        </is>
-      </c>
-      <c r="C44" s="19" t="inlineStr">
-        <is>
-          <t>Dalton, GA</t>
-        </is>
-      </c>
-      <c r="D44" s="20" t="inlineStr">
-        <is>
-          <t>https://trcc.com</t>
-        </is>
-      </c>
-      <c r="E44" s="19" t="inlineStr">
-        <is>
-          <t>SILENT. No mention of jacketed vessels, reactors, heating, or any temperature anywhere on the pages reviewed. The site lists 'Custom Toll &amp; Contract Manufacturing' as a service but publishes no equipment specifications.</t>
-        </is>
-      </c>
-      <c r="F44" s="19" t="inlineStr">
-        <is>
-          <t>SILENT. No minimum batch size or MOQ published.</t>
-        </is>
-      </c>
-      <c r="G44" s="19" t="inlineStr">
-        <is>
-          <t>None found. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no lot traceability language on the pages reviewed.</t>
-        </is>
-      </c>
-      <c r="H44" s="19" t="inlineStr">
-        <is>
-          <t>https://trcc.com/contact/ (general Contact Us form - name, email, company, comments) | Phone (706) 277-1300 | Toll free (888) 706-1300 | Fax (706) 277-1111</t>
-        </is>
-      </c>
-      <c r="I44" s="19" t="inlineStr">
-        <is>
-          <t>CORRECTION: Minor naming issue: the parent entity is Textile Rubber and Chemical Company (TRCC); Tiarco Chemical is its specialty-chemical arm, not the parent. TRCC realigned six North American groups under the TRCC brand in 2023, …  |  MOVE A -&gt; B. Real, long-established toll manufacturer in the right geography, but the website publishes literally zero equipment, temperature, batch-size, or quality-certification da…</t>
-        </is>
-      </c>
-      <c r="J44" s="21" t="inlineStr">
-        <is>
-          <t>M</t>
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B44" s="23" t="inlineStr">
+        <is>
+          <t>Allied International  [NATIONWIDE]</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>Buena Park, CA</t>
+        </is>
+      </c>
+      <c r="D44" s="24" t="inlineStr">
+        <is>
+          <t>https://alliedin.com/</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="inlineStr">
+        <is>
+          <t>SILENT (checked services, about and FAQ pages)</t>
+        </is>
+      </c>
+      <c r="F44" s="23" t="inlineStr">
+        <is>
+          <t>SILENT</t>
+        </is>
+      </c>
+      <c r="G44" s="23" t="inlineStr">
+        <is>
+          <t>EPA facility number only; no ISO 9001 claimed anywhere</t>
+        </is>
+      </c>
+      <c r="H44" s="23" t="inlineStr">
+        <is>
+          <t>alliedin.com/contact (quote within 24 hrs) | 714-736-9811</t>
+        </is>
+      </c>
+      <c r="I44" s="23" t="inlineStr">
+        <is>
+          <t>Small independent since 1972 — the kind of shop that quotes a low conversion fee rather than a big-house rate. But the site discloses nothing about either gate, and no ISO.</t>
+        </is>
+      </c>
+      <c r="J44" s="25" t="inlineStr">
+        <is>
+          <t>L-M</t>
         </is>
       </c>
     </row>
@@ -3358,47 +3402,47 @@
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>Allied International  [NATIONWIDE]</t>
+          <t>Alpha Teknova, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Buena Park, CA</t>
+          <t>Hollister, CA (180,000 sq ft ISO 13485-certified manufacturing)</t>
         </is>
       </c>
       <c r="D45" s="24" t="inlineStr">
         <is>
-          <t>https://alliedin.com/</t>
+          <t>https://www.teknova.com/en/services/custom-manufacturing.html</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>SILENT (checked services, about and FAQ pages)</t>
+          <t>SILENT and a real concern. The only temperature reference on the custom manufacturing page is 'monitored temperature-controlled service' for SHIPPING, not processing. No jacketed vessel or process temperature capability is published. Buffer/reagent formulatio…</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>Strong. GMP batches from 25 L; RUO from 8 L; explicitly 'no minimum order quantities' on their Build-Tek custom platform. Fast turnaround is a marketed differe…</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>EPA facility number only; no ISO 9001 claimed anywhere</t>
+          <t>ISO 13485:2016 certified manufacturing (180,000 sq ft); cGMP-compliant GMP grade tier; USP-based QC assays on raw materials and finished pr…</t>
         </is>
       </c>
       <c r="H45" s="23" t="inlineStr">
         <is>
-          <t>alliedin.com/contact (quote within 24 hrs) | 714-736-9811</t>
+          <t>1.800.209.4488, Mon-Fri 8 AM-5 PM PT; request Custom Manufacturing</t>
         </is>
       </c>
       <c r="I45" s="23" t="inlineStr">
         <is>
-          <t>Small independent since 1972 — the kind of shop that quotes a low conversion fee rather than a big-house rate. But the site discloses nothing about either gate, and no ISO.</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | A dedicated custom AQUEOUS SOLUTION manufacturer operating entirely inside an ISO 13485-certified footprint, with ~30 years of formulating to customer specification. They state they tailor 'everything from formulation to container format t…</t>
         </is>
       </c>
       <c r="J45" s="25" t="inlineStr">
         <is>
-          <t>L-M</t>
+          <t>HIGH on the ISO 13485 c…</t>
         </is>
       </c>
     </row>
@@ -3410,47 +3454,47 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>Alpha Teknova, Inc.  [NEW]</t>
+          <t>Aqua Based Technologies, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>Hollister, CA (180,000 sq ft ISO 13485-certified manufacturing)</t>
+          <t>224 Pegasus Avenue, Northvale, NJ 07647</t>
         </is>
       </c>
       <c r="D46" s="24" t="inlineStr">
         <is>
-          <t>https://www.teknova.com/en/services/custom-manufacturing.html</t>
+          <t>https://www.aquabased.com/customformulations/</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>SILENT and a real concern. The only temperature reference on the custom manufacturing page is 'monitored temperature-controlled service' for SHIPPING, not processing. No jacketed vessel or process temperature capability is published. Buffer/reagent formulatio…</t>
+          <t>NOT PUBLISHED — no heating capability stated anywhere on the site. This is the first question to ask; if they only have ambient/low-heat mix tanks they are disqualified like ILC Dover.</t>
         </is>
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>Strong. GMP batches from 25 L; RUO from 8 L; explicitly 'no minimum order quantities' on their Build-Tek custom platform. Fast turnaround is a marketed differe…</t>
+          <t>GOOD — 'from initial laboratory small testing quantities to multiple drum and tote quantities.' Drum-scale is explicitly in their stated range, so a single 450…</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified manufacturing (180,000 sq ft); cGMP-compliant GMP grade tier; USP-based QC assays on raw materials and finished pr…</t>
+          <t>Not published. Ask about ISO 9001, lot traceability, retained samples, and CoA fields.</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
         <is>
-          <t>1.800.209.4488, Mon-Fri 8 AM-5 PM PT; request Custom Manufacturing</t>
+          <t>201.767.6040 / info@aquabased.com</t>
         </is>
       </c>
       <c r="I46" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | A dedicated custom AQUEOUS SOLUTION manufacturer operating entirely inside an ISO 13485-certified footprint, with ~30 years of formulating to customer specification. They state they tailor 'everything from formulation to container format t…</t>
+          <t>A dedicated WATER-BASED-only house — coatings, adhesives and primers — offering exactly the three services we need bundled: custom formulating, toll manufacturing, and private label. They explicitly scale 'from initial laboratory small testing quantities to multiple drum and tote quantities' and emphasize batch-to-batch consistency, which is the correct posture for a made-fresh-to-order weekly drum with an 18-day sh…</t>
         </is>
       </c>
       <c r="J46" s="25" t="inlineStr">
         <is>
-          <t>HIGH on the ISO 13485 c…</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3462,47 +3506,47 @@
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>Aqua Based Technologies, Inc.  [NEW]</t>
+          <t>Biocoat Incorporated  [NEW]</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>224 Pegasus Avenue, Northvale, NJ 07647</t>
+          <t>Horsham, PA (two facilities, 46,000 sq ft, six ISO 7 cleanrooms)</t>
         </is>
       </c>
       <c r="D47" s="24" t="inlineStr">
         <is>
-          <t>https://www.aquabased.com/customformulations/</t>
+          <t>https://biocoat.com/about/</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>NOT PUBLISHED — no heating capability stated anywhere on the site. This is the first question to ask; if they only have ambient/low-heat mix tanks they are disqualified like ILC Dover.</t>
+          <t>PARTIAL. They publicly describe 'large batch thermal curing' capability, which confirms heated batch equipment on site. However that refers to curing coatings on devices, NOT necessarily to a jacketed solution kettle holding 90-95 C. Specific solution-batch t…</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>GOOD — 'from initial laboratory small testing quantities to multiple drum and tote quantities.' Drum-scale is explicitly in their stated range, so a single 450…</t>
+          <t>Plausible - a specialty coating-solution supplier ships modest volumes of high-value liquid to device OEMs. Their normal package is likely bottles/jugs rather …</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>Not published. Ask about ISO 9001, lot traceability, retained samples, and CoA fields.</t>
+          <t>ISO 13485:2016 certified; quality controls conducted in strict conformance with cGMP regulations; six ISO 7 cleanrooms across two facilitie…</t>
         </is>
       </c>
       <c r="H47" s="23" t="inlineStr">
         <is>
-          <t>201.767.6040 / info@aquabased.com</t>
+          <t>Contact form at biocoat.com; ask for contract manufacturing rather than contract coating services</t>
         </is>
       </c>
       <c r="I47" s="23" t="inlineStr">
         <is>
-          <t>A dedicated WATER-BASED-only house — coatings, adhesives and primers — offering exactly the three services we need bundled: custom formulating, toll manufacturing, and private label. They explicitly scale 'from initial laboratory small testing quantities to multiple drum and tote quantities' and emphasize batch-to-batch consistency, which is the correct posture for a made-fresh-to-order weekly drum with an 18-day sh…</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Biocoat formulates and manufactures AQUEOUS-BASED polymer coating solutions for Class II/III devices (neurovascular, cardiovascular, peripheral, ophthalmic) - so like Hydromer, their finished good is functionally the same kind of product a…</t>
         </is>
       </c>
       <c r="J47" s="25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>HIGH on quality system …</t>
         </is>
       </c>
     </row>
@@ -3514,47 +3558,47 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>Biocoat Incorporated  [NEW]</t>
+          <t>Brainerd Chemical  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>Horsham, PA (two facilities, 46,000 sq ft, six ISO 7 cleanrooms)</t>
+          <t>Tulsa, OK</t>
         </is>
       </c>
       <c r="D48" s="24" t="inlineStr">
         <is>
-          <t>https://biocoat.com/about/</t>
+          <t>https://brainerdchemical.com/blending/</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>PARTIAL. They publicly describe 'large batch thermal curing' capability, which confirms heated batch equipment on site. However that refers to curing coatings on devices, NOT necessarily to a jacketed solution kettle holding 90-95 C. Specific solution-batch t…</t>
+          <t>SILENT — no mention of steam, jackets or temperature anywhere</t>
         </is>
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>Plausible - a specialty coating-solution supplier ships modest volumes of high-value liquid to device OEMs. Their normal package is likely bottles/jugs rather …</t>
+          <t>'Batch sizes from 55 to 40,000 gallons' — the 55-gal floor is exactly our batch</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified; quality controls conducted in strict conformance with cGMP regulations; six ISO 7 cleanrooms across two facilitie…</t>
+          <t>SILENT on ISO, CoA and traceability</t>
         </is>
       </c>
       <c r="H48" s="23" t="inlineStr">
         <is>
-          <t>Contact form at biocoat.com; ask for contract manufacturing rather than contract coating services</t>
+          <t>brainerdchemical.com/getstartednow | 918-622-1214</t>
         </is>
       </c>
       <c r="I48" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Biocoat formulates and manufactures AQUEOUS-BASED polymer coating solutions for Class II/III devices (neurovascular, cardiovascular, peripheral, ophthalmic) - so like Hydromer, their finished good is functionally the same kind of product a…</t>
+          <t>The published 55-gallon floor matches our drum precisely. But with heat, certifications and traceability all unpublished, this is a pure cold call.</t>
         </is>
       </c>
       <c r="J48" s="25" t="inlineStr">
         <is>
-          <t>HIGH on quality system …</t>
+          <t>L-M</t>
         </is>
       </c>
     </row>
@@ -3566,47 +3610,47 @@
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>Brainerd Chemical  [NATIONWIDE]</t>
+          <t>CORECHEM</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
         <is>
-          <t>Tulsa, OK</t>
+          <t>Knoxville TN</t>
         </is>
       </c>
       <c r="D49" s="24" t="inlineStr">
         <is>
-          <t>https://brainerdchemical.com/blending/</t>
+          <t>https://www.corechemtn.com</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>SILENT — no mention of steam, jackets or temperature anywhere</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>'Batch sizes from 55 to 40,000 gallons' — the 55-gal floor is exactly our batch</t>
+          <t>CAUTION — smallest tank ~250 gal (~4.5 drums) may overshoot the 18-day shelf life</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>SILENT on ISO, CoA and traceability</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="H49" s="23" t="inlineStr">
         <is>
-          <t>brainerdchemical.com/getstartednow | 918-622-1214</t>
+          <t>on roster</t>
         </is>
       </c>
       <c r="I49" s="23" t="inlineStr">
         <is>
-          <t>The published 55-gallon floor matches our drum precisely. But with heat, certifications and traceability all unpublished, this is a pure cold call.</t>
+          <t>ON OUR ROSTER. Ask specifically about PARTIAL batches — a full 250-gal batch is ~4.5 drums but only ~2 are usable in 18 days.</t>
         </is>
       </c>
       <c r="J49" s="25" t="inlineStr">
         <is>
-          <t>L-M</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -3618,42 +3662,42 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>CORECHEM</t>
+          <t>Chang Chun Petrochemical</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
         <is>
-          <t>Knoxville TN</t>
+          <t>Taiwan (US = distribution only)</t>
         </is>
       </c>
       <c r="D50" s="24" t="inlineStr">
         <is>
-          <t>https://www.corechemtn.com</t>
+          <t>https://www.ccpgp.com/en/</t>
         </is>
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>silent - could not load the site to check; nothing found in indexed content about vessels or temperature. Not applicable to their role.</t>
         </is>
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>CAUTION — smallest tank ~250 gal (~4.5 drums) may overshoot the 18-day shelf life</t>
+          <t>silent - nothing published. As an overseas resin producer they sell in containerload quantities, but that is not stated on the site so treat as unknown.</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
         <is>
-          <t>Not published</t>
+          <t>none found - could not verify any certification because the site would not load.</t>
         </is>
       </c>
       <c r="H50" s="23" t="inlineStr">
         <is>
-          <t>on roster</t>
+          <t>https://www.ccpgp.com/en/ (site intermittent from this network - try from a normal browser). No verified US phone number. If a US resin source is needed, go th…</t>
         </is>
       </c>
       <c r="I50" s="23" t="inlineStr">
         <is>
-          <t>ON OUR ROSTER. Ask specifically about PARTIAL batches — a full 250-gal batch is ~4.5 drums but only ~2 are usable in 18 days.</t>
+          <t>CORRECTION: No location was claimed in the longlist, so no direct error. Add for accuracy: Chang Chun Petrochemical Co., Ltd. is at No. 5, Zhangbin W. 3rd Rd., Xianxi Township, Changhua County 507001, TAIWAN. US presence is UNVERIF…  |  keep C as a resin-supply / price-benchmark contact only. Flag for the buyer: the website is unreliable from automated access and no US entity could be confirmed, so budget extra time…</t>
         </is>
       </c>
       <c r="J50" s="25" t="inlineStr">
@@ -3670,42 +3714,42 @@
       </c>
       <c r="B51" s="23" t="inlineStr">
         <is>
-          <t>Chang Chun Petrochemical</t>
+          <t>Chemical Solvents Inc</t>
         </is>
       </c>
       <c r="C51" s="23" t="inlineStr">
         <is>
-          <t>Taiwan (US = distribution only)</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="D51" s="24" t="inlineStr">
         <is>
-          <t>https://www.ccpgp.com/en/</t>
+          <t>https://www.chemicalsolvents.com</t>
         </is>
       </c>
       <c r="E51" s="23" t="inlineStr">
         <is>
-          <t>silent - could not load the site to check; nothing found in indexed content about vessels or temperature. Not applicable to their role.</t>
+          <t>silent - the toll manufacturing page describes viscosity capability and quantity range but says NOTHING about heated vessels, jacketed tanks, steam, or any maximum temperature. Direct quote of what they DO say: CSI 'toll manufactures a wide range of Solvent a…</t>
         </is>
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>silent - nothing published. As an overseas resin producer they sell in containerload quantities, but that is not stated on the site so treat as unknown.</t>
+          <t>No numeric MOQ, but a strong positive qualitative signal, quoted: orders are 'routinely...in quantities from pails to full tankers'. Pail-scale work being rout…</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
         <is>
-          <t>none found - could not verify any certification because the site would not load.</t>
+          <t>none found - no ISO 9001, no ISO 13485, no FDA registration, no cGMP, no kosher, and no lot-traceability statement published anywhere on th…</t>
         </is>
       </c>
       <c r="H51" s="23" t="inlineStr">
         <is>
-          <t>https://www.ccpgp.com/en/ (site intermittent from this network - try from a normal browser). No verified US phone number. If a US resin source is needed, go th…</t>
+          <t>https://chemicalsolvents.com/contact/ - Phone 800-362-0693 or 216-741-9310, info@chemicalsolvents.com. Business hours Mon-Thu 8:00 AM - 4:00 PM.</t>
         </is>
       </c>
       <c r="I51" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: No location was claimed in the longlist, so no direct error. Add for accuracy: Chang Chun Petrochemical Co., Ltd. is at No. 5, Zhangbin W. 3rd Rd., Xianxi Township, Changhua County 507001, TAIWAN. US presence is UNVERIF…  |  keep C as a resin-supply / price-benchmark contact only. Flag for the buyer: the website is unreliable from automated access and no US entity could be confirmed, so budget extra time…</t>
+          <t>CORRECTION: none material. Cleveland OH confirmed: 3751 Jennings Road, Cleveland, OH 44109. One IMPORTANT ADDITION the longlist omits: CSI's core business is solvent recycling and hazardous-waste processing - they operate 'a modern…  |  keep C, with a clear promotion path. Two of the three gates look promising - they explicitly advertise toll manufacturing of AQUEOUS blends (not just solvents), they handle up to 1,0…</t>
         </is>
       </c>
       <c r="J51" s="25" t="inlineStr">
@@ -3722,47 +3766,47 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>Chemical Solvents Inc</t>
+          <t>Chemjet</t>
         </is>
       </c>
       <c r="C52" s="23" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>CORRECTED: plants Conroe &amp; Odessa TX (Houston = sales office)</t>
         </is>
       </c>
       <c r="D52" s="24" t="inlineStr">
         <is>
-          <t>https://www.chemicalsolvents.com</t>
+          <t>https://www.chemjet.com</t>
         </is>
       </c>
       <c r="E52" s="23" t="inlineStr">
         <is>
-          <t>silent - the toll manufacturing page describes viscosity capability and quantity range but says NOTHING about heated vessels, jacketed tanks, steam, or any maximum temperature. Direct quote of what they DO say: CSI 'toll manufactures a wide range of Solvent a…</t>
+          <t>DOES NOT CLEAR - and the one heat statement is easy to misread. Verbatim, the ONLY heat reference on the site: 'a large 210 F heat room for high molecular weight intermediates that need heating.' 210 F is 98.9 C, which looks like it clears 90-95 C, but a HEAT…</t>
         </is>
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>No numeric MOQ, but a strong positive qualitative signal, quoted: orders are 'routinely...in quantities from pails to full tankers'. Pail-scale work being rout…</t>
+          <t>SILENT. Site says 'over 20 unique blending/mixing tanks, including multiple high shear blending turbines with patented technology' but publishes no tank sizes,…</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
         <is>
-          <t>none found - no ISO 9001, no ISO 13485, no FDA registration, no cGMP, no kosher, and no lot-traceability statement published anywhere on th…</t>
+          <t>'ISO 9001:2015 and API Spec Q1 Registered.' API Q1 is a petroleum/drilling-sector standard. No ISO 13485, no FDA registration, no cGMP, no …</t>
         </is>
       </c>
       <c r="H52" s="23" t="inlineStr">
         <is>
-          <t>https://chemicalsolvents.com/contact/ - Phone 800-362-0693 or 216-741-9310, info@chemicalsolvents.com. Business hours Mon-Thu 8:00 AM - 4:00 PM.</t>
+          <t>https://www.chemjet.com/contact-us | Phone +1 (281) 994-5416 | info@chemjet.com | Toll blending page: https://www.chemjet.com/toll-blending-private-labeling</t>
         </is>
       </c>
       <c r="I52" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: none material. Cleveland OH confirmed: 3751 Jennings Road, Cleveland, OH 44109. One IMPORTANT ADDITION the longlist omits: CSI's core business is solvent recycling and hazardous-waste processing - they operate 'a modern…  |  keep C, with a clear promotion path. Two of the three gates look promising - they explicitly advertise toll manufacturing of AQUEOUS blends (not just solvents), they handle up to 1,0…</t>
+          <t>CORRECTION: TWO MATERIAL ERRORS. (1) LOCATION: Houston is the corporate OFFICE only - '16290 Katy Freeway, Suite 200, Houston, Texas 77094' is an office suite, not a plant. The actual blending plants are in CONROE TX (Specialty Liq…  |  MOVE A -&gt; C. Three strikes: the heat gate is unproven (a heat room is not a jacketed vessel), the plants are in Conroe/Odessa rather than the listed Houston, and a dedicated drilling…</t>
         </is>
       </c>
       <c r="J52" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -3774,47 +3818,47 @@
       </c>
       <c r="B53" s="23" t="inlineStr">
         <is>
-          <t>Chemjet</t>
+          <t>Cortec Corporation / Cortec Advanced Films  [NEW]</t>
         </is>
       </c>
       <c r="C53" s="23" t="inlineStr">
         <is>
-          <t>CORRECTED: plants Conroe &amp; Odessa TX (Houston = sales office)</t>
+          <t>4119 White Bear Parkway, St. Paul, MN 55110 (film plant: Cambridge, MN)</t>
         </is>
       </c>
       <c r="D53" s="24" t="inlineStr">
         <is>
-          <t>https://www.chemjet.com</t>
+          <t>https://www.cortecvci.com/products/vpci-packaging-products/ecosol-water-soluble-packaging-solution/</t>
         </is>
       </c>
       <c r="E53" s="23" t="inlineStr">
         <is>
-          <t>DOES NOT CLEAR - and the one heat statement is easy to misread. Verbatim, the ONLY heat reference on the site: 'a large 210 F heat room for high molecular weight intermediates that need heating.' 210 F is 98.9 C, which looks like it clears 90-95 C, but a HEAT…</t>
+          <t>NOT PUBLISHED and genuinely uncertain given the extrusion-vs-solution-cast question above. Their liquid chemical blending side would need to be assessed separately for jacketed heating to 90-95 C.</t>
         </is>
       </c>
       <c r="F53" s="23" t="inlineStr">
         <is>
-          <t>SILENT. Site says 'over 20 unique blending/mixing tanks, including multiple high shear blending turbines with patented technology' but publishes no tank sizes,…</t>
+          <t>LIKELY GOOD — Cortec runs a very wide SKU count across many small specialty products and does contract filling, so single-drum lots should be within their norm…</t>
         </is>
       </c>
       <c r="G53" s="23" t="inlineStr">
         <is>
-          <t>'ISO 9001:2015 and API Spec Q1 Registered.' API Q1 is a petroleum/drilling-sector standard. No ISO 13485, no FDA registration, no cGMP, no …</t>
+          <t>STRONG — ISO 9001:2015 and ISO 14001:2015 certified; ISO 9001 registered continuously since 1994. Formal CoA practice on their own products.</t>
         </is>
       </c>
       <c r="H53" s="23" t="inlineStr">
         <is>
-          <t>https://www.chemjet.com/contact-us | Phone +1 (281) 994-5416 | info@chemjet.com | Toll blending page: https://www.chemjet.com/toll-blending-private-labeling</t>
+          <t>Via cortecvci.com contact. Route the inquiry to custom/contract manufacturing rather than the VpCI product lines.</t>
         </is>
       </c>
       <c r="I53" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: TWO MATERIAL ERRORS. (1) LOCATION: Houston is the corporate OFFICE only - '16290 Katy Freeway, Suite 200, Houston, Texas 77094' is an office suite, not a plant. The actual blending plants are in CONROE TX (Specialty Liq…  |  MOVE A -&gt; C. Three strikes: the heat gate is unproven (a heat room is not a jacketed vessel), the plants are in Conroe/Odessa rather than the listed Houston, and a dedicated drilling…</t>
+          <t>Vertically integrated US chemical manufacturer that runs BOTH a PVOH business and a custom-manufacturing business. Cortec Advanced Films produces EcoSol, a water-soluble biodegradable polyvinyl alcohol (PVOH) film, so PVOH handling, specification and QC are in-house competencies. Separately, Cortec offers contract fill and private labeling and states they are 'ready to help customers adapt their own formulas... or c…</t>
         </is>
       </c>
       <c r="J53" s="25" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -3826,47 +3870,43 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>Cortec Corporation / Cortec Advanced Films  [NEW]</t>
+          <t>Ethox Chemicals</t>
         </is>
       </c>
       <c r="C54" s="23" t="inlineStr">
         <is>
-          <t>4119 White Bear Parkway, St. Paul, MN 55110 (film plant: Cambridge, MN)</t>
-        </is>
-      </c>
-      <c r="D54" s="24" t="inlineStr">
-        <is>
-          <t>https://www.cortecvci.com/products/vpci-packaging-products/ecosol-water-soluble-packaging-solution/</t>
-        </is>
-      </c>
+          <t>Greenville, SC</t>
+        </is>
+      </c>
+      <c r="D54" s="23" t="inlineStr"/>
       <c r="E54" s="23" t="inlineStr">
         <is>
-          <t>NOT PUBLISHED and genuinely uncertain given the extrusion-vs-solution-cast question above. Their liquid chemical blending side would need to be assessed separately for jacketed heating to 90-95 C.</t>
+          <t>PASSES ON CAPABILITY. Equipment includes '2500 and 7500 gallon Hot Oil reactors with condensers and receivers,' plus '100 PSI 316SS reactors ranging from 800 gallons to 6500 gallons' and 'assorted mixing tanks.' Hot oil reactors clear 90-95 C with large margi…</t>
         </is>
       </c>
       <c r="F54" s="23" t="inlineStr">
         <is>
-          <t>LIKELY GOOD — Cortec runs a very wide SKU count across many small specialty products and does contract filling, so single-drum lots should be within their norm…</t>
+          <t>POOR FIT. Smallest published reactor is 800 gallons — ~15x our ~53 gal batch. 'Assorted mixing tanks' are mentioned without sizes, which is the only possible s…</t>
         </is>
       </c>
       <c r="G54" s="23" t="inlineStr">
         <is>
-          <t>STRONG — ISO 9001:2015 and ISO 14001:2015 certified; ISO 9001 registered continuously since 1994. Formal CoA practice on their own products.</t>
+          <t>NONE CONFIRMED. No ISO 9001, ISO 13485, FDA registration, or cGMP found on the site or in search. Site does reference laboratory, pilot, an…</t>
         </is>
       </c>
       <c r="H54" s="23" t="inlineStr">
         <is>
-          <t>Via cortecvci.com contact. Route the inquiry to custom/contract manufacturing rather than the VpCI product lines.</t>
+          <t>https://www.ethox.com/contact/ — 864-277-1620</t>
         </is>
       </c>
       <c r="I54" s="23" t="inlineStr">
         <is>
-          <t>Vertically integrated US chemical manufacturer that runs BOTH a PVOH business and a custom-manufacturing business. Cortec Advanced Films produces EcoSol, a water-soluble biodegradable polyvinyl alcohol (PVOH) film, so PVOH handling, specification and QC are in-house competencies. Separately, Cortec offers contract fill and private labeling and states they are 'ready to help customers adapt their own formulas... or c…</t>
+          <t>CORRECTION: Listing omits the Syntha Group parent — Ethox is not an independent company. Location correct: 1801 Perimeter Road, Greenville SC 29605, 45-acre site with rail access off I-85. Also note Ethox has commenced construction…  |  MOVE B → C. Real heat capability, but minimum vessel 800 gal, no confirmed quality certifications, and a high-value custom-synthesis cost structure aimed at surfactant chemistry. Sam…</t>
         </is>
       </c>
       <c r="J54" s="25" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -3878,43 +3918,47 @@
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>Ethox Chemicals</t>
+          <t>FORREST Technical Coatings  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>Greenville, SC</t>
-        </is>
-      </c>
-      <c r="D55" s="23" t="inlineStr"/>
+          <t>Eugene, OR</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="inlineStr">
+        <is>
+          <t>https://forrestpaint.com/toll-chemical-manufacturing/</t>
+        </is>
+      </c>
       <c r="E55" s="23" t="inlineStr">
         <is>
-          <t>PASSES ON CAPABILITY. Equipment includes '2500 and 7500 gallon Hot Oil reactors with condensers and receivers,' plus '100 PSI 316SS reactors ranging from 800 gallons to 6500 gallons' and 'assorted mixing tanks.' Hot oil reactors clear 90-95 C with large margi…</t>
+          <t>SILENT for process heat. CAUTION: the site's '1,200 F' references are the SERVICE temperature of their high-temp paints, not process capability — do not misread as a heat-gate pass.</t>
         </is>
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>POOR FIT. Smallest published reactor is 800 gallons — ~15x our ~53 gal batch. 'Assorted mixing tanks' are mentioned without sizes, which is the only possible s…</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
         <is>
-          <t>NONE CONFIRMED. No ISO 9001, ISO 13485, FDA registration, or cGMP found on the site or in search. Site does reference laboratory, pilot, an…</t>
+          <t>ISO 9001:2015</t>
         </is>
       </c>
       <c r="H55" s="23" t="inlineStr">
         <is>
-          <t>https://www.ethox.com/contact/ — 864-277-1620</t>
+          <t>forrestpaint.com/contact | 1-800-537-7201</t>
         </is>
       </c>
       <c r="I55" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: Listing omits the Syntha Group parent — Ethox is not an independent company. Location correct: 1801 Perimeter Road, Greenville SC 29605, 45-acre site with rail access off I-85. Also note Ethox has commenced construction…  |  MOVE B → C. Real heat capability, but minimum vessel 800 gal, no confirmed quality certifications, and a high-value custom-synthesis cost structure aimed at surfactant chemistry. Sam…</t>
+          <t>The only independent toll manufacturer verifiable in the entire Pacific Northwest. Water-based coatings shop that tolls for other brands, so the model fits even though the equipment is unproven.</t>
         </is>
       </c>
       <c r="J55" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L-M</t>
         </is>
       </c>
     </row>
@@ -3926,22 +3970,22 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>FORREST Technical Coatings  [NATIONWIDE]</t>
+          <t>Florida CirTech  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
         <is>
-          <t>Eugene, OR</t>
+          <t>Greeley, CO</t>
         </is>
       </c>
       <c r="D56" s="24" t="inlineStr">
         <is>
-          <t>https://forrestpaint.com/toll-chemical-manufacturing/</t>
+          <t>https://floridacirtech.com/toll-blending/</t>
         </is>
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>SILENT for process heat. CAUTION: the site's '1,200 F' references are the SERVICE temperature of their high-temp paints, not process capability — do not misread as a heat-gate pass.</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="F56" s="23" t="inlineStr">
@@ -3951,22 +3995,22 @@
       </c>
       <c r="G56" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001:2015</t>
+          <t>ISO 9001:2015; customer portal issues Certificates of Analysis, SDS and quality docs as a productized deliverable</t>
         </is>
       </c>
       <c r="H56" s="23" t="inlineStr">
         <is>
-          <t>forrestpaint.com/contact | 1-800-537-7201</t>
+          <t>floridacirtech.com/contact | 970-346-8002</t>
         </is>
       </c>
       <c r="I56" s="23" t="inlineStr">
         <is>
-          <t>The only independent toll manufacturer verifiable in the entire Pacific Northwest. Water-based coatings shop that tolls for other brands, so the model fits even though the equipment is unproven.</t>
+          <t>The only credible ISO 9001 toll blender verifiable in Colorado, and a PCB-chemistry house so aqueous process chemistry is their day job. Our CoA requirement is already something they ship as standard. Both gates unverified — a discovery call.</t>
         </is>
       </c>
       <c r="J56" s="25" t="inlineStr">
         <is>
-          <t>L-M</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -3978,42 +4022,42 @@
       </c>
       <c r="B57" s="23" t="inlineStr">
         <is>
-          <t>Florida CirTech  [NATIONWIDE]</t>
+          <t>Formula Corp</t>
         </is>
       </c>
       <c r="C57" s="23" t="inlineStr">
         <is>
-          <t>Greeley, CO</t>
+          <t>Auburn, WA</t>
         </is>
       </c>
       <c r="D57" s="24" t="inlineStr">
         <is>
-          <t>https://floridacirtech.com/toll-blending/</t>
+          <t>https://formulacorp.com</t>
         </is>
       </c>
       <c r="E57" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>silent - I found NO statement about heated or jacketed kettles, steam, or any maximum process temperature on any reachable page, including /policies/. Their ISO 22716 scope wording is 'Mixing, blending, and packaging of liquid or pasty water based cosmetic pr…</t>
         </is>
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>NEGATIVE SIGNAL, likely disqualifying. A line sourced to their own site states products are blended in load-cell-mounted tanks with 'a minimum runs batch size …</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001:2015; customer portal issues Certificates of Analysis, SDS and quality docs as a productized deliverable</t>
+          <t>The strongest published quality package in Tier C, verified verbatim from formulacorp.com/policies/: 'ISO 22716:2007 Certified - SGS North …</t>
         </is>
       </c>
       <c r="H57" s="23" t="inlineStr">
         <is>
-          <t>floridacirtech.com/contact | 970-346-8002</t>
+          <t>https://formulacorp.com/contact/ (Request a Manufacturing Quote form) - Phone (253) 880-0170 or 800-772-7005, info@formulacorp.com. Hours Mon-Thu 8:00-4:30, Fr…</t>
         </is>
       </c>
       <c r="I57" s="23" t="inlineStr">
         <is>
-          <t>The only credible ISO 9001 toll blender verifiable in Colorado, and a PCB-chemistry house so aqueous process chemistry is their day job. Our CoA requirement is already something they ship as standard. Both gates unverified — a discovery call.</t>
+          <t>CORRECTION: Auburn WA is CORRECT: 4432 C St NE, Auburn, WA 98002. Note that public revenue figures conflict badly across sources (D&amp;B shows $9.61M / 21 employees; another source shows $38.2M) - do not rely on either. Positioning co…  |  keep C - do NOT promote yet, but this is the highest-value call in Tier C. Uniquely among these 13, toll manufacturing is written into their certified ISO 9001:2015 scope, and they h…</t>
         </is>
       </c>
       <c r="J57" s="25" t="inlineStr">
@@ -4030,47 +4074,47 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>Formula Corp</t>
+          <t>GeminiBio (Gemini Bioproducts, LLC)  [NEW]</t>
         </is>
       </c>
       <c r="C58" s="23" t="inlineStr">
         <is>
-          <t>Auburn, WA</t>
+          <t>920 Stillwater Rd Suite 130, West Sacramento, CA 95605</t>
         </is>
       </c>
       <c r="D58" s="24" t="inlineStr">
         <is>
-          <t>https://formulacorp.com</t>
+          <t>https://www.geminibio.com/solutions-process-liquid/</t>
         </is>
       </c>
       <c r="E58" s="23" t="inlineStr">
         <is>
-          <t>silent - I found NO statement about heated or jacketed kettles, steam, or any maximum process temperature on any reachable page, including /policies/. Their ISO 22716 scope wording is 'Mixing, blending, and packaging of liquid or pasty water based cosmetic pr…</t>
+          <t>SILENT on max temperature. Batch range (10 L to 10,000 L) and tank inventory are published, but jacket capability and process temperature ceiling are not. Media hydration work typically involves controlled heating, but 90-95 C hold is UNVERIFIED. NOTE: biopro…</t>
         </is>
       </c>
       <c r="F58" s="23" t="inlineStr">
         <is>
-          <t>NEGATIVE SIGNAL, likely disqualifying. A line sourced to their own site states products are blended in load-cell-mounted tanks with 'a minimum runs batch size …</t>
+          <t>Strong. Batch sizes start at 10 L, so a ~200 L / 450 lb batch is well within range and not a nuisance-size order. Customizable fill sizes and container types o…</t>
         </is>
       </c>
       <c r="G58" s="23" t="inlineStr">
         <is>
-          <t>The strongest published quality package in Tier C, verified verbatim from formulacorp.com/policies/: 'ISO 22716:2007 Certified - SGS North …</t>
+          <t>ISO 13485:2016 certified; FDA registered as Class I Medical Device Manufacturer; compliant with 21 CFR Part 820; cGMP; WFI-quality water sy…</t>
         </is>
       </c>
       <c r="H58" s="23" t="inlineStr">
         <is>
-          <t>https://formulacorp.com/contact/ (Request a Manufacturing Quote form) - Phone (253) 880-0170 or 800-772-7005, info@formulacorp.com. Hours Mon-Thu 8:00-4:30, Fr…</t>
+          <t>(800) 543-6464; request the custom cGMP process liquid team (ExpressCustom / TrueCustom)</t>
         </is>
       </c>
       <c r="I58" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: Auburn WA is CORRECT: 4432 C St NE, Auburn, WA 98002. Note that public revenue figures conflict badly across sources (D&amp;B shows $9.61M / 21 employees; another source shows $38.2M) - do not rely on either. Positioning co…  |  keep C - do NOT promote yet, but this is the highest-value call in Tier C. Uniquely among these 13, toll manufacturing is written into their certified ISO 9001:2015 scope, and they h…</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | The only candidate found that EXPLICITLY states it accepts customer-specific specifications AND customer-supplied raw materials - which is the toll model you need, stated on the vendor's own site rather than inferred. They custom-manufactu…</t>
         </is>
       </c>
       <c r="J58" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>HIGH on quality credent…</t>
         </is>
       </c>
     </row>
@@ -4082,47 +4126,47 @@
       </c>
       <c r="B59" s="23" t="inlineStr">
         <is>
-          <t>GeminiBio (Gemini Bioproducts, LLC)  [NEW]</t>
+          <t>Griffin Chem Solutions  [UNVERIFIED]</t>
         </is>
       </c>
       <c r="C59" s="23" t="inlineStr">
         <is>
-          <t>920 Stillwater Rd Suite 130, West Sacramento, CA 95605</t>
+          <t>Albany + Salem, OR</t>
         </is>
       </c>
       <c r="D59" s="24" t="inlineStr">
         <is>
-          <t>https://www.geminibio.com/solutions-process-liquid/</t>
+          <t>https://griffinchemsolutions.com</t>
         </is>
       </c>
       <c r="E59" s="23" t="inlineStr">
         <is>
-          <t>SILENT on max temperature. Batch range (10 L to 10,000 L) and tank inventory are published, but jacket capability and process temperature ceiling are not. Media hydration work typically involves controlled heating, but 90-95 C hold is UNVERIFIED. NOTE: biopro…</t>
+          <t>COULD NOT VERIFY — site sits behind a bot-challenge and returned only challenge pages to every fetch attempt.</t>
         </is>
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>Strong. Batch sizes start at 10 L, so a ~200 L / 450 lb batch is well within range and not a nuisance-size order. Customizable fill sizes and container types o…</t>
+          <t>Search-extracted text (NOT read from their server) claims 'the capacity to blend by the truckload down to a gallon at a time' and a 40,000 sq ft Albany facility with fifteen liquid blending systems.</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified; FDA registered as Class I Medical Device Manufacturer; compliant with 21 CFR Part 820; cGMP; WFI-quality water sy…</t>
+          <t>Claims operation 'based on ISO-9001 (2015) standards' — unverified</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
         <is>
-          <t>(800) 543-6464; request the custom cGMP process liquid team (ExpressCustom / TrueCustom)</t>
+          <t>griffinchemsolutions.com (site would not load) — phone via search listing</t>
         </is>
       </c>
       <c r="I59" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | The only candidate found that EXPLICITLY states it accepts customer-specific specifications AND customer-supplied raw materials - which is the toll model you need, stated on the vendor's own site rather than inferred. They custom-manufactu…</t>
+          <t>LISTED WITH A WARNING, NOT AS A VERIFIED LEAD. If the 'truckload down to a gallon' claim is real it is an excellent small-batch answer, and Oregon is otherwise nearly empty. Treat every capability claim as unconfirmed until they say it on the phone.</t>
         </is>
       </c>
       <c r="J59" s="25" t="inlineStr">
         <is>
-          <t>HIGH on quality credent…</t>
+          <t>UNVERIFIED</t>
         </is>
       </c>
     </row>
@@ -4134,47 +4178,47 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>Griffin Chem Solutions  [UNVERIFIED]</t>
+          <t>HR Pharmaceuticals, Inc. / HR HealthCare  [NEW]</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
         <is>
-          <t>Albany + Salem, OR</t>
+          <t>HQ 2600 Eastern Blvd Suite 201, York, PA 17402; Manufacturing 3630 Concord Rd, York, PA 17402</t>
         </is>
       </c>
       <c r="D60" s="24" t="inlineStr">
         <is>
-          <t>https://griffinchemsolutions.com</t>
+          <t>https://www.hrhealthcare.com/contract-manufacturing/</t>
         </is>
       </c>
       <c r="E60" s="23" t="inlineStr">
         <is>
-          <t>COULD NOT VERIFY — site sits behind a bot-challenge and returned only challenge pages to every fetch attempt.</t>
+          <t>SILENT on temperature. Site says 'on-site semi-automated compounding' but publishes no kettle sizes, jacket detail, or max temperature. NOTE: ultrasound-gel and lubricating-jelly manufacture typically uses heated jacketed compounding kettles, so 90-95 C is pl…</t>
         </is>
       </c>
       <c r="F60" s="23" t="inlineStr">
         <is>
-          <t>Search-extracted text (NOT read from their server) claims 'the capacity to blend by the truckload down to a gallon at a time' and a 40,000 sq ft Albany facility with fifteen liquid blending systems.</t>
+          <t>CONCERN. Their published filling formats are consumer-scale: plastic bottles 2 oz-32 oz, tubes, poly foil sachets 3g-36g, and flexible packaging. 55-gallon / 4…</t>
         </is>
       </c>
       <c r="G60" s="23" t="inlineStr">
         <is>
-          <t>Claims operation 'based on ISO-9001 (2015) standards' — unverified</t>
+          <t>cGMP compliant; ISO 13485:2016 certified; MDSAP certified; FDA registered facility for healthcare consumables and OTC products; Health Cana…</t>
         </is>
       </c>
       <c r="H60" s="23" t="inlineStr">
         <is>
-          <t>griffinchemsolutions.com (site would not load) — phone via search listing</t>
+          <t>(877) 302-1110 toll-free or (717) 252-1110; inquiries@hrhealthcare.com</t>
         </is>
       </c>
       <c r="I60" s="23" t="inlineStr">
         <is>
-          <t>LISTED WITH A WARNING, NOT AS A VERIFIED LEAD. If the 'truckload down to a gallon' claim is real it is an excellent small-batch answer, and Oregon is otherwise nearly empty. Treat every capability claim as unconfirmed until they say it on the phone.</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | The closest COST-REALISTIC medical-grade analog on this list. HR makes medical/surgical lubricants and ultrasound gels - high-volume aqueous water-soluble-polymer systems with preservatives - in a 105,000 sq ft cGMP plant, and they explici…</t>
         </is>
       </c>
       <c r="J60" s="25" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>HIGH on quality credent…</t>
         </is>
       </c>
     </row>
@@ -4186,47 +4230,47 @@
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>HR Pharmaceuticals, Inc. / HR HealthCare  [NEW]</t>
+          <t>Hydromer, Inc. (OTC: HYDI)  [NEW]</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
         <is>
-          <t>HQ 2600 Eastern Blvd Suite 201, York, PA 17402; Manufacturing 3630 Concord Rd, York, PA 17402</t>
+          <t>4715 Corporate Dr NW, Concord, NC 28027</t>
         </is>
       </c>
       <c r="D61" s="24" t="inlineStr">
         <is>
-          <t>https://www.hrhealthcare.com/contract-manufacturing/</t>
+          <t>https://hydromer.com/coating-manufacturing-services/</t>
         </is>
       </c>
       <c r="E61" s="23" t="inlineStr">
         <is>
-          <t>SILENT on temperature. Site says 'on-site semi-automated compounding' but publishes no kettle sizes, jacket detail, or max temperature. NOTE: ultrasound-gel and lubricating-jelly manufacture typically uses heated jacketed compounding kettles, so 90-95 C is pl…</t>
+          <t>SILENT. No batch vessel sizes, jacket capability, or temperature ceiling published. Their coating chemistry includes thermal-cure systems, which implies heated process capability, but the specific 90-95 C solution hold is UNVERIFIED.</t>
         </is>
       </c>
       <c r="F61" s="23" t="inlineStr">
         <is>
-          <t>CONCERN. Their published filling formats are consumer-scale: plastic bottles 2 oz-32 oz, tubes, poly foil sachets 3g-36g, and flexible packaging. 55-gallon / 4…</t>
+          <t>Stated they handle 'small &amp; large production runs' and coat prototypes through market-ready devices. A specialty coating-solution house is structurally built f…</t>
         </is>
       </c>
       <c r="G61" s="23" t="inlineStr">
         <is>
-          <t>cGMP compliant; ISO 13485:2016 certified; MDSAP certified; FDA registered facility for healthcare consumables and OTC products; Health Cana…</t>
+          <t>ISO 13485:2016 certified (BSI); ISO 9001:2015 certified (TUV Rheinland); FDA registered production facility; described as an FDA/GMP produc…</t>
         </is>
       </c>
       <c r="H61" s="23" t="inlineStr">
         <is>
-          <t>(877) 302-1110 toll-free or (717) 252-1110; inquiries@hrhealthcare.com</t>
+          <t>+1 704-490-4031; info@hydromer.com</t>
         </is>
       </c>
       <c r="I61" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | The closest COST-REALISTIC medical-grade analog on this list. HR makes medical/surgical lubricants and ultrasound gels - high-volume aqueous water-soluble-polymer systems with preservatives - in a 105,000 sq ft cGMP plant, and they explici…</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Hydromer's entire business is formulating and manufacturing aqueous and solvent polymer solutions that go onto Class II/III medical devices - functionally the same product category as your PVA solution. They state 'all polymer products are…</t>
         </is>
       </c>
       <c r="J61" s="25" t="inlineStr">
         <is>
-          <t>HIGH on quality credent…</t>
+          <t>HIGH on quality system …</t>
         </is>
       </c>
     </row>
@@ -4238,47 +4282,47 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>Hydromer, Inc. (OTC: HYDI)  [NEW]</t>
+          <t>Kingchem Laboratories, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
         <is>
-          <t>4715 Corporate Dr NW, Concord, NC 28027</t>
+          <t>Manufacturing: St. Francis, WI (FDA-registered cGMP site). HQ: Allendale, NJ</t>
         </is>
       </c>
       <c r="D62" s="24" t="inlineStr">
         <is>
-          <t>https://hydromer.com/coating-manufacturing-services/</t>
+          <t>https://www.kingchem.com/facilities/</t>
         </is>
       </c>
       <c r="E62" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No batch vessel sizes, jacket capability, or temperature ceiling published. Their coating chemistry includes thermal-cure systems, which implies heated process capability, but the specific 90-95 C solution hold is UNVERIFIED.</t>
+          <t>STRONGEST of any candidate, though still inferential. Published fleet of glass-lined/SS/Hastelloy reactors 35 L-6,300 L plus 'advanced distillation units' - distillation capability proves the site routinely operates well above 95 C with jacketed, temperature-…</t>
         </is>
       </c>
       <c r="F62" s="23" t="inlineStr">
         <is>
-          <t>Stated they handle 'small &amp; large production runs' and coat prototypes through market-ready devices. A specialty coating-solution house is structurally built f…</t>
+          <t>Strong. Reactor range starts at 35 L, so a ~200 L batch sits comfortably mid-range. A shop with a 35 L reactor does not treat 450 lb as too small.</t>
         </is>
       </c>
       <c r="G62" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified (BSI); ISO 9001:2015 certified (TUV Rheinland); FDA registered production facility; described as an FDA/GMP produc…</t>
+          <t>FDA-registered facility (St. Francis, WI); cGMP compliant; ICH Q7 compliant; on-site analytical lab for validation and release testing. NOT…</t>
         </is>
       </c>
       <c r="H62" s="23" t="inlineStr">
         <is>
-          <t>+1 704-490-4031; info@hydromer.com</t>
+          <t>kingchem.com/contact/ - request the St. Francis, WI cGMP site for custom excipient manufacturing</t>
         </is>
       </c>
       <c r="I62" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Hydromer's entire business is formulating and manufacturing aqueous and solvent polymer solutions that go onto Class II/III medical devices - functionally the same product category as your PVA solution. They state 'all polymer products are…</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | The single best candidate on this list for the 90-95 C HARD GATE. They publish a reactor fleet of 35 L to 6,300 L in glass-lined, stainless steel and Hastelloy - jacketed chemical reactors that routinely run reflux and elevated-temperature…</t>
         </is>
       </c>
       <c r="J62" s="25" t="inlineStr">
         <is>
-          <t>HIGH on quality system …</t>
+          <t>HIGH on the heat gate a…</t>
         </is>
       </c>
     </row>
@@ -4290,47 +4334,47 @@
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>Kingchem Laboratories, Inc.  [NEW]</t>
+          <t>Kuraray America</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
         <is>
-          <t>Manufacturing: St. Francis, WI (FDA-registered cGMP site). HQ: Allendale, NJ</t>
+          <t>Houston / Pasadena / La Porte, TX</t>
         </is>
       </c>
       <c r="D63" s="24" t="inlineStr">
         <is>
-          <t>https://www.kingchem.com/facilities/</t>
+          <t>https://www.kuraray.com/us-en/</t>
         </is>
       </c>
       <c r="E63" s="23" t="inlineStr">
         <is>
-          <t>STRONGEST of any candidate, though still inferential. Published fleet of glass-lined/SS/Hastelloy reactors 35 L-6,300 L plus 'advanced distillation units' - distillation capability proves the site routinely operates well above 95 C with jacketed, temperature-…</t>
+          <t>silent - no mention of heated/jacketed vessels, reactors, or any temperature on the US site. Not applicable to their role (resin supplier).</t>
         </is>
       </c>
       <c r="F63" s="23" t="inlineStr">
         <is>
-          <t>Strong. Reactor range starts at 35 L, so a ~200 L batch sits comfortably mid-range. A shop with a 35 L reactor does not treat 450 lb as too small.</t>
+          <t>silent - no MOQ or minimum batch published. Site offers a 'Request a Sample' route only.</t>
         </is>
       </c>
       <c r="G63" s="23" t="inlineStr">
         <is>
-          <t>FDA-registered facility (St. Francis, WI); cGMP compliant; ICH Q7 compliant; on-site analytical lab for validation and release testing. NOT…</t>
+          <t>Partial. Homepage cites 'Responsible Care' and a 'Quality Management' section but names no certificate numbers. An ISO 14001 certificate co…</t>
         </is>
       </c>
       <c r="H63" s="23" t="inlineStr">
         <is>
-          <t>kingchem.com/contact/ - request the St. Francis, WI cGMP site for custom excipient manufacturing</t>
+          <t>https://www.kuraray.com/us-en/contact-us/request-more-info/ (also /request-a-sample/). Phone +1 800 423 9762. Kuraray Poval Americas HQ page: kuraray-poval.com…</t>
         </is>
       </c>
       <c r="I63" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | The single best candidate on this list for the 90-95 C HARD GATE. They publish a reactor fleet of 35 L to 6,300 L in glass-lined, stainless steel and Hastelloy - jacketed chemical reactors that routinely run reflux and elevated-temperature…</t>
+          <t>CORRECTION: URL correction: kuraray.us.com 301-redirects to kuraray.com/us-en/. Houston TX is CORRECT, but the address changed - HQ relocated 14 Nov 2022 to 3700 Bay Area Blvd, Suite 680, Houston TX 77058. PVA brands confirmed on s…  |  keep - correct C role as resin supplier / technical resource, not a toll blender. Two added angles worth using: (a) Kuraray Exceval is the super-hydrolyzed grade family that matches …</t>
         </is>
       </c>
       <c r="J63" s="25" t="inlineStr">
         <is>
-          <t>HIGH on the heat gate a…</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -4342,42 +4386,42 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>Kuraray America</t>
+          <t>MFG Chemical</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
         <is>
-          <t>Houston / Pasadena / La Porte, TX</t>
+          <t>Chattanooga TN; plants Dalton GA</t>
         </is>
       </c>
       <c r="D64" s="24" t="inlineStr">
         <is>
-          <t>https://www.kuraray.com/us-en/</t>
+          <t>https://mfgchemical.com</t>
         </is>
       </c>
       <c r="E64" s="23" t="inlineStr">
         <is>
-          <t>silent - no mention of heated/jacketed vessels, reactors, or any temperature on the US site. Not applicable to their role (resin supplier).</t>
+          <t>CLEARS THE GATE BY A WIDE MARGIN - the only candidate of the nine with published temperature data. Verbatim: '26 reactors ranging from 2,000 gal (7,500L) to 8,000 gal (30,000L)'; construction 'Glass-Lined, 316 Stainless, and Hastelloy'; hot oil systems 'up to…</t>
         </is>
       </c>
       <c r="F64" s="23" t="inlineStr">
         <is>
-          <t>silent - no MOQ or minimum batch published. Site offers a 'Request a Sample' route only.</t>
+          <t>SILENT on stated MOQ, but the equipment list disqualifies on scale. Smallest PRODUCTION reactor is 2,000 gal; your batch is ~50 gal. Only the 100-gal pilot uni…</t>
         </is>
       </c>
       <c r="G64" s="23" t="inlineStr">
         <is>
-          <t>Partial. Homepage cites 'Responsible Care' and a 'Quality Management' section but names no certificate numbers. An ISO 14001 certificate co…</t>
+          <t>ISO 9001:2015. No ISO 13485, no FDA registration, no cGMP, no lot traceability language found.</t>
         </is>
       </c>
       <c r="H64" s="23" t="inlineStr">
         <is>
-          <t>https://www.kuraray.com/us-en/contact-us/request-more-info/ (also /request-a-sample/). Phone +1 800 423 9762. Kuraray Poval Americas HQ page: kuraray-poval.com…</t>
+          <t>https://mfgchemical.com/contact-us/ | Phone (706) 226-4114</t>
         </is>
       </c>
       <c r="I64" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: URL correction: kuraray.us.com 301-redirects to kuraray.com/us-en/. Houston TX is CORRECT, but the address changed - HQ relocated 14 Nov 2022 to 3700 Bay Area Blvd, Suite 680, Houston TX 77058. PVA brands confirmed on s…  |  keep - correct C role as resin supplier / technical resource, not a toll blender. Two added angles worth using: (a) Kuraray Exceval is the super-hydrolyzed grade family that matches …</t>
+          <t>CORRECTION: Listed location is CORRECT: HQ at 605 Chestnut Street, Suite 1250, Chattanooga TN 37450, with three of its plants in Dalton GA (Brooks Road, Callahan Road, Kimberly Park Drive). Two things the list misses: (1) the Janua…  |  MOVE A -&gt; C on scale mismatch, not on capability. The heat gate is a slam dunk, but asking a 26-reactor custom synthesis operation with a 2,000-gallon minimum vessel to make one 450 …</t>
         </is>
       </c>
       <c r="J64" s="25" t="inlineStr">
@@ -4394,47 +4438,47 @@
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>MFG Chemical</t>
+          <t>Medical Products Laboratories, Inc. (MPL)  [NEW]</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
         <is>
-          <t>Chattanooga TN; plants Dalton GA</t>
+          <t>Northeast Philadelphia, PA (250,000 sq ft)</t>
         </is>
       </c>
       <c r="D65" s="24" t="inlineStr">
         <is>
-          <t>https://mfgchemical.com</t>
+          <t>https://www.mplusa.com/liquid-pharmaceutical-contract-manufacturing.html</t>
         </is>
       </c>
       <c r="E65" s="23" t="inlineStr">
         <is>
-          <t>CLEARS THE GATE BY A WIDE MARGIN - the only candidate of the nine with published temperature data. Verbatim: '26 reactors ranging from 2,000 gal (7,500L) to 8,000 gal (30,000L)'; construction 'Glass-Lined, 316 Stainless, and Hastelloy'; hot oil systems 'up to…</t>
+          <t>SILENT on specific temperature, but the strongest DOCUMENTED liquid-batch infrastructure among the device/pharma candidates: 30-3,000 gallon liquid batch capability with overhead Lightnin mixers (VFD, low speed to 5,000+ RPM). Syrup and suspension manufacture…</t>
         </is>
       </c>
       <c r="F65" s="23" t="inlineStr">
         <is>
-          <t>SILENT on stated MOQ, but the equipment list disqualifies on scale. Smallest PRODUCTION reactor is 2,000 gal; your batch is ~50 gal. Only the 100-gal pilot uni…</t>
+          <t>WEAK for your cadence. Their published floor is 30 gallons, so a single ~55-gal drum is technically feasible, but a 250,000 sq ft plant geared to 3,000-gallon …</t>
         </is>
       </c>
       <c r="G65" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001:2015. No ISO 13485, no FDA registration, no cGMP, no lot traceability language found.</t>
+          <t>FDA-registered manufacturer for drug and devices; ISO certified; cGMP/cGxP compliant per their own site. COUNTERVAILING: open FDA Warning L…</t>
         </is>
       </c>
       <c r="H65" s="23" t="inlineStr">
         <is>
-          <t>https://mfgchemical.com/contact-us/ | Phone (706) 226-4114</t>
+          <t>mplusa.com contact page (note: some pages return HTTP 403 to automated fetches; site is live in a normal browser)</t>
         </is>
       </c>
       <c r="I65" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: Listed location is CORRECT: HQ at 605 Chestnut Street, Suite 1250, Chattanooga TN 37450, with three of its plants in Dalton GA (Brooks Road, Callahan Road, Kimberly Park Drive). Two things the list misses: (1) the Janua…  |  MOVE A -&gt; C on scale mismatch, not on capability. The heat gate is a slam dunk, but asking a 26-reactor custom synthesis operation with a 2,000-gallon minimum vessel to make one 450 …</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Included for process-capability completeness and, more importantly, as a DILIGENCE WARNING. On paper MPL is an excellent process match: founded 1928, 250,000 sq ft, FDA-registered for both drug and device, cGMP/cGxP compliant, with publish…</t>
         </is>
       </c>
       <c r="J65" s="25" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>LOW as a recommended ca…</t>
         </is>
       </c>
     </row>
@@ -4446,47 +4490,47 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>Medical Products Laboratories, Inc. (MPL)  [NEW]</t>
+          <t>Miles Chemical  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
         <is>
-          <t>Northeast Philadelphia, PA (250,000 sq ft)</t>
+          <t>Arleta + Anaheim, CA</t>
         </is>
       </c>
       <c r="D66" s="24" t="inlineStr">
         <is>
-          <t>https://www.mplusa.com/liquid-pharmaceutical-contract-manufacturing.html</t>
+          <t>https://mileschemical.com/chemical-blending/</t>
         </is>
       </c>
       <c r="E66" s="23" t="inlineStr">
         <is>
-          <t>SILENT on specific temperature, but the strongest DOCUMENTED liquid-batch infrastructure among the device/pharma candidates: 30-3,000 gallon liquid batch capability with overhead Lightnin mixers (VFD, low speed to 5,000+ RPM). Syrup and suspension manufacture…</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="F66" s="23" t="inlineStr">
         <is>
-          <t>WEAK for your cadence. Their published floor is 30 gallons, so a single ~55-gal drum is technically feasible, but a 250,000 sq ft plant geared to 3,000-gallon …</t>
+          <t>SILENT. Packaging list runs 5-gal pails to totes — 55-gal drums conspicuously absent, so confirm they fill 55s</t>
         </is>
       </c>
       <c r="G66" s="23" t="inlineStr">
         <is>
-          <t>FDA-registered manufacturer for drug and devices; ISO certified; cGMP/cGxP compliant per their own site. COUNTERVAILING: open FDA Warning L…</t>
+          <t>ISO 9001 + ISO 14001 + OHSAS 18001 + NACD Responsible Distribution; lab with titration, AA, ICP</t>
         </is>
       </c>
       <c r="H66" s="23" t="inlineStr">
         <is>
-          <t>mplusa.com contact page (note: some pages return HTTP 403 to automated fetches; site is live in a normal browser)</t>
+          <t>mileschemical.com contact page | 818-504-3355 | cs@mileschemical.com</t>
         </is>
       </c>
       <c r="I66" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Included for process-capability completeness and, more importantly, as a DILIGENCE WARNING. On paper MPL is an excellent process match: founded 1928, 250,000 sq ft, FDA-registered for both drug and device, cGMP/cGxP compliant, with publish…</t>
+          <t>A distributor that blends, so they already think in conversion-fee terms, and the certification stack plus in-house lab covers the CoA and traceability ask. Two blanks to clear: heat, and whether they fill 55-gal drums.</t>
         </is>
       </c>
       <c r="J66" s="25" t="inlineStr">
         <is>
-          <t>LOW as a recommended ca…</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -4498,42 +4542,42 @@
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>Miles Chemical  [NATIONWIDE]</t>
+          <t>Mitsubishi Chemical America (Gohsenol)</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
         <is>
-          <t>Arleta + Anaheim, CA</t>
+          <t>US sales office only (no US plant)</t>
         </is>
       </c>
       <c r="D67" s="24" t="inlineStr">
         <is>
-          <t>https://mileschemical.com/chemical-blending/</t>
+          <t>https://us.mitsubishi-chemical.com</t>
         </is>
       </c>
       <c r="E67" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>silent - no vessels, reactors, or temperature stated anywhere. Not applicable to their role.</t>
         </is>
       </c>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t>SILENT. Packaging list runs 5-gal pails to totes — 55-gal drums conspicuously absent, so confirm they fill 55s</t>
+          <t>silent - no MOQ published. Only a 'Request a Sample' form.</t>
         </is>
       </c>
       <c r="G67" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001 + ISO 14001 + OHSAS 18001 + NACD Responsible Distribution; lab with titration, AA, ICP</t>
+          <t>none found on the US site. (Parent Mitsubishi Chemical publishes a GOHSENOL EG pharmaceutical-excipient grade on m-chemical.co.jp, which im…</t>
         </is>
       </c>
       <c r="H67" s="23" t="inlineStr">
         <is>
-          <t>mileschemical.com contact page | 818-504-3355 | cs@mileschemical.com</t>
+          <t>https://us.mitsubishi-chemical.com/contact/ (web form) plus a per-product 'Request a Sample' form on the GOHSENX/GOHSENOL page. No phone number published anywh…</t>
         </is>
       </c>
       <c r="I67" s="23" t="inlineStr">
         <is>
-          <t>A distributor that blends, so they already think in conversion-fee terms, and the certification stack plus in-house lab covers the CoA and traceability ask. Two blanks to clear: heat, and whether they fill 55-gal drums.</t>
+          <t>CORRECTION: none on the facts as listed (no location was claimed, so nothing to contradict). GOHSENOL/GOHSENX PVA is genuinely on their US product catalog at us.mitsubishi-chemical.com/product/gohsenx-and-gohsenol/. IMPORTANT ROLE …  |  keep - correct C role as an alternate resin source only. Useful as a second resin supply line and, like Kuraray, as a source of toll-blender referrals. Never a blending candidate.</t>
         </is>
       </c>
       <c r="J67" s="25" t="inlineStr">
@@ -4550,47 +4594,47 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>Mitsubishi Chemical America (Gohsenol)</t>
+          <t>MonoSol (Kuraray)</t>
         </is>
       </c>
       <c r="C68" s="23" t="inlineStr">
         <is>
-          <t>US sales office only (no US plant)</t>
+          <t>Merrillville, IN</t>
         </is>
       </c>
       <c r="D68" s="24" t="inlineStr">
         <is>
-          <t>https://us.mitsubishi-chemical.com</t>
+          <t>https://www.monosol.com</t>
         </is>
       </c>
       <c r="E68" s="23" t="inlineStr">
         <is>
-          <t>silent - no vessels, reactors, or temperature stated anywhere. Not applicable to their role.</t>
+          <t>silent - no vessel, jacket, reactor or temperature information anywhere on monosol.com. Do not infer heat capability from the fact that they cast film.</t>
         </is>
       </c>
       <c r="F68" s="23" t="inlineStr">
         <is>
-          <t>silent - no MOQ published. Only a 'Request a Sample' form.</t>
+          <t>silent - no MOQ or minimum batch published. Their business model is continuous film casting lines, which is a structural mismatch with a 450 lb weekly batch.</t>
         </is>
       </c>
       <c r="G68" s="23" t="inlineStr">
         <is>
-          <t>none found on the US site. (Parent Mitsubishi Chemical publishes a GOHSENOL EG pharmaceutical-excipient grade on m-chemical.co.jp, which im…</t>
+          <t>none found - no ISO 9001, ISO 13485, FDA registration, cGMP, or traceability language published on the site or the contact page.</t>
         </is>
       </c>
       <c r="H68" s="23" t="inlineStr">
         <is>
-          <t>https://us.mitsubishi-chemical.com/contact/ (web form) plus a per-product 'Request a Sample' form on the GOHSENX/GOHSENOL page. No phone number published anywh…</t>
+          <t>https://www.monosol.com/contact/ (structured web form). Phone +1 888 902 9951; corporate HQ +1 219 763 7589; fax +1 219 370 6448</t>
         </is>
       </c>
       <c r="I68" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: none on the facts as listed (no location was claimed, so nothing to contradict). GOHSENOL/GOHSENX PVA is genuinely on their US product catalog at us.mitsubishi-chemical.com/product/gohsenx-and-gohsenol/. IMPORTANT ROLE …  |  keep - correct C role as an alternate resin source only. Useful as a second resin supply line and, like Kuraray, as a source of toll-blender referrals. Never a blending candidate.</t>
+          <t>CORRECTION: LOCATION ERROR. Merrillville IN is the OLD headquarters (707 E 80th Pl, Suite 301). Current corporate HQ per monosol.com/locations is 1500 Louis Sullivan Drive, Portage, IN 46368. Plants: County Line Road Portage IN; Ge…  |  keep C, but low priority. They have the PVA dissolution know-how, but they are a continuous film converter with no published toll service, no published certifications, and recent lay…</t>
         </is>
       </c>
       <c r="J68" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -4602,47 +4646,47 @@
       </c>
       <c r="B69" s="23" t="inlineStr">
         <is>
-          <t>MonoSol (Kuraray)</t>
+          <t>NEXT Medical Products Company  [NEW]</t>
         </is>
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>Merrillville, IN</t>
+          <t>45 Columbia Road, Branchburg, NJ 08876</t>
         </is>
       </c>
       <c r="D69" s="24" t="inlineStr">
         <is>
-          <t>https://www.monosol.com</t>
+          <t>https://nextmedicalproducts.com/about/</t>
         </is>
       </c>
       <c r="E69" s="23" t="inlineStr">
         <is>
-          <t>silent - no vessel, jacket, reactor or temperature information anywhere on monosol.com. Do not infer heat capability from the fact that they cast film.</t>
+          <t>SILENT. No process temperature, kettle size, or jacket capability published anywhere on the site. Ultrasound gel manufacture commonly uses heated jacketed mixers for polymer hydration, so capability is plausible - but this is INFERENCE ONLY and 90-95 C is UNV…</t>
         </is>
       </c>
       <c r="F69" s="23" t="inlineStr">
         <is>
-          <t>silent - no MOQ or minimum batch published. Their business model is continuous film casting lines, which is a structural mismatch with a 450 lb weekly batch.</t>
+          <t>Plausible - they market both single-use and bulk gel formats and are a mid-size specialist. Specific batch minimums and 55-gal drum filling are SILENT.</t>
         </is>
       </c>
       <c r="G69" s="23" t="inlineStr">
         <is>
-          <t>none found - no ISO 9001, ISO 13485, FDA registration, cGMP, or traceability language published on the site or the contact page.</t>
+          <t>ISO 13485:2016 certified; FDA registered; Health Canada registered; UDI compliant; WBENC certified (may matter for supplier-diversity credi…</t>
         </is>
       </c>
       <c r="H69" s="23" t="inlineStr">
         <is>
-          <t>https://www.monosol.com/contact/ (structured web form). Phone +1 888 902 9951; corporate HQ +1 219 763 7589; fax +1 219 370 6448</t>
+          <t>nextmedicalproducts.com/contact/ - see their OEM Capability page and request an OEM/custom manufacturing discussion</t>
         </is>
       </c>
       <c r="I69" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: LOCATION ERROR. Merrillville IN is the OLD headquarters (707 E 80th Pl, Suite 301). Current corporate HQ per monosol.com/locations is 1500 Louis Sullivan Drive, Portage, IN 46368. Plants: County Line Road Portage IN; Ge…  |  keep C, but low priority. They have the PVA dissolution know-how, but they are a continuous film converter with no published toll service, no published certifications, and recent lay…</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Manufactures aqueous water-soluble-polymer gels (Clear Image brand, plus the former Sonotech gel business acquired from Magnaflux in 2012) at their New Jersey plant under ISO 13485:2016 and FDA registration - and the site explicitly states…</t>
         </is>
       </c>
       <c r="J69" s="25" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>MEDIUM-HIGH on quality …</t>
         </is>
       </c>
     </row>
@@ -4654,47 +4698,43 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>NEXT Medical Products Company  [NEW]</t>
+          <t>Nation Ford Chemical</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
         <is>
-          <t>45 Columbia Road, Branchburg, NJ 08876</t>
-        </is>
-      </c>
-      <c r="D70" s="24" t="inlineStr">
-        <is>
-          <t>https://nextmedicalproducts.com/about/</t>
-        </is>
-      </c>
+          <t>Fort Mill, SC</t>
+        </is>
+      </c>
+      <c r="D70" s="23" t="inlineStr"/>
       <c r="E70" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No process temperature, kettle size, or jacket capability published anywhere on the site. Ultrasound gel manufacture commonly uses heated jacketed mixers for polymer hydration, so capability is plausible - but this is INFERENCE ONLY and 90-95 C is UNV…</t>
+          <t>NOT DIRECTLY QUOTED (site 403-blocked). Inferable-but-unconfirmed: nitration, hydrogenation and distillation operations necessarily run well above 95 C. Per the audit rule I am NOT scoring this as a documented pass — no published temperature statement was obt…</t>
         </is>
       </c>
       <c r="F70" s="23" t="inlineStr">
         <is>
-          <t>Plausible - they market both single-use and bulk gel formats and are a mid-size specialist. Specific batch minimums and 55-gal drum filling are SILENT.</t>
+          <t>POOR FIT. Reactor fleet: three 6,000 gal Hastelloy, one 6,000 gal Furan, seven 2,000 gal glass-lined, 'and various other sizes and types of reactors ranging fr…</t>
         </is>
       </c>
       <c r="G70" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified; FDA registered; Health Canada registered; UDI compliant; WBENC certified (may matter for supplier-diversity credi…</t>
+          <t>ISO 9001 certified (privately owned, ISO-9001 certified custom manufacturer of organic chemicals). SOCMA recognition for safety performance…</t>
         </is>
       </c>
       <c r="H70" s="23" t="inlineStr">
         <is>
-          <t>nextmedicalproducts.com/contact/ - see their OEM Capability page and request an OEM/custom manufacturing discussion</t>
+          <t>https://nationfordchem.com/contact/ (site 403s to automated tools — open in a browser). No phone number could be confirmed from the site itself due to the bloc…</t>
         </is>
       </c>
       <c r="I70" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Manufactures aqueous water-soluble-polymer gels (Clear Image brand, plus the former Sonotech gel business acquired from Magnaflux in 2012) at their New Jersey plant under ISO 13485:2016 and FDA registration - and the site explicitly states…</t>
+          <t>CORRECTION: Location correct (Fort Mill SC). The capability framing is the problem: this is a heavy custom ORGANIC SYNTHESIS house — polymerization, nitration, sulfonation, hydrogenation, alkylation, distillation, flaking, crystall…  |  MOVE B → C. Wrong shop type and wrong scale: hazardous-synthesis capability (aniline, nitration, hydrogenation) in Hastelloy and glass-lined reactors, minimum 750 gal. Running a simp…</t>
         </is>
       </c>
       <c r="J70" s="25" t="inlineStr">
         <is>
-          <t>MEDIUM-HIGH on quality …</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -4706,43 +4746,47 @@
       </c>
       <c r="B71" s="23" t="inlineStr">
         <is>
-          <t>Nation Ford Chemical</t>
+          <t>Nelson Brothers Specialty Chemicals  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C71" s="23" t="inlineStr">
         <is>
-          <t>Fort Mill, SC</t>
-        </is>
-      </c>
-      <c r="D71" s="23" t="inlineStr"/>
+          <t>Parrish, AL</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>https://www.nbspecchem.com/services/toll-manufacturing/</t>
+        </is>
+      </c>
       <c r="E71" s="23" t="inlineStr">
         <is>
-          <t>NOT DIRECTLY QUOTED (site 403-blocked). Inferable-but-unconfirmed: nitration, hydrogenation and distillation operations necessarily run well above 95 C. Per the audit rule I am NOT scoring this as a documented pass — no published temperature statement was obt…</t>
+          <t>SILENT — only 'multiple reaction vessels which provide a high degree of manufacturing flexibility'</t>
         </is>
       </c>
       <c r="F71" s="23" t="inlineStr">
         <is>
-          <t>POOR FIT. Reactor fleet: three 6,000 gal Hastelloy, one 6,000 gal Furan, seven 2,000 gal glass-lined, 'and various other sizes and types of reactors ranging fr…</t>
+          <t>'whether you need one drum or a rail car of product' — an unusually explicit welcome for small orders</t>
         </is>
       </c>
       <c r="G71" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001 certified (privately owned, ISO-9001 certified custom manufacturer of organic chemicals). SOCMA recognition for safety performance…</t>
+          <t>No ISO stated</t>
         </is>
       </c>
       <c r="H71" s="23" t="inlineStr">
         <is>
-          <t>https://nationfordchem.com/contact/ (site 403s to automated tools — open in a browser). No phone number could be confirmed from the site itself due to the bloc…</t>
+          <t>nbspecchem.com/rfq | 866-753-6902</t>
         </is>
       </c>
       <c r="I71" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: Location correct (Fort Mill SC). The capability framing is the problem: this is a heavy custom ORGANIC SYNTHESIS house — polymerization, nitration, sulfonation, hydrogenation, alkylation, distillation, flaking, crystall…  |  MOVE B → C. Wrong shop type and wrong scale: hazardous-synthesis capability (aniline, nitration, hydrogenation) in Hastelloy and glass-lined reactors, minimum 750 gal. Running a simp…</t>
+          <t>'One drum' language is rare and worth testing. Their emulsifier business implies real reaction vessels. Everything else needs verifying.</t>
         </is>
       </c>
       <c r="J71" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>M-L</t>
         </is>
       </c>
     </row>
@@ -4754,47 +4798,47 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>Nelson Brothers Specialty Chemicals  [NATIONWIDE]</t>
+          <t>Northstar Chemical</t>
         </is>
       </c>
       <c r="C72" s="23" t="inlineStr">
         <is>
-          <t>Parrish, AL</t>
+          <t>Charlotte NC</t>
         </is>
       </c>
       <c r="D72" s="24" t="inlineStr">
         <is>
-          <t>https://www.nbspecchem.com/services/toll-manufacturing/</t>
+          <t>https://www.northstarchemical.com</t>
         </is>
       </c>
       <c r="E72" s="23" t="inlineStr">
         <is>
-          <t>SILENT — only 'multiple reaction vessels which provide a high degree of manufacturing flexibility'</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="F72" s="23" t="inlineStr">
         <is>
-          <t>'whether you need one drum or a rail car of product' — an unusually explicit welcome for small orders</t>
+          <t>Unknown (small custom/toll)</t>
         </is>
       </c>
       <c r="G72" s="23" t="inlineStr">
         <is>
-          <t>No ISO stated</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="H72" s="23" t="inlineStr">
         <is>
-          <t>nbspecchem.com/rfq | 866-753-6902</t>
+          <t>(800) 570-0204</t>
         </is>
       </c>
       <c r="I72" s="23" t="inlineStr">
         <is>
-          <t>'One drum' language is rare and worth testing. Their emulsifier business implies real reaction vessels. Everything else needs verifying.</t>
+          <t>ON OUR ROSTER as backup. Smaller dry-to-liquid custom/toll blender — verify.</t>
         </is>
       </c>
       <c r="J72" s="25" t="inlineStr">
         <is>
-          <t>M-L</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -4806,42 +4850,42 @@
       </c>
       <c r="B73" s="23" t="inlineStr">
         <is>
-          <t>Northstar Chemical</t>
+          <t>PCI Manufacturing  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C73" s="23" t="inlineStr">
         <is>
-          <t>Charlotte NC</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>https://www.northstarchemical.com</t>
+          <t>https://pcistl.com/</t>
         </is>
       </c>
       <c r="E73" s="23" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="F73" s="23" t="inlineStr">
         <is>
-          <t>Unknown (small custom/toll)</t>
+          <t>'batch sizes ranging from 100 to 3,000 gallons' — an honest published floor at 2x our batch, where most competitors publish nothing</t>
         </is>
       </c>
       <c r="G73" s="23" t="inlineStr">
         <is>
-          <t>Not published</t>
+          <t>No ISO claimed; 'documented quality systems, batch tracking, SOP-driven processes'</t>
         </is>
       </c>
       <c r="H73" s="23" t="inlineStr">
         <is>
-          <t>(800) 570-0204</t>
+          <t>pcistl.com/start-your-quote | 314-872-9333 | sales@pcistl.com</t>
         </is>
       </c>
       <c r="I73" s="23" t="inlineStr">
         <is>
-          <t>ON OUR ROSTER as backup. Smaller dry-to-liquid custom/toll blender — verify.</t>
+          <t>Publishes a real minimum close to our size and advertises 'viscosity-flexible liquid filling', which says they handle syrupy material. Two unknowns: heat, and no ISO certificate.</t>
         </is>
       </c>
       <c r="J73" s="25" t="inlineStr">
@@ -4858,47 +4902,47 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>PCI Manufacturing  [NATIONWIDE]</t>
+          <t>Polysciences, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C74" s="23" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>400 Valley Road, Warrington, PA 18976</t>
         </is>
       </c>
       <c r="D74" s="24" t="inlineStr">
         <is>
-          <t>https://pcistl.com/</t>
+          <t>https://www.polysciences.com/default/contract-manufacturing-capabilities/</t>
         </is>
       </c>
       <c r="E74" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>SILENT. The site does not publish reactor sizes, vessel types, jacket capability, or max process temperature. They do state they handle flammable/hazardous materials, which implies real jacketed/temperature-controlled process vessels, but 90-95 C hold capabil…</t>
         </is>
       </c>
       <c r="F74" s="23" t="inlineStr">
         <is>
-          <t>'batch sizes ranging from 100 to 3,000 gallons' — an honest published floor at 2x our batch, where most competitors publish nothing</t>
+          <t>Strong. Custom synthesis described as scaling from gram to multi-kilogram; pilot AND commercial scale offered. A ~450 lb weekly batch is comfortably within a s…</t>
         </is>
       </c>
       <c r="G74" s="23" t="inlineStr">
         <is>
-          <t>No ISO claimed; 'documented quality systems, batch tracking, SOP-driven processes'</t>
+          <t>ISO 13485:2016 certified QMS; FDA Establishment Registration (21 CFR 820); GMP-aligned manufacturing; ISO Class 7 and Class 8 cleanrooms</t>
         </is>
       </c>
       <c r="H74" s="23" t="inlineStr">
         <is>
-          <t>pcistl.com/start-your-quote | 314-872-9333 | sales@pcistl.com</t>
+          <t>Phone (800) 523-2575 or (215) 343-6484; info@polysciences.com. Ask for the Contract Manufacturing / Custom Synthesis group.</t>
         </is>
       </c>
       <c r="I74" s="23" t="inlineStr">
         <is>
-          <t>Publishes a real minimum close to our size and advertises 'viscosity-flexible liquid filling', which says they handle syrupy material. Two unknowns: heat, and no ISO certificate.</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Best combined fit on the list: a genuine polymer chemistry manufacturer that ALSO carries ISO 13485:2016 + FDA establishment registration. Their contract manufacturing page explicitly lists 'blending and filling of liquids, powders, slurri…</t>
         </is>
       </c>
       <c r="J74" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>HIGH on quality credent…</t>
         </is>
       </c>
     </row>
@@ -4910,47 +4954,47 @@
       </c>
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>Polysciences, Inc.  [NEW]</t>
+          <t>Polytek Development Corp.  [NEW]</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
         <is>
-          <t>400 Valley Road, Warrington, PA 18976</t>
+          <t>55 Hilton Street, Easton, PA 18042 (plus Pomona, CA; Kalamazoo, MI; Franklin, IN)</t>
         </is>
       </c>
       <c r="D75" s="24" t="inlineStr">
         <is>
-          <t>https://www.polysciences.com/default/contract-manufacturing-capabilities/</t>
+          <t>https://polytek.com/products/poly-pva-solution</t>
         </is>
       </c>
       <c r="E75" s="23" t="inlineStr">
         <is>
-          <t>SILENT. The site does not publish reactor sizes, vessel types, jacket capability, or max process temperature. They do state they handle flammable/hazardous materials, which implies real jacketed/temperature-controlled process vessels, but 90-95 C hold capabil…</t>
+          <t>NOT PUBLISHED and genuinely uncertain. Solvent-cut PVA release films do not require a 90-95 C hold, so they may not own the high-temperature cook at all. Treat the heat gate as unverified and ask early — this could disqualify them the way it disqualified ILC …</t>
         </is>
       </c>
       <c r="F75" s="23" t="inlineStr">
         <is>
-          <t>Strong. Custom synthesis described as scaling from gram to multi-kilogram; pilot AND commercial scale offered. A ~450 lb weekly batch is comfortably within a s…</t>
+          <t>LIKELY GOOD — their own PVA product ships in 2-lb and 35-lb units, so they run small lots. A 450-lb drum is a large batch by their standards, which cuts the ot…</t>
         </is>
       </c>
       <c r="G75" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified QMS; FDA Establishment Registration (21 CFR 820); GMP-aligned manufacturing; ISO Class 7 and Class 8 cleanrooms</t>
+          <t>Not published. Ask about ISO 9001 and CoA capability; they serve medical and food manufacturing per their industries list.</t>
         </is>
       </c>
       <c r="H75" s="23" t="inlineStr">
         <is>
-          <t>Phone (800) 523-2575 or (215) 343-6484; info@polysciences.com. Ask for the Contract Manufacturing / Custom Synthesis group.</t>
+          <t>Via polytek.com contact / corporation.polytek.com. Easton, PA HQ.</t>
         </is>
       </c>
       <c r="I75" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | Best combined fit on the list: a genuine polymer chemistry manufacturer that ALSO carries ISO 13485:2016 + FDA establishment registration. Their contract manufacturing page explicitly lists 'blending and filling of liquids, powders, slurri…</t>
+          <t>The only US manufacturer besides REXCO found that formulates and sells its OWN branded PVA solution product — 'Poly PVA Solution,' a water-soluble removable sealer and release agent for mold making and casting, sold in 2-lb and 35-lb units. Founded 1984, they are a genuine manufacturer (not a reseller) of specialty polymers across four US plants: liquid rubbers, plastics, resins, foams, release agents, elastomers, e…</t>
         </is>
       </c>
       <c r="J75" s="25" t="inlineStr">
         <is>
-          <t>HIGH on quality credent…</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4962,47 +5006,47 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>Polytek Development Corp.  [NEW]</t>
+          <t>RBP Chemical Technology, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C76" s="23" t="inlineStr">
         <is>
-          <t>55 Hilton Street, Easton, PA 18042 (plus Pomona, CA; Kalamazoo, MI; Franklin, IN)</t>
+          <t>150 S. 118th Street, Milwaukee, WI 53214</t>
         </is>
       </c>
       <c r="D76" s="24" t="inlineStr">
         <is>
-          <t>https://polytek.com/products/poly-pva-solution</t>
+          <t>https://rbpchemical.com/custom-chemical-blending-2/</t>
         </is>
       </c>
       <c r="E76" s="23" t="inlineStr">
         <is>
-          <t>NOT PUBLISHED and genuinely uncertain. Solvent-cut PVA release films do not require a 90-95 C hold, so they may not own the high-temperature cook at all. Treat the heat gate as unverified and ask early — this could disqualify them the way it disqualified ILC …</t>
+          <t>UNVERIFIED. Their custom blending page describes 'high-end, precision toll blending equipment including variable-speed mixing systems' but publishes NO vessel type, jacket, or temperature data. Must be asked directly.</t>
         </is>
       </c>
       <c r="F76" s="23" t="inlineStr">
         <is>
-          <t>LIKELY GOOD — their own PVA product ships in 2-lb and 35-lb units, so they run small lots. A 450-lb drum is a large batch by their standards, which cuts the ot…</t>
+          <t>Published packaging range 'from one quart to bulk truckload shipments' implies genuine small-volume flexibility; actual minimum batch size not published.</t>
         </is>
       </c>
       <c r="G76" s="23" t="inlineStr">
         <is>
-          <t>Not published. Ask about ISO 9001 and CoA capability; they serve medical and food manufacturing per their industries list.</t>
+          <t>ISO 9001 compliant, US and international facilities. One-year retained-sample policy.</t>
         </is>
       </c>
       <c r="H76" s="23" t="inlineStr">
         <is>
-          <t>Via polytek.com contact / corporation.polytek.com. Easton, PA HQ.</t>
+          <t>(414) 258-0911 or consultation request form on rbpchemical.com</t>
         </is>
       </c>
       <c r="I76" s="23" t="inlineStr">
         <is>
-          <t>The only US manufacturer besides REXCO found that formulates and sells its OWN branded PVA solution product — 'Poly PVA Solution,' a water-soluble removable sealer and release agent for mold making and casting, sold in 2-lb and 35-lb units. Founded 1984, they are a genuine manufacturer (not a reseller) of specialty polymers across four US plants: liquid rubbers, plastics, resins, foams, release agents, elastomers, e…</t>
+          <t>A Milwaukee technical toll blender whose day job is electronics/printed-circuit and printing chemistry - meaning tight spec control, not commodity drum mixing. Two things stand out for your application: they are ISO 9001 compliant, and they publish a product retention policy of holding samples for one year for quality verification, which is precisely the traceability behavior you want behind an Intuitive Surgical co…</t>
         </is>
       </c>
       <c r="J76" s="25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>High on realness, ISO a…</t>
         </is>
       </c>
     </row>
@@ -5014,47 +5058,47 @@
       </c>
       <c r="B77" s="23" t="inlineStr">
         <is>
-          <t>RBP Chemical Technology, Inc.  [NEW]</t>
+          <t>REXCO-USA (PARTALL)</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
         <is>
-          <t>150 S. 118th Street, Milwaukee, WI 53214</t>
+          <t>Conyers, GA</t>
         </is>
       </c>
       <c r="D77" s="24" t="inlineStr">
         <is>
-          <t>https://rbpchemical.com/custom-chemical-blending-2/</t>
+          <t>https://rexco-usa.com</t>
         </is>
       </c>
       <c r="E77" s="23" t="inlineStr">
         <is>
-          <t>UNVERIFIED. Their custom blending page describes 'high-end, precision toll blending equipment including variable-speed mixing systems' but publishes NO vessel type, jacket, or temperature data. Must be asked directly.</t>
+          <t>SILENT. No mention of vessels, jackets, heating, or temperature anywhere on the site - though the fact that they commercially produce PVA parting films means they almost certainly dissolve PVA with heat in-house. That is an inference, not a published claim.</t>
         </is>
       </c>
       <c r="F77" s="23" t="inlineStr">
         <is>
-          <t>Published packaging range 'from one quart to bulk truckload shipments' implies genuine small-volume flexibility; actual minimum batch size not published.</t>
+          <t>SILENT. No batch size or MOQ published.</t>
         </is>
       </c>
       <c r="G77" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001 compliant, US and international facilities. One-year retained-sample policy.</t>
+          <t>NONE FOUND - the weakest of the nine. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no lot traceability anywhere on the site.</t>
         </is>
       </c>
       <c r="H77" s="23" t="inlineStr">
         <is>
-          <t>(414) 258-0911 or consultation request form on rbpchemical.com</t>
+          <t>https://rexco-usa.com/contact-us/ | Toll free (800) 888-1060 | Direct +1-770-483-7610 | Fax +1-770-483-8550 | info@rexco-usa.com</t>
         </is>
       </c>
       <c r="I77" s="23" t="inlineStr">
         <is>
-          <t>A Milwaukee technical toll blender whose day job is electronics/printed-circuit and printing chemistry - meaning tight spec control, not commodity drum mixing. Two things stand out for your application: they are ISO 9001 compliant, and they publish a product retention policy of holding samples for one year for quality verification, which is precisely the traceability behavior you want behind an Intuitive Surgical co…</t>
+          <t>CORRECTION: MATERIAL ERROR - CATEGORY MISTAKE. REXCO is a branded product manufacturer, NOT a toll blender. Their site describes them as 'Manufacturer of simple, effective and economical mold release waxes, buffing compounds and pa…  |  MOVE A -&gt; C, reclassified as a technical resource / long-shot rather than a toll candidate. Nothing published supports toll manufacturing, heat capability, or any quality system. The…</t>
         </is>
       </c>
       <c r="J77" s="25" t="inlineStr">
         <is>
-          <t>High on realness, ISO a…</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -5066,47 +5110,47 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>REXCO-USA (PARTALL)</t>
+          <t>SNP Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C78" s="23" t="inlineStr">
         <is>
-          <t>Conyers, GA</t>
+          <t>1301 S. Briggs Ave., Durham, NC 27703</t>
         </is>
       </c>
       <c r="D78" s="24" t="inlineStr">
         <is>
-          <t>https://rexco-usa.com</t>
+          <t>https://www.snpinc.com/chemical-products-polymers/liquid/polyvinyl-alcohol/</t>
         </is>
       </c>
       <c r="E78" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No mention of vessels, jackets, heating, or temperature anywhere on the site - though the fact that they commercially produce PVA parting films means they almost certainly dissolve PVA with heat in-house. That is an inference, not a published claim.</t>
+          <t>NOT PUBLISHED — must be verified by phone. However, the entire premise of their PVA product line is doing the dissolution cook that customers cannot do, and super/fully-hydrolyzed PVOH cannot be dissolved below ~90 C, so a 90-95 C hold is implied by the produ…</t>
         </is>
       </c>
       <c r="F78" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No batch size or MOQ published.</t>
+          <t>STRONG. Company states 'Whether you need 5 gallons or 20,000 gallons of solution, SNP can provide it.' A ~50-gallon / 450-lb drum batch sits comfortably in tha…</t>
         </is>
       </c>
       <c r="G78" s="23" t="inlineStr">
         <is>
-          <t>NONE FOUND - the weakest of the nine. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no lot traceability anywhere on the site.</t>
+          <t>Not published on site. Must ask about ISO 9001, CoA content, lot traceability, and retained samples.</t>
         </is>
       </c>
       <c r="H78" s="23" t="inlineStr">
         <is>
-          <t>https://rexco-usa.com/contact-us/ | Toll free (800) 888-1060 | Direct +1-770-483-7610 | Fax +1-770-483-8550 | info@rexco-usa.com</t>
+          <t>(919) 598-0400 / service@snpinc.com — lead with 'we need a toll cook of an aqueous super-hydrolyzed PVOH solution, ~10-12% solids, one 450-lb drum per week, we…</t>
         </is>
       </c>
       <c r="I78" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: MATERIAL ERROR - CATEGORY MISTAKE. REXCO is a branded product manufacturer, NOT a toll blender. Their site describes them as 'Manufacturer of simple, effective and economical mold release waxes, buffing compounds and pa…  |  MOVE A -&gt; C, reclassified as a technical resource / long-shot rather than a toll candidate. Nothing published supports toll manufacturing, heat capability, or any quality system. The…</t>
+          <t>Closest match found in the entire US market. SNP is a custom LIQUID chemical manufacturer whose stated PVA business is exactly our process: they manufacture aqueous solutions of polyvinyl alcohol for customers who 'don't have the equipment to cook the dry product into an aqueous solution' or don't want to disrupt their own process to do it. They span the full range of molecular weight and degree of hydrolysis, which…</t>
         </is>
       </c>
       <c r="J78" s="25" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -5118,47 +5162,47 @@
       </c>
       <c r="B79" s="23" t="inlineStr">
         <is>
-          <t>SNP Inc.  [NEW]</t>
+          <t>Sanco Industries  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
         <is>
-          <t>1301 S. Briggs Ave., Durham, NC 27703</t>
+          <t>Fort Wayne, IN</t>
         </is>
       </c>
       <c r="D79" s="24" t="inlineStr">
         <is>
-          <t>https://www.snpinc.com/chemical-products-polymers/liquid/polyvinyl-alcohol/</t>
+          <t>https://www.sancoind.com/en/toll-blending</t>
         </is>
       </c>
       <c r="E79" s="23" t="inlineStr">
         <is>
-          <t>NOT PUBLISHED — must be verified by phone. However, the entire premise of their PVA product line is doing the dissolution cook that customers cannot do, and super/fully-hydrolyzed PVOH cannot be dissolved below ~90 C, so a 90-95 C hold is implied by the produ…</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="F79" s="23" t="inlineStr">
         <is>
-          <t>STRONG. Company states 'Whether you need 5 gallons or 20,000 gallons of solution, SNP can provide it.' A ~50-gallon / 450-lb drum batch sits comfortably in tha…</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="G79" s="23" t="inlineStr">
         <is>
-          <t>Not published on site. Must ask about ISO 9001, CoA content, lot traceability, and retained samples.</t>
+          <t>SILENT</t>
         </is>
       </c>
       <c r="H79" s="23" t="inlineStr">
         <is>
-          <t>(919) 598-0400 / service@snpinc.com — lead with 'we need a toll cook of an aqueous super-hydrolyzed PVOH solution, ~10-12% solids, one 450-lb drum per week, we…</t>
+          <t>sancoind.com/en/contact-us | 260-426-6281</t>
         </is>
       </c>
       <c r="I79" s="23" t="inlineStr">
         <is>
-          <t>Closest match found in the entire US market. SNP is a custom LIQUID chemical manufacturer whose stated PVA business is exactly our process: they manufacture aqueous solutions of polyvinyl alcohol for customers who 'don't have the equipment to cook the dry product into an aqueous solution' or don't want to disrupt their own process to do it. They span the full range of molecular weight and degree of hydrolysis, which…</t>
+          <t>Describes our exact business model in one sentence: 'Our Biologist and Chemist can take your formula, raw materials, and packaging and turn it into a finished product, ready for shipping.' Cheapest possible qualifying call; both gates completely unverified.</t>
         </is>
       </c>
       <c r="J79" s="25" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>M-L</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5214,17 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>Sanco Industries  [NATIONWIDE]</t>
+          <t>Sky Blue Chemical  [NATIONWIDE]</t>
         </is>
       </c>
       <c r="C80" s="23" t="inlineStr">
         <is>
-          <t>Fort Wayne, IN</t>
+          <t>Ogden, UT</t>
         </is>
       </c>
       <c r="D80" s="24" t="inlineStr">
         <is>
-          <t>https://www.sancoind.com/en/toll-blending</t>
+          <t>https://www.skybluechemical.com/services</t>
         </is>
       </c>
       <c r="E80" s="23" t="inlineStr">
@@ -5195,17 +5239,17 @@
       </c>
       <c r="G80" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>SILENT (third-party profiles mention pursuing ISO 9001:2015 — unverified)</t>
         </is>
       </c>
       <c r="H80" s="23" t="inlineStr">
         <is>
-          <t>sancoind.com/en/contact-us | 260-426-6281</t>
+          <t>skybluechemical.com/request-a-quote | 801-394-8611 | cs@skybluechemical.com</t>
         </is>
       </c>
       <c r="I80" s="23" t="inlineStr">
         <is>
-          <t>Describes our exact business model in one sentence: 'Our Biologist and Chemist can take your formula, raw materials, and packaging and turn it into a finished product, ready for shipping.' Cheapest possible qualifying call; both gates completely unverified.</t>
+          <t>An 11-50 person family shop since 1963 — the size profile that quotes $0.75-1.50/lb rather than $8. Also the only real toll blender verifiable in Utah. Everything technical is unverified.</t>
         </is>
       </c>
       <c r="J80" s="25" t="inlineStr">
@@ -5222,47 +5266,47 @@
       </c>
       <c r="B81" s="23" t="inlineStr">
         <is>
-          <t>Sky Blue Chemical  [NATIONWIDE]</t>
+          <t>Southern Chemical &amp; Textiles</t>
         </is>
       </c>
       <c r="C81" s="23" t="inlineStr">
         <is>
-          <t>Ogden, UT</t>
+          <t>Dalton, GA</t>
         </is>
       </c>
       <c r="D81" s="24" t="inlineStr">
         <is>
-          <t>https://www.skybluechemical.com/services</t>
+          <t>https://www.southern-chemical.com</t>
         </is>
       </c>
       <c r="E81" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>silent - I found NO mention of reactors, jacketed vessels, heating, steam, or any maximum temperature on southern-chemical.com. Surfactant manufacturers commonly run jacketed reactors, but that is an inference and the site does not say it - treat as unknown u…</t>
         </is>
       </c>
       <c r="F81" s="23" t="inlineStr">
         <is>
-          <t>SILENT</t>
+          <t>silent - no minimum batch size or MOQ published anywhere on the site.</t>
         </is>
       </c>
       <c r="G81" s="23" t="inlineStr">
         <is>
-          <t>SILENT (third-party profiles mention pursuing ISO 9001:2015 — unverified)</t>
+          <t>none found - no ISO 9001, no ISO 13485, no FDA registration, no cGMP, and no lot-traceability statement published on the site or the contac…</t>
         </is>
       </c>
       <c r="H81" s="23" t="inlineStr">
         <is>
-          <t>skybluechemical.com/request-a-quote | 801-394-8611 | cs@skybluechemical.com</t>
+          <t>https://southern-chemical.com/contact-us/ (web form, routed by sales / customer service / regulatory) - Phone 706-277-3993, Fax 706-277-2966. Hours Mon-Fri 8:0…</t>
         </is>
       </c>
       <c r="I81" s="23" t="inlineStr">
         <is>
-          <t>An 11-50 person family shop since 1963 — the size profile that quotes $0.75-1.50/lb rather than $8. Also the only real toll blender verifiable in Utah. Everything technical is unverified.</t>
+          <t>CORRECTION: Dalton GA is CORRECT, and they have real manufacturing there, not just an office: HQ 1407 Abutment Road, Dalton GA 30721; MANUFACTURING at 653 Peek Road, Dalton GA 30721; plus an R&amp;D/Innovation lab at 11 Deerpark Dr #10…  |  keep C, promotable to B on two answers. What is verified is encouraging: a real owned manufacturing plant in Dalton, an in-house R&amp;D lab, and a company small enough that a weekly 450…</t>
         </is>
       </c>
       <c r="J81" s="25" t="inlineStr">
         <is>
-          <t>M-L</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -5274,42 +5318,42 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>Southern Chemical &amp; Textiles</t>
+          <t>Spectra Colorants (Union, SC)</t>
         </is>
       </c>
       <c r="C82" s="23" t="inlineStr">
         <is>
-          <t>Dalton, GA</t>
+          <t>Union, SC</t>
         </is>
       </c>
       <c r="D82" s="24" t="inlineStr">
         <is>
-          <t>https://www.southern-chemical.com</t>
+          <t>https://spectracolorants.com</t>
         </is>
       </c>
       <c r="E82" s="23" t="inlineStr">
         <is>
-          <t>silent - I found NO mention of reactors, jacketed vessels, heating, steam, or any maximum temperature on southern-chemical.com. Surfactant manufacturers commonly run jacketed reactors, but that is an inference and the site does not say it - treat as unknown u…</t>
+          <t>SILENT. No mention of heated, jacketed or steam vessels, no temperature specification, no equipment detail published. Heat gate UNKNOWN, with no product-mix reason to expect 90-95 C capability.</t>
         </is>
       </c>
       <c r="F82" s="23" t="inlineStr">
         <is>
-          <t>silent - no minimum batch size or MOQ published anywhere on the site.</t>
+          <t>SILENT. No batch size, no minimum, no MOQ published anywhere on the site.</t>
         </is>
       </c>
       <c r="G82" s="23" t="inlineStr">
         <is>
-          <t>none found - no ISO 9001, no ISO 13485, no FDA registration, no cGMP, and no lot-traceability statement published on the site or the contac…</t>
+          <t>NONE FOUND. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no traceability or CoA language. They do reference "regulatory complia…</t>
         </is>
       </c>
       <c r="H82" s="23" t="inlineStr">
         <is>
-          <t>https://southern-chemical.com/contact-us/ (web form, routed by sales / customer service / regulatory) - Phone 706-277-3993, Fax 706-277-2966. Hours Mon-Fri 8:0…</t>
+          <t>https://spectracolorants.com/contact/ | customerservice@spectracolorants.com | NO PHONE NUMBER IS PUBLISHED ANYWHERE ON THE SITE — email-only outreach, which i…</t>
         </is>
       </c>
       <c r="I82" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: Dalton GA is CORRECT, and they have real manufacturing there, not just an office: HQ 1407 Abutment Road, Dalton GA 30721; MANUFACTURING at 653 Peek Road, Dalton GA 30721; plus an R&amp;D/Innovation lab at 11 Deerpark Dr #10…  |  keep C, promotable to B on two answers. What is verified is encouraging: a real owned manufacturing plant in Dalton, an in-house R&amp;D lab, and a company small enough that a weekly 450…</t>
+          <t>CORRECTION: MISCATEGORIZED IN THE LONGLIST, same error as Spectrachem. Address is correct (228 Industrial Park Rd, Union, SC 29379), but Spectra Colorants is a manufacturer of water-based PIGMENT DISPERSIONS for the ink, coating, t…  |  MOVE DOWN from B to C, with a REDEFINED ROLE identical to Spectrachem. Not a viable toll blender for the PVA solution: wrong equipment class, no heat evidence, no published batch cap…</t>
         </is>
       </c>
       <c r="J82" s="25" t="inlineStr">
@@ -5326,42 +5370,42 @@
       </c>
       <c r="B83" s="23" t="inlineStr">
         <is>
-          <t>Spectra Colorants (Union, SC)</t>
+          <t>Spectrachem (Lodi, NJ)</t>
         </is>
       </c>
       <c r="C83" s="23" t="inlineStr">
         <is>
-          <t>Union, SC</t>
+          <t>Lodi, NJ</t>
         </is>
       </c>
       <c r="D83" s="24" t="inlineStr">
         <is>
-          <t>https://spectracolorants.com</t>
+          <t>https://spectrachem.net</t>
         </is>
       </c>
       <c r="E83" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No mention of heated, jacketed or steam vessels, no temperature specification, no equipment detail published. Heat gate UNKNOWN, with no product-mix reason to expect 90-95 C capability.</t>
+          <t>SILENT. No mention of heated, jacketed or steam vessels, no temperature specification, no equipment detail of any kind on the site. Heat gate UNKNOWN, and there is no product-mix reason to expect 90-95 C hold capability — pigment dispersion is a milling/dispe…</t>
         </is>
       </c>
       <c r="F83" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No batch size, no minimum, no MOQ published anywhere on the site.</t>
+          <t>"short run orders made to customer requirements" — genuinely small-run friendly in intent, but NO number, NO minimum batch, NO MOQ published.</t>
         </is>
       </c>
       <c r="G83" s="23" t="inlineStr">
         <is>
-          <t>NONE FOUND. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no traceability or CoA language. They do reference "regulatory complia…</t>
+          <t>NONE FOUND. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no lot-traceability or CoA language. Site emphasizes "R&amp;D, strict Qual…</t>
         </is>
       </c>
       <c r="H83" s="23" t="inlineStr">
         <is>
-          <t>https://spectracolorants.com/contact/ | customerservice@spectracolorants.com | NO PHONE NUMBER IS PUBLISHED ANYWHERE ON THE SITE — email-only outreach, which i…</t>
+          <t>https://spectrachem.net (contact/about pages) | 973-253-3553 | sales@spectrachem.net</t>
         </is>
       </c>
       <c r="I83" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: MISCATEGORIZED IN THE LONGLIST, same error as Spectrachem. Address is correct (228 Industrial Park Rd, Union, SC 29379), but Spectra Colorants is a manufacturer of water-based PIGMENT DISPERSIONS for the ink, coating, t…  |  MOVE DOWN from B to C, with a REDEFINED ROLE identical to Spectrachem. Not a viable toll blender for the PVA solution: wrong equipment class, no heat evidence, no published batch cap…</t>
+          <t>CORRECTION: MISCATEGORIZED IN THE LONGLIST. Spectrachem is NOT a general-purpose toll blender. Address is correct (10 Dell Glen Avenue, Lodi, NJ 07644), but their actual business is manufacturing water-based PIGMENT DISPERSIONS, aq…  |  MOVE DOWN from B to C, with a REDEFINED ROLE. They are not a candidate to toll-blend the PVA solution — wrong equipment class, no heat evidence, no quality certifications. They ARE, …</t>
         </is>
       </c>
       <c r="J83" s="25" t="inlineStr">
@@ -5378,42 +5422,42 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>Spectrachem (Lodi, NJ)</t>
+          <t>Stoner Molding Solutions</t>
         </is>
       </c>
       <c r="C84" s="23" t="inlineStr">
         <is>
-          <t>Lodi, NJ</t>
+          <t>Quarryville, PA</t>
         </is>
       </c>
       <c r="D84" s="24" t="inlineStr">
         <is>
-          <t>https://spectrachem.net</t>
+          <t>https://www.stonermolding.com</t>
         </is>
       </c>
       <c r="E84" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No mention of heated, jacketed or steam vessels, no temperature specification, no equipment detail of any kind on the site. Heat gate UNKNOWN, and there is no product-mix reason to expect 90-95 C hold capability — pigment dispersion is a milling/dispe…</t>
+          <t>silent - I found NO mention of heated vessels, jacketed kettles, reactors, or any maximum process temperature on stonermolding.com. This is the single unanswered question that decides their tier.</t>
         </is>
       </c>
       <c r="F84" s="23" t="inlineStr">
         <is>
-          <t>"short run orders made to customer requirements" — genuinely small-run friendly in intent, but NO number, NO minimum batch, NO MOQ published.</t>
+          <t>silent on a stated MOQ, but there is a genuine POSITIVE signal: third-party profiles describe Stoner as running 'lean manufacturing, which translates into shor…</t>
         </is>
       </c>
       <c r="G84" s="23" t="inlineStr">
         <is>
-          <t>NONE FOUND. No ISO 9001, no ISO 13485, no FDA registration, no cGMP, no lot-traceability or CoA language. Site emphasizes "R&amp;D, strict Qual…</t>
+          <t>ISO 9001 certified (badge on site footer; also confirmed in third-party listings for Stoner Molding Solutions). No ISO 13485, no FDA regist…</t>
         </is>
       </c>
       <c r="H84" s="23" t="inlineStr">
         <is>
-          <t>https://spectrachem.net (contact/about pages) | 973-253-3553 | sales@spectrachem.net</t>
+          <t>https://stonermolding.com/contact-us - Phone 1-800-227-5538 (US toll-free) or +1-717-786-7355. Hours Mon-Fri 8:00-5:00 EST.</t>
         </is>
       </c>
       <c r="I84" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: MISCATEGORIZED IN THE LONGLIST. Spectrachem is NOT a general-purpose toll blender. Address is correct (10 Dell Glen Avenue, Lodi, NJ 07644), but their actual business is manufacturing water-based PIGMENT DISPERSIONS, aq…  |  MOVE DOWN from B to C, with a REDEFINED ROLE. They are not a candidate to toll-blend the PVA solution — wrong equipment class, no heat evidence, no quality certifications. They ARE, …</t>
+          <t>CORRECTION: none. Quarryville PA confirmed: 1070 Robert Fulton Hwy, PO Box 65, Quarryville PA 17566. Manufacturing since 1942. One nuance: the site offers CUSTOM FORMULATION ('If we don't already offer a product that suits your bus…  |  keep C for now, but PROMOTE TO B immediately if they confirm a jacketed/heated vessel that reaches and holds 90-95 C. The rest of the profile fits unusually well for a Tier C name: I…</t>
         </is>
       </c>
       <c r="J84" s="25" t="inlineStr">
@@ -5430,47 +5474,47 @@
       </c>
       <c r="B85" s="23" t="inlineStr">
         <is>
-          <t>Stoner Molding Solutions</t>
+          <t>Strukmyer, LLC (Strukmyer Labs)  [NEW]</t>
         </is>
       </c>
       <c r="C85" s="23" t="inlineStr">
         <is>
-          <t>Quarryville, PA</t>
+          <t>Dallas / Lewisville, TX (DFW metro)</t>
         </is>
       </c>
       <c r="D85" s="24" t="inlineStr">
         <is>
-          <t>https://www.stonermolding.com</t>
+          <t>https://strukmyer.com/filling-compounding/medical-devices/</t>
         </is>
       </c>
       <c r="E85" s="23" t="inlineStr">
         <is>
-          <t>silent - I found NO mention of heated vessels, jacketed kettles, reactors, or any maximum process temperature on stonermolding.com. This is the single unanswered question that decides their tier.</t>
+          <t>SILENT. No published kettle temperature ceiling or jacketed-vessel specification. Hydrogel casting and cream/lotion compounding both normally require heated vessels, so the capability is plausible, but 90-95 C hold is UNVERIFIED.</t>
         </is>
       </c>
       <c r="F85" s="23" t="inlineStr">
         <is>
-          <t>silent on a stated MOQ, but there is a genuine POSITIVE signal: third-party profiles describe Stoner as running 'lean manufacturing, which translates into shor…</t>
+          <t>Plausible. A 503B-registered compounder is structurally set up for small, frequent, made-to-order lots with short dating - which is exactly your 1-drum-per-wee…</t>
         </is>
       </c>
       <c r="G85" s="23" t="inlineStr">
         <is>
-          <t>ISO 9001 certified (badge on site footer; also confirmed in third-party listings for Stoner Molding Solutions). No ISO 13485, no FDA regist…</t>
+          <t>ISO 13485:2016 certified; FDA registered for drug and device manufacturing; cGMP compliant; DEA and FDA registered 503B outsourcing facilit…</t>
         </is>
       </c>
       <c r="H85" s="23" t="inlineStr">
         <is>
-          <t>https://stonermolding.com/contact-us - Phone 1-800-227-5538 (US toll-free) or +1-717-786-7355. Hours Mon-Fri 8:00-5:00 EST.</t>
+          <t>Contact form at strukmyer.com; request the contract filling and compounding team</t>
         </is>
       </c>
       <c r="I85" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: none. Quarryville PA confirmed: 1070 Robert Fulton Hwy, PO Box 65, Quarryville PA 17566. Manufacturing since 1942. One nuance: the site offers CUSTOM FORMULATION ('If we don't already offer a product that suits your bus…  |  keep C for now, but PROMOTE TO B immediately if they confirm a jacketed/heated vessel that reaches and holds 90-95 C. The rest of the profile fits unusually well for a Tier C name: I…</t>
+          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | One of the few US contract manufacturers that stacks ISO 13485:2016, FDA drug AND device registration, cGMP, and 503B outsourcing-facility registration in one house, while its actual day-to-day work is compounding and filling liquids. They…</t>
         </is>
       </c>
       <c r="J85" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>HIGH on quality system …</t>
         </is>
       </c>
     </row>
@@ -5482,47 +5526,47 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>Strukmyer, LLC (Strukmyer Labs)  [NEW]</t>
+          <t>TBK One (TBK Manufacturing) — Carrollton, TX</t>
         </is>
       </c>
       <c r="C86" s="23" t="inlineStr">
         <is>
-          <t>Dallas / Lewisville, TX (DFW metro)</t>
+          <t>Carrollton, TX</t>
         </is>
       </c>
       <c r="D86" s="24" t="inlineStr">
         <is>
-          <t>https://strukmyer.com/filling-compounding/medical-devices/</t>
+          <t>https://tbk-one.com</t>
         </is>
       </c>
       <c r="E86" s="23" t="inlineStr">
         <is>
-          <t>SILENT. No published kettle temperature ceiling or jacketed-vessel specification. Hydrogel casting and cream/lotion compounding both normally require heated vessels, so the capability is plausible, but 90-95 C hold is UNVERIFIED.</t>
+          <t>SILENT — and conspicuously so. No mention of heated, jacketed, or steam vessels, no temperature specification, no tank sizes anywhere on the site, including the toll-blending page. The only process language is marketing-grade: their "precision blending proces…</t>
         </is>
       </c>
       <c r="F86" s="23" t="inlineStr">
         <is>
-          <t>Plausible. A 503B-registered compounder is structurally set up for small, frequent, made-to-order lots with short dating - which is exactly your 1-drum-per-wee…</t>
+          <t>BEST EXPLICIT SMALL-BATCH LANGUAGE OF ALL TEN: "Low minimum order quantities (MOQs) ideal for startups and growing businesses," plus "Flexible container sizes,…</t>
         </is>
       </c>
       <c r="G86" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485:2016 certified; FDA registered for drug and device manufacturing; cGMP compliant; DEA and FDA registered 503B outsourcing facilit…</t>
+          <t>NONE FOUND. EPA, OSHA and ISO compliance badges are displayed, but no ISO standard is named and no certificate is evidenced. NO ISO 9001, N…</t>
         </is>
       </c>
       <c r="H86" s="23" t="inlineStr">
         <is>
-          <t>Contact form at strukmyer.com; request the contract filling and compounding team</t>
+          <t>https://tbk-one.com/contact-tbk-one/ | 469-778-0088</t>
         </is>
       </c>
       <c r="I86" s="23" t="inlineStr">
         <is>
-          <t>ISO 13485 NOT REQUIRED (confirmed by Oscar) — deprioritized. Medical-grade pricing would run well above the incumbent for a certification we do not need. Keep only as a fallback if Quality later asks for a stricter supply chain. | One of the few US contract manufacturers that stacks ISO 13485:2016, FDA drug AND device registration, cGMP, and 503B outsourcing-facility registration in one house, while its actual day-to-day work is compounding and filling liquids. They…</t>
+          <t>CORRECTION: Address is correct (1813 Kelly Blvd, Carrollton, TX 75006). TWO CORRECTIONS: (1) The parenthetical alternate name "TBK Manufacturing" is NOT SUPPORTED by anything found — the affiliated sister entity is TBK ENVIRONMENTA…  |  MOVE DOWN from B to C. The small-batch fit is genuinely the best on the list, which is why they should not be dropped outright — but everything else is weak: zero heat evidence on th…</t>
         </is>
       </c>
       <c r="J86" s="25" t="inlineStr">
         <is>
-          <t>HIGH on quality system …</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -5534,47 +5578,47 @@
       </c>
       <c r="B87" s="23" t="inlineStr">
         <is>
-          <t>TBK One (TBK Manufacturing) — Carrollton, TX</t>
+          <t>The Chemical Company (TCC)</t>
         </is>
       </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
-          <t>Carrollton, TX</t>
+          <t>Jamestown, RI</t>
         </is>
       </c>
       <c r="D87" s="24" t="inlineStr">
         <is>
-          <t>https://tbk-one.com</t>
+          <t>https://www.thechemco.com</t>
         </is>
       </c>
       <c r="E87" s="23" t="inlineStr">
         <is>
-          <t>SILENT — and conspicuously so. No mention of heated, jacketed, or steam vessels, no temperature specification, no tank sizes anywhere on the site, including the toll-blending page. The only process language is marketing-grade: their "precision blending proces…</t>
+          <t>silent - no mention of reactors, jacketed or heated vessels, kettles, or any maximum temperature anywhere on the site. Do not assume they can heat anything; they would have to sub-contract it.</t>
         </is>
       </c>
       <c r="F87" s="23" t="inlineStr">
         <is>
-          <t>BEST EXPLICIT SMALL-BATCH LANGUAGE OF ALL TEN: "Low minimum order quantities (MOQs) ideal for startups and growing businesses," plus "Flexible container sizes,…</t>
+          <t>silent - no minimum batch size or MOQ published.</t>
         </is>
       </c>
       <c r="G87" s="23" t="inlineStr">
         <is>
-          <t>NONE FOUND. EPA, OSHA and ISO compliance badges are displayed, but no ISO standard is named and no certificate is evidenced. NO ISO 9001, N…</t>
+          <t>Good for a distributor: ISO 9001 certified and ISO 14001 certified (both stated on site). Participates in the Alliance for Chemical Distrib…</t>
         </is>
       </c>
       <c r="H87" s="23" t="inlineStr">
         <is>
-          <t>https://tbk-one.com/contact-tbk-one/ | 469-778-0088</t>
+          <t>https://thechemco.com/contact-tcc/ - Phone (401) 360-2800</t>
         </is>
       </c>
       <c r="I87" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: Address is correct (1813 Kelly Blvd, Carrollton, TX 75006). TWO CORRECTIONS: (1) The parenthetical alternate name "TBK Manufacturing" is NOT SUPPORTED by anything found — the affiliated sister entity is TBK ENVIRONMENTA…  |  MOVE DOWN from B to C. The small-batch fit is genuinely the best on the list, which is why they should not be dropped outright — but everything else is weak: zero heat evidence on th…</t>
+          <t>CORRECTION: none. Jamestown RI confirmed: 44 Southwest Avenue, Jamestown, RI 02835. One clarification for expectation-setting: TCC self-describes as 'the largest international supplier &amp; distributor of chemicals, composites, and pl…  |  keep - correct C role. They cannot blend this themselves (no equipment published, heat gate entirely silent), but as an ISO 9001 / Responsible Distribution distributor with a manufac…</t>
         </is>
       </c>
       <c r="J87" s="25" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -5586,47 +5630,47 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>The Chemical Company (TCC)</t>
+          <t>The Seydel Companies, Inc.  [NEW]</t>
         </is>
       </c>
       <c r="C88" s="23" t="inlineStr">
         <is>
-          <t>Jamestown, RI</t>
+          <t>244 John B. Brooks Road, Pendergrass, GA 30567 (plus a North Carolina plant)</t>
         </is>
       </c>
       <c r="D88" s="24" t="inlineStr">
         <is>
-          <t>https://www.thechemco.com</t>
+          <t>https://seydel.com/</t>
         </is>
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>silent - no mention of reactors, jacketed or heated vessels, kettles, or any maximum temperature anywhere on the site. Do not assume they can heat anything; they would have to sub-contract it.</t>
+          <t>NOT PUBLISHED. Their marketed PVA products are dry blends that the MILL cooks, so the cook may sit at the customer rather than at Seydel. This is the key question: do they have steam-jacketed liquid kettles that reach and hold 90-95 C, or only dry blending pl…</t>
         </is>
       </c>
       <c r="F88" s="23" t="inlineStr">
         <is>
-          <t>silent - no minimum batch size or MOQ published.</t>
+          <t>UNKNOWN. Family-owned mid-size specialty house; historically these shops will run small custom lots. Worth asking about a 450-lb weekly batch.</t>
         </is>
       </c>
       <c r="G88" s="23" t="inlineStr">
         <is>
-          <t>Good for a distributor: ISO 9001 certified and ISO 14001 certified (both stated on site). Participates in the Alliance for Chemical Distrib…</t>
+          <t>Not published. Ask about ISO 9001 and CoA capability.</t>
         </is>
       </c>
       <c r="H88" s="23" t="inlineStr">
         <is>
-          <t>https://thechemco.com/contact-tcc/ - Phone (401) 360-2800</t>
+          <t>706-693-2266 or 706-693-2074 / customerservice@seydel.com</t>
         </is>
       </c>
       <c r="I88" s="23" t="inlineStr">
         <is>
-          <t>CORRECTION: none. Jamestown RI confirmed: 44 Southwest Avenue, Jamestown, RI 02835. One clarification for expectation-setting: TCC self-describes as 'the largest international supplier &amp; distributor of chemicals, composites, and pl…  |  keep - correct C role. They cannot blend this themselves (no equipment published, heat gate entirely silent), but as an ISO 9001 / Responsible Distribution distributor with a manufac…</t>
+          <t>Family-owned chemical manufacturer since 1907 whose core business is textile sizing — including PVA-based sizes such as SEYCOSIZE PVA-G-R (a non-starch PVA size for polyester/cotton) and SEYCOSIZE MC-3 (medium-hydrolysis PVA). Textile size houses are the classic owners of the PVA cook. Importantly for us, Seydel explicitly offers toll-manufacturing plus technical laboratory and warehousing services, and the site ref…</t>
         </is>
       </c>
       <c r="J88" s="25" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5638,99 +5682,99 @@
       </c>
       <c r="B89" s="23" t="inlineStr">
         <is>
-          <t>The Seydel Companies, Inc.  [NEW]</t>
+          <t>Tilley (Tilley Distribution / Tilley Chemical)  [NEW]</t>
         </is>
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>244 John B. Brooks Road, Pendergrass, GA 30567 (plus a North Carolina plant)</t>
+          <t>Baltimore, MD (HQ and blending plant); second North American blending facility</t>
         </is>
       </c>
       <c r="D89" s="24" t="inlineStr">
         <is>
-          <t>https://seydel.com/</t>
+          <t>https://www.tilleydistribution.com/blending-packaging/</t>
         </is>
       </c>
       <c r="E89" s="23" t="inlineStr">
         <is>
-          <t>NOT PUBLISHED. Their marketed PVA products are dry blends that the MILL cooks, so the cook may sit at the customer rather than at Seydel. This is the key question: do they have steam-jacketed liquid kettles that reach and hold 90-95 C, or only dry blending pl…</t>
+          <t>NOT PUBLISHED and likely a problem. Their blending page describes 'nine blending tanks (10,000 gallons each)' for liquid-to-liquid and dry-to-liquid blending with no jacket, steam or temperature capability mentioned anywhere. Large ambient blend tanks are typ…</t>
         </is>
       </c>
       <c r="F89" s="23" t="inlineStr">
         <is>
-          <t>UNKNOWN. Family-owned mid-size specialty house; historically these shops will run small custom lots. Worth asking about a 450-lb weekly batch.</t>
+          <t>POOR. Published batch range is 220 to 10,000 gallons, and the published tanks are 10,000 gal each. A 220-gallon minimum is over four drums of a product with an…</t>
         </is>
       </c>
       <c r="G89" s="23" t="inlineStr">
         <is>
-          <t>Not published. Ask about ISO 9001 and CoA capability.</t>
+          <t>cGMP for pharmaceutical excipients, full-time QA lab, chemical engineering staff on site. Specific ISO numbers not published.</t>
         </is>
       </c>
       <c r="H89" s="23" t="inlineStr">
         <is>
-          <t>706-693-2266 or 706-693-2074 / customerservice@seydel.com</t>
+          <t>US 800-638-6968; Baltimore, MD headquarters</t>
         </is>
       </c>
       <c r="I89" s="23" t="inlineStr">
         <is>
-          <t>Family-owned chemical manufacturer since 1907 whose core business is textile sizing — including PVA-based sizes such as SEYCOSIZE PVA-G-R (a non-starch PVA size for polyester/cotton) and SEYCOSIZE MC-3 (medium-hydrolysis PVA). Textile size houses are the classic owners of the PVA cook. Importantly for us, Seydel explicitly offers toll-manufacturing plus technical laboratory and warehousing services, and the site ref…</t>
+          <t>You asked whether distributor-type firms actually run their own blending plants. Tilley is the clearest verified YES: a value-added chemical distributor founded 1952 that operates its own blending and packaging plants, publishes a cGMP pharmaceutical-excipient market segment, and fills 30- and 55-gallon drums directly. If you want a distributor-integrated route where the same firm could also supply some of the raw m…</t>
         </is>
       </c>
       <c r="J89" s="25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>High that the company a…</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="22" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B90" s="23" t="inlineStr">
-        <is>
-          <t>Tilley (Tilley Distribution / Tilley Chemical)  [NEW]</t>
-        </is>
-      </c>
-      <c r="C90" s="23" t="inlineStr">
-        <is>
-          <t>Baltimore, MD (HQ and blending plant); second North American blending facility</t>
-        </is>
-      </c>
-      <c r="D90" s="24" t="inlineStr">
-        <is>
-          <t>https://www.tilleydistribution.com/blending-packaging/</t>
-        </is>
-      </c>
-      <c r="E90" s="23" t="inlineStr">
-        <is>
-          <t>NOT PUBLISHED and likely a problem. Their blending page describes 'nine blending tanks (10,000 gallons each)' for liquid-to-liquid and dry-to-liquid blending with no jacket, steam or temperature capability mentioned anywhere. Large ambient blend tanks are typ…</t>
-        </is>
-      </c>
-      <c r="F90" s="23" t="inlineStr">
-        <is>
-          <t>POOR. Published batch range is 220 to 10,000 gallons, and the published tanks are 10,000 gal each. A 220-gallon minimum is over four drums of a product with an…</t>
-        </is>
-      </c>
-      <c r="G90" s="23" t="inlineStr">
-        <is>
-          <t>cGMP for pharmaceutical excipients, full-time QA lab, chemical engineering staff on site. Specific ISO numbers not published.</t>
-        </is>
-      </c>
-      <c r="H90" s="23" t="inlineStr">
-        <is>
-          <t>US 800-638-6968; Baltimore, MD headquarters</t>
-        </is>
-      </c>
-      <c r="I90" s="23" t="inlineStr">
-        <is>
-          <t>You asked whether distributor-type firms actually run their own blending plants. Tilley is the clearest verified YES: a value-added chemical distributor founded 1952 that operates its own blending and packaging plants, publishes a cGMP pharmaceutical-excipient market segment, and fills 30- and 55-gallon drums directly. If you want a distributor-integrated route where the same firm could also supply some of the raw m…</t>
-        </is>
-      </c>
-      <c r="J90" s="25" t="inlineStr">
-        <is>
-          <t>High that the company a…</t>
+      <c r="A90" s="26" t="inlineStr">
+        <is>
+          <t>ELIM</t>
+        </is>
+      </c>
+      <c r="B90" s="27" t="inlineStr">
+        <is>
+          <t>Columbus Chemical Industries (CCI)</t>
+        </is>
+      </c>
+      <c r="C90" s="27" t="inlineStr">
+        <is>
+          <t>Columbus WI / Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="D90" s="28" t="inlineStr">
+        <is>
+          <t>https://www.columbuschemical.com</t>
+        </is>
+      </c>
+      <c r="E90" s="27" t="inlineStr">
+        <is>
+          <t>FAILS — CANNOT HOLD THE TEMPERATURE. Confirmed directly by CCI Phoenix to Oscar. This OVERRIDES the earlier roster note of 'Yes — heating/cooling', which was never verified.</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="inlineStr">
+        <is>
+          <t>Was excellent on paper (20 L to 20,000 L, ~5 gal floor). Irrelevant now — the heat gate is binary.</t>
+        </is>
+      </c>
+      <c r="G90" s="27" t="inlineStr">
+        <is>
+          <t>ISO 9001, in-house lab</t>
+        </is>
+      </c>
+      <c r="H90" s="27" t="inlineStr">
+        <is>
+          <t>CLOSED OUT — no further action</t>
+        </is>
+      </c>
+      <c r="I90" s="27" t="inlineStr">
+        <is>
+          <t>ELIMINATED on the hard gate. WATCH THE NAME: this is COLUMBUS Chemical INDUSTRIES (Columbus WI / Phoenix AZ). It is a DIFFERENT company from COLUMBIA Chemical of Akron OH, which remains an active Tier B candidate. Do not confuse the two.</t>
+        </is>
+      </c>
+      <c r="J90" s="29" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
         </is>
       </c>
     </row>
@@ -6017,14 +6061,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId36"/>
@@ -6037,7 +6081,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId49"/>
@@ -6052,7 +6096,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId64"/>

</xml_diff>